<commit_message>
Add scenario support: Target and Forecast period columns
The extract's right-hand block carries -Tar (Target, incl. multi-year
FY'27..FY'30) and -FC (Forecast) columns alongside Actuals:
- Map Tar/Tgt -> Target, FC/Fcst -> Forecast in the semantic layer
- Group sidebar period picker by year x scenario
- 'Latest FY vs PY' preset now prefers Actuals so FY'30-Tar can't hijack it
- New 'Act vs Target' preset (latest year with both, ready for variance)
- Classification tolerant of duplicated headers' dedupe suffix
- Sample generator emits Target + FC columns; scenario list in summary

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018B5qKH9JxzLywUkLopxf6J
</commit_message>
<xml_diff>
--- a/tm1-dashboard/sample/GPS_Driller_sample.xlsx
+++ b/tm1-dashboard/sample/GPS_Driller_sample.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE17"/>
+  <dimension ref="A1:BU17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -702,6 +702,86 @@
           <t>YTD Dec'20-Act</t>
         </is>
       </c>
+      <c r="BF1" t="inlineStr">
+        <is>
+          <t>Apr'26-Tar</t>
+        </is>
+      </c>
+      <c r="BG1" t="inlineStr">
+        <is>
+          <t>Q1'26-Tar</t>
+        </is>
+      </c>
+      <c r="BH1" t="inlineStr">
+        <is>
+          <t>Q2'26-Tar</t>
+        </is>
+      </c>
+      <c r="BI1" t="inlineStr">
+        <is>
+          <t>Q3'26-Tar</t>
+        </is>
+      </c>
+      <c r="BJ1" t="inlineStr">
+        <is>
+          <t>Q4'26-Tar</t>
+        </is>
+      </c>
+      <c r="BK1" t="inlineStr">
+        <is>
+          <t>H1'26-Tar</t>
+        </is>
+      </c>
+      <c r="BL1" t="inlineStr">
+        <is>
+          <t>H2'26-Tar</t>
+        </is>
+      </c>
+      <c r="BM1" t="inlineStr">
+        <is>
+          <t>FY'26-Tar</t>
+        </is>
+      </c>
+      <c r="BN1" t="inlineStr">
+        <is>
+          <t>YTD Apr'26-Tar</t>
+        </is>
+      </c>
+      <c r="BO1" t="inlineStr">
+        <is>
+          <t>FY'27-Tar</t>
+        </is>
+      </c>
+      <c r="BP1" t="inlineStr">
+        <is>
+          <t>FY'28-Tar</t>
+        </is>
+      </c>
+      <c r="BQ1" t="inlineStr">
+        <is>
+          <t>FY'29-Tar</t>
+        </is>
+      </c>
+      <c r="BR1" t="inlineStr">
+        <is>
+          <t>FY'30-Tar</t>
+        </is>
+      </c>
+      <c r="BS1" t="inlineStr">
+        <is>
+          <t>Apr'26-FC</t>
+        </is>
+      </c>
+      <c r="BT1" t="inlineStr">
+        <is>
+          <t>May'26-FC</t>
+        </is>
+      </c>
+      <c r="BU1" t="inlineStr">
+        <is>
+          <t>Jun'26-FC</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -881,6 +961,54 @@
       <c r="BE2" t="n">
         <v>97.47</v>
       </c>
+      <c r="BF2" t="n">
+        <v>61.29</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>78.47</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>66.27</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>68.52</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>-30.86</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>78.62</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>75.18000000000001</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>87.42</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>120.69</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>98.12</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>73.26000000000001</v>
+      </c>
+      <c r="BQ2" t="n">
+        <v>134.07</v>
+      </c>
+      <c r="BR2" t="n">
+        <v>85.70999999999999</v>
+      </c>
+      <c r="BS2" t="n">
+        <v>101.18</v>
+      </c>
+      <c r="BT2" t="n">
+        <v>92.73999999999999</v>
+      </c>
+      <c r="BU2" t="n">
+        <v>92.05</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -958,116 +1086,158 @@
           <t>PR05011002 - Current Accounts - Interest Bearing</t>
         </is>
       </c>
-      <c r="P3" t="n">
-        <v>47.11</v>
-      </c>
       <c r="Q3" t="n">
-        <v>59.87</v>
-      </c>
-      <c r="R3" t="n">
-        <v>47.3</v>
+        <v>33.37</v>
       </c>
       <c r="S3" t="n">
-        <v>52.45</v>
+        <v>53.17</v>
+      </c>
+      <c r="T3" t="n">
+        <v>47.07</v>
       </c>
       <c r="U3" t="n">
-        <v>63.49</v>
+        <v>48.69</v>
       </c>
       <c r="V3" t="n">
-        <v>38.76</v>
+        <v>32.08</v>
+      </c>
+      <c r="W3" t="n">
+        <v>34.79</v>
       </c>
       <c r="X3" t="n">
-        <v>40.23</v>
+        <v>16.17</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>3.24</v>
       </c>
       <c r="Z3" t="n">
-        <v>33.58</v>
+        <v>30.38</v>
       </c>
       <c r="AA3" t="n">
-        <v>19.87</v>
+        <v>37.22</v>
       </c>
       <c r="AB3" t="n">
-        <v>37.7</v>
+        <v>40.5</v>
       </c>
       <c r="AC3" t="n">
-        <v>15.91</v>
+        <v>-7.5</v>
       </c>
       <c r="AD3" t="n">
-        <v>30.41</v>
+        <v>44.72</v>
       </c>
       <c r="AE3" t="n">
-        <v>21.49</v>
+        <v>6.34</v>
       </c>
       <c r="AF3" t="n">
-        <v>40.94</v>
+        <v>-9.82</v>
       </c>
       <c r="AG3" t="n">
-        <v>-10.91</v>
+        <v>40.79</v>
       </c>
       <c r="AH3" t="n">
-        <v>43.93</v>
+        <v>32.81</v>
       </c>
       <c r="AI3" t="n">
-        <v>38.3</v>
+        <v>18.9</v>
       </c>
       <c r="AJ3" t="n">
-        <v>31.63</v>
+        <v>29.11</v>
       </c>
       <c r="AK3" t="n">
-        <v>50.06</v>
+        <v>24.29</v>
       </c>
       <c r="AL3" t="n">
-        <v>28.96</v>
+        <v>30.28</v>
       </c>
       <c r="AM3" t="n">
-        <v>46.05</v>
+        <v>26.68</v>
       </c>
       <c r="AN3" t="n">
-        <v>42.79</v>
+        <v>34.53</v>
       </c>
       <c r="AO3" t="n">
-        <v>40.88</v>
+        <v>29.27</v>
       </c>
       <c r="AP3" t="n">
-        <v>34.73</v>
+        <v>46.6</v>
       </c>
       <c r="AQ3" t="n">
-        <v>40.23</v>
+        <v>45.59</v>
       </c>
       <c r="AR3" t="n">
-        <v>47.83</v>
+        <v>19.16</v>
       </c>
       <c r="AS3" t="n">
-        <v>12.29</v>
+        <v>23.85</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>17.76</v>
       </c>
       <c r="AU3" t="n">
-        <v>43.88</v>
-      </c>
-      <c r="AV3" t="n">
-        <v>56.77</v>
+        <v>39.97</v>
       </c>
       <c r="AW3" t="n">
-        <v>24.58</v>
+        <v>-19.7</v>
       </c>
       <c r="AX3" t="n">
-        <v>46.54</v>
+        <v>29.98</v>
       </c>
       <c r="AY3" t="n">
-        <v>39.63</v>
+        <v>46.32</v>
       </c>
       <c r="AZ3" t="n">
-        <v>7.83</v>
+        <v>15.47</v>
       </c>
       <c r="BA3" t="n">
-        <v>49.72</v>
-      </c>
-      <c r="BB3" t="n">
-        <v>25.88</v>
+        <v>6.39</v>
       </c>
       <c r="BC3" t="n">
-        <v>66.41</v>
-      </c>
-      <c r="BE3" t="n">
-        <v>11.12</v>
+        <v>10.09</v>
+      </c>
+      <c r="BD3" t="n">
+        <v>35.61</v>
+      </c>
+      <c r="BF3" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="BG3" t="n">
+        <v>28.88</v>
+      </c>
+      <c r="BH3" t="n">
+        <v>23.31</v>
+      </c>
+      <c r="BI3" t="n">
+        <v>32.98</v>
+      </c>
+      <c r="BJ3" t="n">
+        <v>-7.94</v>
+      </c>
+      <c r="BK3" t="n">
+        <v>24.94</v>
+      </c>
+      <c r="BL3" t="n">
+        <v>24.05</v>
+      </c>
+      <c r="BO3" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="BP3" t="n">
+        <v>22.76</v>
+      </c>
+      <c r="BQ3" t="n">
+        <v>22.19</v>
+      </c>
+      <c r="BR3" t="n">
+        <v>51.55</v>
+      </c>
+      <c r="BS3" t="n">
+        <v>30.34</v>
+      </c>
+      <c r="BT3" t="n">
+        <v>35.27</v>
+      </c>
+      <c r="BU3" t="n">
+        <v>44.14</v>
       </c>
     </row>
     <row r="4">
@@ -1146,107 +1316,155 @@
           <t>PR05012100 - Current Accounts - Non Interest Bearing</t>
         </is>
       </c>
-      <c r="Q4" t="n">
-        <v>114.07</v>
+      <c r="P4" t="n">
+        <v>195.37</v>
       </c>
       <c r="R4" t="n">
-        <v>117.39</v>
+        <v>70.43000000000001</v>
       </c>
       <c r="S4" t="n">
-        <v>135.83</v>
+        <v>199.75</v>
       </c>
       <c r="T4" t="n">
-        <v>68.72</v>
+        <v>121.83</v>
       </c>
       <c r="U4" t="n">
-        <v>141.5</v>
+        <v>98.17</v>
       </c>
       <c r="V4" t="n">
-        <v>118.37</v>
+        <v>83.31999999999999</v>
       </c>
       <c r="W4" t="n">
-        <v>155.96</v>
+        <v>-37.77</v>
       </c>
       <c r="X4" t="n">
-        <v>155.68</v>
+        <v>78.53</v>
       </c>
       <c r="Y4" t="n">
-        <v>-40.56</v>
+        <v>189.58</v>
       </c>
       <c r="Z4" t="n">
-        <v>106.52</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>209.11</v>
+        <v>167.78</v>
       </c>
       <c r="AB4" t="n">
-        <v>147.15</v>
+        <v>111.25</v>
       </c>
       <c r="AC4" t="n">
-        <v>60.98</v>
+        <v>115.36</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>136.83</v>
       </c>
       <c r="AE4" t="n">
-        <v>97.28</v>
+        <v>76.89</v>
       </c>
       <c r="AF4" t="n">
-        <v>172.29</v>
+        <v>114.36</v>
       </c>
       <c r="AH4" t="n">
-        <v>107.78</v>
+        <v>53.73</v>
       </c>
       <c r="AI4" t="n">
-        <v>170.03</v>
-      </c>
-      <c r="AJ4" t="n">
-        <v>27.95</v>
+        <v>101.61</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>100.06</v>
       </c>
       <c r="AL4" t="n">
-        <v>121.81</v>
+        <v>148.46</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>82.33</v>
       </c>
       <c r="AN4" t="n">
-        <v>94.97</v>
+        <v>139.93</v>
       </c>
       <c r="AO4" t="n">
-        <v>91.58</v>
+        <v>78.19</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>37.73</v>
       </c>
       <c r="AR4" t="n">
-        <v>157.29</v>
+        <v>68.37</v>
       </c>
       <c r="AS4" t="n">
-        <v>86.67</v>
+        <v>140.32</v>
       </c>
       <c r="AT4" t="n">
-        <v>84.51000000000001</v>
+        <v>30.21</v>
       </c>
       <c r="AU4" t="n">
-        <v>196.31</v>
+        <v>132.07</v>
       </c>
       <c r="AV4" t="n">
-        <v>115.55</v>
+        <v>92.38</v>
       </c>
       <c r="AW4" t="n">
-        <v>134.32</v>
+        <v>89.76000000000001</v>
       </c>
       <c r="AX4" t="n">
-        <v>168.09</v>
+        <v>120.13</v>
       </c>
       <c r="AY4" t="n">
-        <v>192.42</v>
-      </c>
-      <c r="AZ4" t="n">
-        <v>180.71</v>
+        <v>125.93</v>
       </c>
       <c r="BA4" t="n">
-        <v>125.73</v>
+        <v>98.76000000000001</v>
       </c>
       <c r="BB4" t="n">
-        <v>127.35</v>
-      </c>
-      <c r="BD4" t="n">
-        <v>85.94</v>
+        <v>97.62</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>185.66</v>
       </c>
       <c r="BE4" t="n">
-        <v>133.73</v>
+        <v>119.65</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>104.17</v>
+      </c>
+      <c r="BG4" t="n">
+        <v>115.78</v>
+      </c>
+      <c r="BH4" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="BI4" t="n">
+        <v>11.31</v>
+      </c>
+      <c r="BJ4" t="n">
+        <v>107.93</v>
+      </c>
+      <c r="BK4" t="n">
+        <v>69.51000000000001</v>
+      </c>
+      <c r="BL4" t="n">
+        <v>85.87</v>
+      </c>
+      <c r="BM4" t="n">
+        <v>122.3</v>
+      </c>
+      <c r="BN4" t="n">
+        <v>-28.28</v>
+      </c>
+      <c r="BO4" t="n">
+        <v>93.76000000000001</v>
+      </c>
+      <c r="BP4" t="n">
+        <v>95.56999999999999</v>
+      </c>
+      <c r="BQ4" t="n">
+        <v>111.67</v>
+      </c>
+      <c r="BS4" t="n">
+        <v>76.23</v>
+      </c>
+      <c r="BT4" t="n">
+        <v>106.01</v>
+      </c>
+      <c r="BU4" t="n">
+        <v>90.11</v>
       </c>
     </row>
     <row r="5">
@@ -1325,113 +1543,158 @@
           <t>PR05040100 - Savings Accounts - Other</t>
         </is>
       </c>
-      <c r="P5" t="n">
-        <v>-18.66</v>
-      </c>
       <c r="Q5" t="n">
-        <v>64.59999999999999</v>
+        <v>17.06</v>
       </c>
       <c r="R5" t="n">
-        <v>155.96</v>
+        <v>65.77</v>
       </c>
       <c r="S5" t="n">
-        <v>138.02</v>
+        <v>43.62</v>
+      </c>
+      <c r="T5" t="n">
+        <v>-15.67</v>
       </c>
       <c r="U5" t="n">
-        <v>91.52</v>
+        <v>66.66</v>
       </c>
       <c r="V5" t="n">
-        <v>94.90000000000001</v>
+        <v>58.49</v>
       </c>
       <c r="W5" t="n">
-        <v>112.56</v>
+        <v>-19.57</v>
       </c>
       <c r="X5" t="n">
-        <v>63.25</v>
+        <v>45.07</v>
       </c>
       <c r="Y5" t="n">
-        <v>94.08</v>
+        <v>47.17</v>
       </c>
       <c r="AA5" t="n">
-        <v>44.2</v>
+        <v>52.36</v>
       </c>
       <c r="AB5" t="n">
-        <v>83.59</v>
+        <v>63.48</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>-14.59</v>
       </c>
       <c r="AD5" t="n">
-        <v>82.31</v>
+        <v>55.8</v>
       </c>
       <c r="AE5" t="n">
-        <v>122.13</v>
+        <v>31.28</v>
       </c>
       <c r="AF5" t="n">
-        <v>67.73</v>
+        <v>24.67</v>
       </c>
       <c r="AG5" t="n">
-        <v>115.11</v>
+        <v>58.47</v>
       </c>
       <c r="AH5" t="n">
-        <v>64.31999999999999</v>
+        <v>50</v>
       </c>
       <c r="AI5" t="n">
-        <v>31.04</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>56.24</v>
+        <v>39.65</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>21.08</v>
       </c>
       <c r="AL5" t="n">
-        <v>115.43</v>
+        <v>-17.01</v>
       </c>
       <c r="AM5" t="n">
-        <v>24.85</v>
+        <v>46.95</v>
       </c>
       <c r="AN5" t="n">
-        <v>108.65</v>
+        <v>-8.16</v>
       </c>
       <c r="AO5" t="n">
-        <v>75.98999999999999</v>
-      </c>
-      <c r="AP5" t="n">
-        <v>73.84</v>
+        <v>65.09</v>
       </c>
       <c r="AQ5" t="n">
-        <v>98.81999999999999</v>
+        <v>62.36</v>
       </c>
       <c r="AR5" t="n">
-        <v>103.59</v>
+        <v>30.07</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>33.96</v>
       </c>
       <c r="AT5" t="n">
-        <v>81.23999999999999</v>
+        <v>55.88</v>
       </c>
       <c r="AU5" t="n">
-        <v>80.3</v>
+        <v>82.95999999999999</v>
       </c>
       <c r="AV5" t="n">
-        <v>152.73</v>
+        <v>75.47</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>44.24</v>
       </c>
       <c r="AX5" t="n">
-        <v>98.43000000000001</v>
+        <v>4.71</v>
       </c>
       <c r="AY5" t="n">
-        <v>85.7</v>
+        <v>23.33</v>
       </c>
       <c r="AZ5" t="n">
-        <v>95.23999999999999</v>
-      </c>
-      <c r="BA5" t="n">
-        <v>46.81</v>
+        <v>59.63</v>
       </c>
       <c r="BB5" t="n">
-        <v>9.300000000000001</v>
+        <v>49.48</v>
       </c>
       <c r="BC5" t="n">
-        <v>88.79000000000001</v>
+        <v>-20.34</v>
       </c>
       <c r="BD5" t="n">
-        <v>57.18</v>
+        <v>53.64</v>
       </c>
       <c r="BE5" t="n">
-        <v>70.64</v>
+        <v>59.46</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>48.34</v>
+      </c>
+      <c r="BH5" t="n">
+        <v>51.15</v>
+      </c>
+      <c r="BI5" t="n">
+        <v>39.78</v>
+      </c>
+      <c r="BJ5" t="n">
+        <v>25.85</v>
+      </c>
+      <c r="BK5" t="n">
+        <v>43.53</v>
+      </c>
+      <c r="BL5" t="n">
+        <v>35.12</v>
+      </c>
+      <c r="BM5" t="n">
+        <v>48.35</v>
+      </c>
+      <c r="BN5" t="n">
+        <v>33.46</v>
+      </c>
+      <c r="BO5" t="n">
+        <v>51.78</v>
+      </c>
+      <c r="BP5" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="BQ5" t="n">
+        <v>21.48</v>
+      </c>
+      <c r="BR5" t="n">
+        <v>51.46</v>
+      </c>
+      <c r="BT5" t="n">
+        <v>-15.08</v>
+      </c>
+      <c r="BU5" t="n">
+        <v>59.37</v>
       </c>
     </row>
     <row r="6">
@@ -1511,115 +1774,157 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>81.7</v>
+        <v>110.14</v>
       </c>
       <c r="Q6" t="n">
-        <v>76.64</v>
+        <v>96.91</v>
       </c>
       <c r="R6" t="n">
-        <v>89.20999999999999</v>
-      </c>
-      <c r="S6" t="n">
-        <v>91.16</v>
+        <v>73.70999999999999</v>
       </c>
       <c r="T6" t="n">
-        <v>-28.06</v>
+        <v>125.48</v>
       </c>
       <c r="U6" t="n">
-        <v>50.92</v>
-      </c>
-      <c r="V6" t="n">
-        <v>70.81</v>
+        <v>104</v>
       </c>
       <c r="W6" t="n">
-        <v>60.19</v>
+        <v>126.43</v>
       </c>
       <c r="X6" t="n">
-        <v>-8.23</v>
+        <v>137.6</v>
       </c>
       <c r="Y6" t="n">
-        <v>79.5</v>
+        <v>116.26</v>
       </c>
       <c r="Z6" t="n">
-        <v>24.61</v>
+        <v>72.66</v>
       </c>
       <c r="AA6" t="n">
-        <v>62.91</v>
+        <v>110.71</v>
       </c>
       <c r="AB6" t="n">
-        <v>-19.99</v>
+        <v>76.33</v>
       </c>
       <c r="AC6" t="n">
-        <v>66.31</v>
+        <v>78.31999999999999</v>
       </c>
       <c r="AD6" t="n">
-        <v>53.15</v>
-      </c>
-      <c r="AE6" t="n">
-        <v>105.38</v>
+        <v>104.27</v>
       </c>
       <c r="AG6" t="n">
-        <v>82.95999999999999</v>
+        <v>96.79000000000001</v>
       </c>
       <c r="AH6" t="n">
-        <v>103.77</v>
+        <v>124.5</v>
       </c>
       <c r="AI6" t="n">
-        <v>86.65000000000001</v>
+        <v>180.79</v>
       </c>
       <c r="AJ6" t="n">
-        <v>78.98</v>
-      </c>
-      <c r="AM6" t="n">
-        <v>26.56</v>
+        <v>130.55</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>61.28</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>63.32</v>
       </c>
       <c r="AN6" t="n">
-        <v>50.27</v>
+        <v>45.37</v>
       </c>
       <c r="AO6" t="n">
-        <v>39.64</v>
+        <v>86.38</v>
       </c>
       <c r="AP6" t="n">
-        <v>93.97</v>
+        <v>102.8</v>
       </c>
       <c r="AQ6" t="n">
-        <v>80.34</v>
-      </c>
-      <c r="AR6" t="n">
-        <v>63.72</v>
+        <v>69.23999999999999</v>
       </c>
       <c r="AS6" t="n">
-        <v>33.88</v>
+        <v>116.9</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>205</v>
       </c>
       <c r="AU6" t="n">
-        <v>-27.34</v>
+        <v>173.9</v>
       </c>
       <c r="AV6" t="n">
-        <v>75.45</v>
+        <v>-30.54</v>
       </c>
       <c r="AW6" t="n">
-        <v>-13.12</v>
+        <v>88.37</v>
       </c>
       <c r="AX6" t="n">
-        <v>104.6</v>
-      </c>
-      <c r="AZ6" t="n">
-        <v>100.21</v>
+        <v>139.45</v>
+      </c>
+      <c r="AY6" t="n">
+        <v>104</v>
       </c>
       <c r="BA6" t="n">
-        <v>48.33</v>
+        <v>86.55</v>
       </c>
       <c r="BB6" t="n">
-        <v>54.58</v>
+        <v>169.89</v>
       </c>
       <c r="BC6" t="n">
-        <v>89.81</v>
+        <v>187.72</v>
       </c>
       <c r="BD6" t="n">
-        <v>133.32</v>
+        <v>91.7</v>
       </c>
       <c r="BE6" t="n">
-        <v>121.28</v>
+        <v>158</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>109.28</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>94.47</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>130.73</v>
+      </c>
+      <c r="BI6" t="n">
+        <v>131.92</v>
+      </c>
+      <c r="BJ6" t="n">
+        <v>166.57</v>
+      </c>
+      <c r="BK6" t="n">
+        <v>172.38</v>
+      </c>
+      <c r="BL6" t="n">
+        <v>107.62</v>
+      </c>
+      <c r="BM6" t="n">
+        <v>223.49</v>
+      </c>
+      <c r="BN6" t="n">
+        <v>187.65</v>
+      </c>
+      <c r="BO6" t="n">
+        <v>51.99</v>
+      </c>
+      <c r="BP6" t="n">
+        <v>117.71</v>
+      </c>
+      <c r="BQ6" t="n">
+        <v>119.09</v>
+      </c>
+      <c r="BR6" t="n">
+        <v>168.86</v>
+      </c>
+      <c r="BS6" t="n">
+        <v>138.68</v>
+      </c>
+      <c r="BT6" t="n">
+        <v>92.2</v>
+      </c>
+      <c r="BU6" t="n">
+        <v>131.37</v>
       </c>
     </row>
     <row r="7">
@@ -1699,115 +2004,160 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>70.02</v>
+        <v>53.81</v>
       </c>
       <c r="Q7" t="n">
-        <v>51.79</v>
+        <v>49.83</v>
       </c>
       <c r="R7" t="n">
-        <v>53.27</v>
+        <v>66.89</v>
       </c>
       <c r="S7" t="n">
-        <v>39.95</v>
+        <v>87.25</v>
       </c>
       <c r="T7" t="n">
-        <v>55.91</v>
-      </c>
-      <c r="U7" t="n">
-        <v>-22.99</v>
+        <v>108.86</v>
       </c>
       <c r="V7" t="n">
-        <v>60.61</v>
+        <v>59.63</v>
       </c>
       <c r="W7" t="n">
-        <v>67.19</v>
+        <v>27.97</v>
       </c>
       <c r="X7" t="n">
-        <v>54.63</v>
+        <v>65.53</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>72.7</v>
       </c>
       <c r="Z7" t="n">
-        <v>57.8</v>
+        <v>43.65</v>
       </c>
       <c r="AA7" t="n">
-        <v>44.95</v>
+        <v>83.86</v>
       </c>
       <c r="AB7" t="n">
-        <v>29.21</v>
+        <v>88.65000000000001</v>
       </c>
       <c r="AC7" t="n">
-        <v>49.19</v>
+        <v>96.06</v>
       </c>
       <c r="AD7" t="n">
-        <v>39.69</v>
+        <v>102.11</v>
       </c>
       <c r="AE7" t="n">
-        <v>54.64</v>
+        <v>32.67</v>
       </c>
       <c r="AF7" t="n">
-        <v>37.81</v>
-      </c>
-      <c r="AG7" t="n">
-        <v>58.51</v>
+        <v>-22.66</v>
       </c>
       <c r="AH7" t="n">
-        <v>64.18000000000001</v>
+        <v>21.1</v>
       </c>
       <c r="AI7" t="n">
-        <v>24.27</v>
+        <v>71.95</v>
       </c>
       <c r="AJ7" t="n">
-        <v>58.15</v>
+        <v>45.43</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>-16.08</v>
       </c>
       <c r="AL7" t="n">
-        <v>-17.04</v>
+        <v>21</v>
       </c>
       <c r="AM7" t="n">
-        <v>67.08</v>
+        <v>91.55</v>
       </c>
       <c r="AN7" t="n">
-        <v>26.93</v>
-      </c>
-      <c r="AO7" t="n">
-        <v>45.27</v>
+        <v>97.23999999999999</v>
       </c>
       <c r="AP7" t="n">
-        <v>35.68</v>
+        <v>58.74</v>
       </c>
       <c r="AQ7" t="n">
-        <v>-13.6</v>
+        <v>59.63</v>
       </c>
       <c r="AR7" t="n">
-        <v>19.61</v>
+        <v>72.38</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>75.98</v>
       </c>
       <c r="AT7" t="n">
-        <v>-18.02</v>
+        <v>50.68</v>
       </c>
       <c r="AU7" t="n">
-        <v>39.94</v>
+        <v>80.86</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>82.03</v>
       </c>
       <c r="AW7" t="n">
-        <v>48.77</v>
+        <v>58.53</v>
       </c>
       <c r="AX7" t="n">
-        <v>58.65</v>
+        <v>1.54</v>
       </c>
       <c r="AY7" t="n">
-        <v>78.25</v>
+        <v>36.45</v>
       </c>
       <c r="AZ7" t="n">
-        <v>45.92</v>
-      </c>
-      <c r="BA7" t="n">
-        <v>80.33</v>
+        <v>37.15</v>
       </c>
       <c r="BB7" t="n">
-        <v>61.95</v>
+        <v>56.96</v>
       </c>
       <c r="BC7" t="n">
-        <v>-24.77</v>
+        <v>62.25</v>
+      </c>
+      <c r="BD7" t="n">
+        <v>116.77</v>
       </c>
       <c r="BE7" t="n">
-        <v>41.78</v>
+        <v>54.72</v>
+      </c>
+      <c r="BF7" t="n">
+        <v>36.06</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>59.27</v>
+      </c>
+      <c r="BH7" t="n">
+        <v>55.15</v>
+      </c>
+      <c r="BJ7" t="n">
+        <v>72.25</v>
+      </c>
+      <c r="BK7" t="n">
+        <v>56.73</v>
+      </c>
+      <c r="BL7" t="n">
+        <v>113.41</v>
+      </c>
+      <c r="BM7" t="n">
+        <v>47.77</v>
+      </c>
+      <c r="BN7" t="n">
+        <v>72</v>
+      </c>
+      <c r="BO7" t="n">
+        <v>49.43</v>
+      </c>
+      <c r="BP7" t="n">
+        <v>98.48999999999999</v>
+      </c>
+      <c r="BQ7" t="n">
+        <v>41.14</v>
+      </c>
+      <c r="BR7" t="n">
+        <v>73.56999999999999</v>
+      </c>
+      <c r="BS7" t="n">
+        <v>68.39</v>
+      </c>
+      <c r="BT7" t="n">
+        <v>31.83</v>
       </c>
     </row>
     <row r="8">
@@ -1886,125 +2236,140 @@
           <t>PR05040200 - Time Deposits Other</t>
         </is>
       </c>
-      <c r="P8" t="n">
-        <v>72.37</v>
-      </c>
       <c r="Q8" t="n">
-        <v>133.52</v>
+        <v>21.38</v>
       </c>
       <c r="R8" t="n">
-        <v>61.83</v>
+        <v>32.61</v>
       </c>
       <c r="S8" t="n">
-        <v>44.37</v>
+        <v>35.86</v>
       </c>
       <c r="T8" t="n">
-        <v>-22.27</v>
+        <v>49.12</v>
       </c>
       <c r="U8" t="n">
-        <v>68.52</v>
+        <v>52.66</v>
       </c>
       <c r="V8" t="n">
-        <v>133.26</v>
+        <v>39.97</v>
       </c>
       <c r="W8" t="n">
-        <v>63.87</v>
+        <v>41.13</v>
       </c>
       <c r="X8" t="n">
-        <v>17.64</v>
+        <v>31.58</v>
       </c>
       <c r="Z8" t="n">
-        <v>76.23</v>
+        <v>25.43</v>
       </c>
       <c r="AA8" t="n">
-        <v>106.9</v>
+        <v>42.4</v>
       </c>
       <c r="AB8" t="n">
-        <v>199.63</v>
-      </c>
-      <c r="AC8" t="n">
-        <v>-15.03</v>
+        <v>34.08</v>
       </c>
       <c r="AD8" t="n">
-        <v>43.19</v>
+        <v>2.28</v>
       </c>
       <c r="AE8" t="n">
-        <v>94.38</v>
+        <v>23.39</v>
       </c>
       <c r="AF8" t="n">
-        <v>73.09999999999999</v>
+        <v>38.99</v>
       </c>
       <c r="AG8" t="n">
-        <v>86.98999999999999</v>
-      </c>
-      <c r="AH8" t="n">
-        <v>63.97</v>
+        <v>21.86</v>
       </c>
       <c r="AI8" t="n">
-        <v>127.04</v>
-      </c>
-      <c r="AJ8" t="n">
-        <v>61.1</v>
+        <v>32.12</v>
       </c>
       <c r="AK8" t="n">
-        <v>93.65000000000001</v>
+        <v>37.68</v>
       </c>
       <c r="AL8" t="n">
-        <v>130.4</v>
+        <v>38.7</v>
       </c>
       <c r="AM8" t="n">
-        <v>83</v>
+        <v>-7.38</v>
       </c>
       <c r="AN8" t="n">
-        <v>88.01000000000001</v>
+        <v>35.51</v>
       </c>
       <c r="AO8" t="n">
-        <v>44.01</v>
-      </c>
-      <c r="AP8" t="n">
-        <v>43.03</v>
-      </c>
-      <c r="AQ8" t="n">
-        <v>104.03</v>
+        <v>36.54</v>
       </c>
       <c r="AR8" t="n">
-        <v>107.1</v>
+        <v>32.64</v>
       </c>
       <c r="AT8" t="n">
-        <v>118.36</v>
+        <v>41.73</v>
       </c>
       <c r="AU8" t="n">
-        <v>128.52</v>
-      </c>
-      <c r="AV8" t="n">
-        <v>124.7</v>
+        <v>12.74</v>
       </c>
       <c r="AW8" t="n">
-        <v>129.25</v>
-      </c>
-      <c r="AX8" t="n">
-        <v>13.39</v>
+        <v>34.77</v>
       </c>
       <c r="AY8" t="n">
-        <v>24.27</v>
+        <v>40.98</v>
       </c>
       <c r="AZ8" t="n">
-        <v>83.08</v>
+        <v>-6.55</v>
       </c>
       <c r="BA8" t="n">
-        <v>119.24</v>
+        <v>18.04</v>
       </c>
       <c r="BB8" t="n">
-        <v>71.86</v>
-      </c>
-      <c r="BC8" t="n">
-        <v>121.33</v>
+        <v>-12.52</v>
       </c>
       <c r="BD8" t="n">
-        <v>86.06</v>
+        <v>40.09</v>
       </c>
       <c r="BE8" t="n">
-        <v>54.24</v>
+        <v>35.48</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>19.84</v>
+      </c>
+      <c r="BH8" t="n">
+        <v>29.55</v>
+      </c>
+      <c r="BI8" t="n">
+        <v>34.01</v>
+      </c>
+      <c r="BJ8" t="n">
+        <v>14.19</v>
+      </c>
+      <c r="BK8" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="BL8" t="n">
+        <v>35.22</v>
+      </c>
+      <c r="BM8" t="n">
+        <v>-13.92</v>
+      </c>
+      <c r="BN8" t="n">
+        <v>52.58</v>
+      </c>
+      <c r="BP8" t="n">
+        <v>37.27</v>
+      </c>
+      <c r="BQ8" t="n">
+        <v>18.72</v>
+      </c>
+      <c r="BR8" t="n">
+        <v>21.88</v>
+      </c>
+      <c r="BS8" t="n">
+        <v>45.03</v>
+      </c>
+      <c r="BT8" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="BU8" t="n">
+        <v>25.76</v>
       </c>
     </row>
     <row r="9">
@@ -2083,122 +2448,158 @@
           <t>PR05040220 - Time Deposits 3 - 6 Months</t>
         </is>
       </c>
-      <c r="P9" t="n">
-        <v>23.92</v>
-      </c>
       <c r="Q9" t="n">
-        <v>27.14</v>
+        <v>18.48</v>
       </c>
       <c r="R9" t="n">
-        <v>23.94</v>
+        <v>44.3</v>
       </c>
       <c r="S9" t="n">
-        <v>17.75</v>
-      </c>
-      <c r="T9" t="n">
-        <v>-3.56</v>
+        <v>36.98</v>
       </c>
       <c r="U9" t="n">
-        <v>10.78</v>
+        <v>17.28</v>
       </c>
       <c r="V9" t="n">
-        <v>16.57</v>
+        <v>37.89</v>
       </c>
       <c r="W9" t="n">
-        <v>25.04</v>
+        <v>-13.8</v>
       </c>
       <c r="X9" t="n">
-        <v>17.24</v>
+        <v>20.82</v>
       </c>
       <c r="Y9" t="n">
-        <v>19.11</v>
+        <v>-7.91</v>
       </c>
       <c r="Z9" t="n">
-        <v>38.88</v>
+        <v>33.23</v>
       </c>
       <c r="AA9" t="n">
-        <v>20.75</v>
+        <v>41.76</v>
       </c>
       <c r="AB9" t="n">
-        <v>32.28</v>
+        <v>-7.99</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>28.92</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>28.59</v>
       </c>
       <c r="AE9" t="n">
-        <v>55.06</v>
+        <v>46.51</v>
       </c>
       <c r="AF9" t="n">
-        <v>11.32</v>
+        <v>39.41</v>
       </c>
       <c r="AG9" t="n">
-        <v>33.74</v>
+        <v>38.28</v>
       </c>
       <c r="AH9" t="n">
-        <v>-5.83</v>
-      </c>
-      <c r="AI9" t="n">
-        <v>24.26</v>
+        <v>41.16</v>
       </c>
       <c r="AJ9" t="n">
-        <v>35.42</v>
+        <v>33.83</v>
       </c>
       <c r="AK9" t="n">
-        <v>28.52</v>
+        <v>-9.130000000000001</v>
       </c>
       <c r="AL9" t="n">
-        <v>30.02</v>
+        <v>40.39</v>
       </c>
       <c r="AM9" t="n">
-        <v>33.16</v>
+        <v>27.15</v>
       </c>
       <c r="AN9" t="n">
-        <v>-10.45</v>
+        <v>-5.59</v>
       </c>
       <c r="AO9" t="n">
-        <v>38.13</v>
+        <v>32.81</v>
       </c>
       <c r="AP9" t="n">
-        <v>18.52</v>
+        <v>31.34</v>
       </c>
       <c r="AQ9" t="n">
-        <v>20.39</v>
-      </c>
-      <c r="AR9" t="n">
-        <v>19.17</v>
+        <v>27.97</v>
       </c>
       <c r="AS9" t="n">
-        <v>19.86</v>
+        <v>19.94</v>
       </c>
       <c r="AT9" t="n">
-        <v>27.42</v>
+        <v>42.72</v>
       </c>
       <c r="AU9" t="n">
-        <v>40.25</v>
+        <v>9.73</v>
       </c>
       <c r="AV9" t="n">
-        <v>24.8</v>
+        <v>20.09</v>
       </c>
       <c r="AW9" t="n">
-        <v>38.85</v>
+        <v>29.17</v>
       </c>
       <c r="AX9" t="n">
-        <v>30.56</v>
+        <v>25.5</v>
       </c>
       <c r="AY9" t="n">
-        <v>19.88</v>
+        <v>30.44</v>
       </c>
       <c r="AZ9" t="n">
-        <v>21.27</v>
+        <v>39.1</v>
       </c>
       <c r="BA9" t="n">
-        <v>17.06</v>
+        <v>12.82</v>
       </c>
       <c r="BB9" t="n">
-        <v>11.68</v>
+        <v>31.8</v>
       </c>
       <c r="BC9" t="n">
-        <v>15.24</v>
+        <v>15.09</v>
+      </c>
+      <c r="BD9" t="n">
+        <v>31.52</v>
       </c>
       <c r="BE9" t="n">
-        <v>31.16</v>
+        <v>19.05</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>40.75</v>
+      </c>
+      <c r="BH9" t="n">
+        <v>19.39</v>
+      </c>
+      <c r="BI9" t="n">
+        <v>42.82</v>
+      </c>
+      <c r="BJ9" t="n">
+        <v>-10.57</v>
+      </c>
+      <c r="BK9" t="n">
+        <v>49.87</v>
+      </c>
+      <c r="BL9" t="n">
+        <v>40.77</v>
+      </c>
+      <c r="BM9" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="BN9" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="BO9" t="n">
+        <v>25.47</v>
+      </c>
+      <c r="BR9" t="n">
+        <v>41.82</v>
+      </c>
+      <c r="BS9" t="n">
+        <v>24.16</v>
+      </c>
+      <c r="BT9" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="BU9" t="n">
+        <v>36.43</v>
       </c>
     </row>
     <row r="10">
@@ -2278,106 +2679,160 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>2.39</v>
+        <v>66.78</v>
       </c>
       <c r="Q10" t="n">
-        <v>19.43</v>
+        <v>47.97</v>
       </c>
       <c r="R10" t="n">
-        <v>29.77</v>
+        <v>46.64</v>
       </c>
       <c r="S10" t="n">
-        <v>16.18</v>
+        <v>30.06</v>
+      </c>
+      <c r="T10" t="n">
+        <v>19.03</v>
       </c>
       <c r="U10" t="n">
-        <v>39.77</v>
+        <v>24.02</v>
       </c>
       <c r="V10" t="n">
-        <v>42.98</v>
+        <v>90.63</v>
       </c>
       <c r="W10" t="n">
-        <v>28.03</v>
+        <v>45.54</v>
+      </c>
+      <c r="X10" t="n">
+        <v>68.48</v>
       </c>
       <c r="Y10" t="n">
-        <v>17.27</v>
+        <v>50.06</v>
       </c>
       <c r="Z10" t="n">
-        <v>19.72</v>
+        <v>24.39</v>
       </c>
       <c r="AA10" t="n">
-        <v>14.87</v>
+        <v>44.55</v>
       </c>
       <c r="AB10" t="n">
-        <v>43.29</v>
+        <v>60.73</v>
       </c>
       <c r="AC10" t="n">
-        <v>28.07</v>
+        <v>56.74</v>
       </c>
       <c r="AE10" t="n">
-        <v>31.5</v>
+        <v>57.56</v>
       </c>
       <c r="AF10" t="n">
-        <v>21.17</v>
+        <v>68.04000000000001</v>
       </c>
       <c r="AG10" t="n">
-        <v>21.21</v>
+        <v>55.88</v>
       </c>
       <c r="AH10" t="n">
-        <v>25.38</v>
+        <v>67.3</v>
       </c>
       <c r="AI10" t="n">
-        <v>24.28</v>
+        <v>24.74</v>
       </c>
       <c r="AJ10" t="n">
-        <v>3.91</v>
+        <v>46.02</v>
       </c>
       <c r="AK10" t="n">
-        <v>33.51</v>
+        <v>40.01</v>
       </c>
       <c r="AL10" t="n">
-        <v>-9.35</v>
+        <v>36.7</v>
       </c>
       <c r="AM10" t="n">
-        <v>4.92</v>
+        <v>48.69</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>101.66</v>
       </c>
       <c r="AO10" t="n">
-        <v>32.73</v>
+        <v>34.88</v>
       </c>
       <c r="AP10" t="n">
-        <v>19.59</v>
+        <v>84.8</v>
       </c>
       <c r="AQ10" t="n">
-        <v>32.09</v>
+        <v>44.95</v>
       </c>
       <c r="AR10" t="n">
-        <v>18.61</v>
+        <v>68.29000000000001</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>35.55</v>
       </c>
       <c r="AT10" t="n">
-        <v>14.41</v>
+        <v>53.2</v>
       </c>
       <c r="AU10" t="n">
-        <v>22.14</v>
+        <v>37.53</v>
       </c>
       <c r="AV10" t="n">
-        <v>23.89</v>
-      </c>
-      <c r="AW10" t="n">
-        <v>22.84</v>
+        <v>55.49</v>
       </c>
       <c r="AY10" t="n">
-        <v>29.59</v>
+        <v>71.64</v>
       </c>
       <c r="AZ10" t="n">
-        <v>25.18</v>
+        <v>48.93</v>
+      </c>
+      <c r="BA10" t="n">
+        <v>55.09</v>
+      </c>
+      <c r="BB10" t="n">
+        <v>61.72</v>
       </c>
       <c r="BC10" t="n">
-        <v>30.66</v>
+        <v>63.4</v>
       </c>
       <c r="BD10" t="n">
-        <v>26.52</v>
+        <v>-15.07</v>
       </c>
       <c r="BE10" t="n">
-        <v>27.77</v>
+        <v>52.6</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>48.83</v>
+      </c>
+      <c r="BG10" t="n">
+        <v>29.94</v>
+      </c>
+      <c r="BI10" t="n">
+        <v>57.49</v>
+      </c>
+      <c r="BJ10" t="n">
+        <v>32.65</v>
+      </c>
+      <c r="BL10" t="n">
+        <v>52.52</v>
+      </c>
+      <c r="BM10" t="n">
+        <v>62.13</v>
+      </c>
+      <c r="BN10" t="n">
+        <v>48.06</v>
+      </c>
+      <c r="BP10" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="BQ10" t="n">
+        <v>34.93</v>
+      </c>
+      <c r="BR10" t="n">
+        <v>45.96</v>
+      </c>
+      <c r="BS10" t="n">
+        <v>83.93000000000001</v>
+      </c>
+      <c r="BT10" t="n">
+        <v>55.28</v>
+      </c>
+      <c r="BU10" t="n">
+        <v>-15.15</v>
       </c>
     </row>
     <row r="11">
@@ -2457,112 +2912,148 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>49.75</v>
+        <v>46.55</v>
       </c>
       <c r="Q11" t="n">
-        <v>-17.68</v>
+        <v>32.11</v>
       </c>
       <c r="R11" t="n">
-        <v>76.8</v>
+        <v>-22.76</v>
       </c>
       <c r="S11" t="n">
-        <v>-12.28</v>
+        <v>-14.61</v>
       </c>
       <c r="T11" t="n">
-        <v>33.82</v>
+        <v>-21.9</v>
       </c>
       <c r="U11" t="n">
-        <v>-23.47</v>
+        <v>-3.22</v>
+      </c>
+      <c r="V11" t="n">
+        <v>60.91</v>
       </c>
       <c r="W11" t="n">
-        <v>75.14</v>
+        <v>42.05</v>
       </c>
       <c r="X11" t="n">
-        <v>66.5</v>
+        <v>100.14</v>
       </c>
       <c r="Y11" t="n">
-        <v>37.19</v>
+        <v>97.86</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>42.75</v>
       </c>
       <c r="AA11" t="n">
-        <v>55.38</v>
+        <v>13.89</v>
       </c>
       <c r="AB11" t="n">
-        <v>63.74</v>
-      </c>
-      <c r="AC11" t="n">
-        <v>26.59</v>
+        <v>68.63</v>
       </c>
       <c r="AD11" t="n">
-        <v>38.99</v>
-      </c>
-      <c r="AE11" t="n">
-        <v>66.02</v>
+        <v>80.87</v>
       </c>
       <c r="AF11" t="n">
-        <v>-26.09</v>
+        <v>41.02</v>
       </c>
       <c r="AG11" t="n">
-        <v>98.55</v>
+        <v>35.33</v>
       </c>
       <c r="AI11" t="n">
-        <v>69.86</v>
+        <v>84.05</v>
       </c>
       <c r="AJ11" t="n">
-        <v>35.08</v>
-      </c>
-      <c r="AK11" t="n">
-        <v>41.01</v>
+        <v>57.59</v>
       </c>
       <c r="AL11" t="n">
-        <v>84.39</v>
+        <v>133.38</v>
       </c>
       <c r="AM11" t="n">
-        <v>44.04</v>
+        <v>42.63</v>
       </c>
       <c r="AN11" t="n">
-        <v>48.28</v>
-      </c>
-      <c r="AO11" t="n">
-        <v>91.2</v>
-      </c>
-      <c r="AP11" t="n">
-        <v>85.18000000000001</v>
+        <v>14.83</v>
       </c>
       <c r="AQ11" t="n">
-        <v>91.67</v>
+        <v>52.23</v>
       </c>
       <c r="AR11" t="n">
-        <v>12.92</v>
+        <v>85.15000000000001</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>39.86</v>
       </c>
       <c r="AT11" t="n">
-        <v>67.67</v>
+        <v>96.79000000000001</v>
       </c>
       <c r="AU11" t="n">
-        <v>45.28</v>
+        <v>67.81999999999999</v>
       </c>
       <c r="AV11" t="n">
-        <v>101.98</v>
+        <v>79.44</v>
       </c>
       <c r="AW11" t="n">
-        <v>61.39</v>
+        <v>66.43000000000001</v>
       </c>
       <c r="AX11" t="n">
-        <v>93.77</v>
+        <v>86.17</v>
       </c>
       <c r="AY11" t="n">
-        <v>66.40000000000001</v>
+        <v>55.67</v>
       </c>
       <c r="AZ11" t="n">
-        <v>53.34</v>
-      </c>
-      <c r="BC11" t="n">
-        <v>24.11</v>
+        <v>68.45999999999999</v>
+      </c>
+      <c r="BA11" t="n">
+        <v>98.38</v>
+      </c>
+      <c r="BB11" t="n">
+        <v>86.61</v>
       </c>
       <c r="BD11" t="n">
-        <v>55.5</v>
+        <v>103.73</v>
       </c>
       <c r="BE11" t="n">
-        <v>90.28</v>
+        <v>38.56</v>
+      </c>
+      <c r="BF11" t="n">
+        <v>55.74</v>
+      </c>
+      <c r="BG11" t="n">
+        <v>67.13</v>
+      </c>
+      <c r="BI11" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="BJ11" t="n">
+        <v>99.2</v>
+      </c>
+      <c r="BK11" t="n">
+        <v>105.59</v>
+      </c>
+      <c r="BL11" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="BN11" t="n">
+        <v>51.55</v>
+      </c>
+      <c r="BO11" t="n">
+        <v>47.56</v>
+      </c>
+      <c r="BP11" t="n">
+        <v>58.19</v>
+      </c>
+      <c r="BQ11" t="n">
+        <v>56.22</v>
+      </c>
+      <c r="BS11" t="n">
+        <v>75.94</v>
+      </c>
+      <c r="BT11" t="n">
+        <v>79.45999999999999</v>
+      </c>
+      <c r="BU11" t="n">
+        <v>104.04</v>
       </c>
     </row>
     <row r="12">
@@ -2641,107 +3132,173 @@
           <t>PR11020100 - GPS Current Accounts - Other</t>
         </is>
       </c>
+      <c r="P12" t="n">
+        <v>45.64</v>
+      </c>
       <c r="Q12" t="n">
-        <v>81.78</v>
+        <v>46.47</v>
       </c>
       <c r="R12" t="n">
-        <v>-41.75</v>
+        <v>71.29000000000001</v>
       </c>
       <c r="S12" t="n">
-        <v>88.58</v>
+        <v>71.2</v>
       </c>
       <c r="T12" t="n">
-        <v>89.48999999999999</v>
-      </c>
-      <c r="U12" t="n">
-        <v>89.93000000000001</v>
-      </c>
-      <c r="V12" t="n">
-        <v>95.34999999999999</v>
+        <v>41.43</v>
       </c>
       <c r="W12" t="n">
-        <v>30.98</v>
+        <v>42.92</v>
+      </c>
+      <c r="X12" t="n">
+        <v>59.65</v>
       </c>
       <c r="Y12" t="n">
-        <v>-27.52</v>
+        <v>62.28</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>61.84</v>
       </c>
       <c r="AA12" t="n">
-        <v>119.07</v>
+        <v>-22.47</v>
       </c>
       <c r="AB12" t="n">
-        <v>59.75</v>
+        <v>88.19</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>63.34</v>
       </c>
       <c r="AE12" t="n">
-        <v>105.95</v>
+        <v>95.93000000000001</v>
       </c>
       <c r="AF12" t="n">
-        <v>49.53</v>
+        <v>97.27</v>
       </c>
       <c r="AG12" t="n">
-        <v>93.62</v>
+        <v>78.19</v>
       </c>
       <c r="AH12" t="n">
-        <v>134.63</v>
+        <v>90.36</v>
       </c>
       <c r="AI12" t="n">
-        <v>82.09999999999999</v>
+        <v>88.70999999999999</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>65.97</v>
       </c>
       <c r="AK12" t="n">
-        <v>108.72</v>
+        <v>45.19</v>
       </c>
       <c r="AL12" t="n">
-        <v>83.40000000000001</v>
+        <v>-23.52</v>
       </c>
       <c r="AM12" t="n">
-        <v>33</v>
+        <v>6.84</v>
       </c>
       <c r="AN12" t="n">
-        <v>48.37</v>
+        <v>-22.68</v>
       </c>
       <c r="AO12" t="n">
-        <v>59.24</v>
+        <v>107.45</v>
       </c>
       <c r="AP12" t="n">
-        <v>93.33</v>
+        <v>51.21</v>
       </c>
       <c r="AQ12" t="n">
-        <v>37.56</v>
+        <v>110.6</v>
       </c>
       <c r="AR12" t="n">
-        <v>46.27</v>
+        <v>48.38</v>
       </c>
       <c r="AS12" t="n">
-        <v>-13.96</v>
+        <v>-26.95</v>
       </c>
       <c r="AT12" t="n">
-        <v>-25.03</v>
+        <v>110.63</v>
       </c>
       <c r="AU12" t="n">
-        <v>116.17</v>
+        <v>119.19</v>
       </c>
       <c r="AV12" t="n">
-        <v>-44.59</v>
+        <v>75.20999999999999</v>
       </c>
       <c r="AW12" t="n">
-        <v>113.05</v>
+        <v>43.74</v>
       </c>
       <c r="AX12" t="n">
-        <v>56.03</v>
+        <v>132.76</v>
       </c>
       <c r="AY12" t="n">
-        <v>90.23</v>
+        <v>92.26000000000001</v>
       </c>
       <c r="AZ12" t="n">
-        <v>108.95</v>
+        <v>82.2</v>
       </c>
       <c r="BA12" t="n">
-        <v>48.39</v>
+        <v>53.8</v>
+      </c>
+      <c r="BB12" t="n">
+        <v>75.66</v>
+      </c>
+      <c r="BC12" t="n">
+        <v>70.5</v>
       </c>
       <c r="BD12" t="n">
-        <v>63.64</v>
+        <v>101.59</v>
       </c>
       <c r="BE12" t="n">
-        <v>134.17</v>
+        <v>88.54000000000001</v>
+      </c>
+      <c r="BF12" t="n">
+        <v>54.05</v>
+      </c>
+      <c r="BG12" t="n">
+        <v>-21.48</v>
+      </c>
+      <c r="BH12" t="n">
+        <v>36.85</v>
+      </c>
+      <c r="BI12" t="n">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="BJ12" t="n">
+        <v>42.66</v>
+      </c>
+      <c r="BK12" t="n">
+        <v>39.78</v>
+      </c>
+      <c r="BL12" t="n">
+        <v>-12.67</v>
+      </c>
+      <c r="BM12" t="n">
+        <v>82.15000000000001</v>
+      </c>
+      <c r="BN12" t="n">
+        <v>81.43000000000001</v>
+      </c>
+      <c r="BO12" t="n">
+        <v>87.64</v>
+      </c>
+      <c r="BP12" t="n">
+        <v>-5.2</v>
+      </c>
+      <c r="BQ12" t="n">
+        <v>84.44</v>
+      </c>
+      <c r="BR12" t="n">
+        <v>101.38</v>
+      </c>
+      <c r="BS12" t="n">
+        <v>99.31999999999999</v>
+      </c>
+      <c r="BT12" t="n">
+        <v>64.92</v>
+      </c>
+      <c r="BU12" t="n">
+        <v>64.95999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -2821,115 +3378,154 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>44.07</v>
+        <v>18.34</v>
       </c>
       <c r="Q13" t="n">
-        <v>53.72</v>
+        <v>30.51</v>
       </c>
       <c r="R13" t="n">
-        <v>27.43</v>
+        <v>42.56</v>
+      </c>
+      <c r="S13" t="n">
+        <v>52.36</v>
+      </c>
+      <c r="T13" t="n">
+        <v>24.94</v>
       </c>
       <c r="U13" t="n">
-        <v>35.62</v>
+        <v>54.74</v>
       </c>
       <c r="V13" t="n">
-        <v>31.99</v>
+        <v>30.67</v>
       </c>
       <c r="W13" t="n">
-        <v>20.25</v>
+        <v>30.94</v>
       </c>
       <c r="X13" t="n">
-        <v>25.56</v>
+        <v>22.86</v>
       </c>
       <c r="Y13" t="n">
-        <v>96.43000000000001</v>
+        <v>7</v>
       </c>
       <c r="Z13" t="n">
-        <v>48.46</v>
+        <v>26.84</v>
       </c>
       <c r="AA13" t="n">
-        <v>72.87</v>
+        <v>34.17</v>
       </c>
       <c r="AB13" t="n">
-        <v>53.27</v>
+        <v>-15.21</v>
       </c>
       <c r="AC13" t="n">
-        <v>25.96</v>
-      </c>
-      <c r="AD13" t="n">
-        <v>47.4</v>
+        <v>32.26</v>
       </c>
       <c r="AE13" t="n">
-        <v>64.62</v>
+        <v>28.09</v>
       </c>
       <c r="AF13" t="n">
-        <v>60.38</v>
+        <v>55.34</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>23.84</v>
       </c>
       <c r="AH13" t="n">
-        <v>61.25</v>
+        <v>17.84</v>
       </c>
       <c r="AI13" t="n">
-        <v>72.40000000000001</v>
+        <v>13.12</v>
       </c>
       <c r="AJ13" t="n">
-        <v>59.47</v>
+        <v>57.14</v>
       </c>
       <c r="AK13" t="n">
-        <v>71.61</v>
+        <v>23.35</v>
       </c>
       <c r="AL13" t="n">
-        <v>26.33</v>
+        <v>45.09</v>
       </c>
       <c r="AM13" t="n">
-        <v>48.98</v>
+        <v>33.14</v>
       </c>
       <c r="AN13" t="n">
-        <v>42.58</v>
-      </c>
-      <c r="AO13" t="n">
-        <v>39.05</v>
+        <v>34.49</v>
       </c>
       <c r="AP13" t="n">
-        <v>51.81</v>
+        <v>32.24</v>
       </c>
       <c r="AQ13" t="n">
-        <v>108.18</v>
+        <v>20.23</v>
       </c>
       <c r="AR13" t="n">
-        <v>37.12</v>
+        <v>29.69</v>
       </c>
       <c r="AS13" t="n">
-        <v>90.23999999999999</v>
+        <v>38.63</v>
       </c>
       <c r="AT13" t="n">
-        <v>47.83</v>
+        <v>37.87</v>
       </c>
       <c r="AU13" t="n">
-        <v>72.66</v>
+        <v>37.18</v>
       </c>
       <c r="AV13" t="n">
-        <v>37.83</v>
+        <v>18.72</v>
       </c>
       <c r="AW13" t="n">
-        <v>56.61</v>
+        <v>39.88</v>
       </c>
       <c r="AX13" t="n">
-        <v>39.93</v>
+        <v>20.91</v>
       </c>
       <c r="AY13" t="n">
-        <v>59.05</v>
+        <v>29.42</v>
+      </c>
+      <c r="AZ13" t="n">
+        <v>41.24</v>
+      </c>
+      <c r="BA13" t="n">
+        <v>-8.210000000000001</v>
       </c>
       <c r="BB13" t="n">
-        <v>76.23</v>
-      </c>
-      <c r="BC13" t="n">
-        <v>52.07</v>
-      </c>
-      <c r="BD13" t="n">
-        <v>58.62</v>
+        <v>51.06</v>
       </c>
       <c r="BE13" t="n">
-        <v>65.68000000000001</v>
+        <v>21.92</v>
+      </c>
+      <c r="BF13" t="n">
+        <v>41.07</v>
+      </c>
+      <c r="BH13" t="n">
+        <v>28.85</v>
+      </c>
+      <c r="BI13" t="n">
+        <v>48.83</v>
+      </c>
+      <c r="BJ13" t="n">
+        <v>23.82</v>
+      </c>
+      <c r="BK13" t="n">
+        <v>25.89</v>
+      </c>
+      <c r="BL13" t="n">
+        <v>35.09</v>
+      </c>
+      <c r="BM13" t="n">
+        <v>41.98</v>
+      </c>
+      <c r="BN13" t="n">
+        <v>32</v>
+      </c>
+      <c r="BP13" t="n">
+        <v>28.84</v>
+      </c>
+      <c r="BQ13" t="n">
+        <v>39.48</v>
+      </c>
+      <c r="BS13" t="n">
+        <v>41.77</v>
+      </c>
+      <c r="BU13" t="n">
+        <v>37.97</v>
       </c>
     </row>
     <row r="14">
@@ -3008,110 +3604,164 @@
           <t>PR05040400 - Term Deposits Liabilities - Other</t>
         </is>
       </c>
-      <c r="P14" t="n">
-        <v>103.67</v>
-      </c>
       <c r="Q14" t="n">
-        <v>97.14</v>
+        <v>36.89</v>
       </c>
       <c r="R14" t="n">
-        <v>85.45</v>
+        <v>28.1</v>
       </c>
       <c r="S14" t="n">
-        <v>70.81999999999999</v>
+        <v>-24.02</v>
       </c>
       <c r="T14" t="n">
-        <v>-24.76</v>
-      </c>
-      <c r="U14" t="n">
-        <v>94.01000000000001</v>
+        <v>116.96</v>
       </c>
       <c r="V14" t="n">
-        <v>53.39</v>
+        <v>-24.81</v>
+      </c>
+      <c r="W14" t="n">
+        <v>61.61</v>
       </c>
       <c r="X14" t="n">
-        <v>85.89</v>
+        <v>23.46</v>
       </c>
       <c r="Y14" t="n">
-        <v>101.6</v>
+        <v>27.47</v>
       </c>
       <c r="Z14" t="n">
-        <v>78.59</v>
+        <v>84.89</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>29.1</v>
       </c>
       <c r="AB14" t="n">
-        <v>74.23</v>
+        <v>50.37</v>
       </c>
       <c r="AC14" t="n">
-        <v>57.13</v>
-      </c>
-      <c r="AD14" t="n">
-        <v>75.16</v>
+        <v>-16.66</v>
       </c>
       <c r="AE14" t="n">
-        <v>137.25</v>
+        <v>43.38</v>
       </c>
       <c r="AF14" t="n">
-        <v>90.39</v>
+        <v>20.79</v>
       </c>
       <c r="AG14" t="n">
-        <v>-24.77</v>
+        <v>50.06</v>
       </c>
       <c r="AH14" t="n">
-        <v>58.4</v>
+        <v>55.99</v>
       </c>
       <c r="AI14" t="n">
-        <v>91.11</v>
+        <v>47.8</v>
       </c>
       <c r="AJ14" t="n">
-        <v>52.33</v>
+        <v>71.15000000000001</v>
       </c>
       <c r="AL14" t="n">
-        <v>-18.33</v>
-      </c>
-      <c r="AM14" t="n">
-        <v>-27.47</v>
+        <v>58.87</v>
       </c>
       <c r="AN14" t="n">
-        <v>-4.04</v>
+        <v>45.51</v>
       </c>
       <c r="AO14" t="n">
-        <v>76.41</v>
+        <v>-19.8</v>
       </c>
       <c r="AP14" t="n">
-        <v>52.75</v>
+        <v>48.49</v>
       </c>
       <c r="AQ14" t="n">
-        <v>125.63</v>
+        <v>93.45</v>
       </c>
       <c r="AR14" t="n">
-        <v>122.77</v>
+        <v>50.2</v>
       </c>
       <c r="AS14" t="n">
-        <v>53.63</v>
+        <v>72.94</v>
       </c>
       <c r="AT14" t="n">
-        <v>17.42</v>
+        <v>103.03</v>
       </c>
       <c r="AU14" t="n">
-        <v>86.09999999999999</v>
+        <v>75.86</v>
+      </c>
+      <c r="AV14" t="n">
+        <v>3.63</v>
       </c>
       <c r="AW14" t="n">
-        <v>101.46</v>
+        <v>59.02</v>
+      </c>
+      <c r="AX14" t="n">
+        <v>47.63</v>
       </c>
       <c r="AY14" t="n">
-        <v>51.46</v>
+        <v>63.28</v>
       </c>
       <c r="AZ14" t="n">
-        <v>44.33</v>
+        <v>47.64</v>
+      </c>
+      <c r="BA14" t="n">
+        <v>87.52</v>
       </c>
       <c r="BB14" t="n">
-        <v>105.44</v>
+        <v>47.42</v>
       </c>
       <c r="BC14" t="n">
-        <v>72.25</v>
+        <v>53.73</v>
+      </c>
+      <c r="BD14" t="n">
+        <v>62.62</v>
       </c>
       <c r="BE14" t="n">
-        <v>167.34</v>
+        <v>50.26</v>
+      </c>
+      <c r="BF14" t="n">
+        <v>24.85</v>
+      </c>
+      <c r="BG14" t="n">
+        <v>32.85</v>
+      </c>
+      <c r="BH14" t="n">
+        <v>17.24</v>
+      </c>
+      <c r="BI14" t="n">
+        <v>-18.83</v>
+      </c>
+      <c r="BJ14" t="n">
+        <v>67.31</v>
+      </c>
+      <c r="BK14" t="n">
+        <v>55.16</v>
+      </c>
+      <c r="BL14" t="n">
+        <v>70.14</v>
+      </c>
+      <c r="BM14" t="n">
+        <v>100.44</v>
+      </c>
+      <c r="BN14" t="n">
+        <v>47.59</v>
+      </c>
+      <c r="BO14" t="n">
+        <v>69.66</v>
+      </c>
+      <c r="BP14" t="n">
+        <v>19.71</v>
+      </c>
+      <c r="BQ14" t="n">
+        <v>64.87</v>
+      </c>
+      <c r="BR14" t="n">
+        <v>59.56</v>
+      </c>
+      <c r="BS14" t="n">
+        <v>68.66</v>
+      </c>
+      <c r="BT14" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="BU14" t="n">
+        <v>72.27</v>
       </c>
     </row>
     <row r="15">
@@ -3191,115 +3841,145 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>115.17</v>
+        <v>77.88</v>
       </c>
       <c r="Q15" t="n">
-        <v>-27.48</v>
+        <v>132.39</v>
+      </c>
+      <c r="R15" t="n">
+        <v>85.05</v>
       </c>
       <c r="S15" t="n">
-        <v>74.83</v>
+        <v>63.85</v>
       </c>
       <c r="T15" t="n">
-        <v>121.99</v>
+        <v>-22.24</v>
       </c>
       <c r="U15" t="n">
-        <v>57.11</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="V15" t="n">
-        <v>138.68</v>
+        <v>82.89</v>
       </c>
       <c r="W15" t="n">
-        <v>97.17</v>
-      </c>
-      <c r="X15" t="n">
-        <v>113.81</v>
+        <v>51.42</v>
       </c>
       <c r="Y15" t="n">
-        <v>95.17</v>
+        <v>53.04</v>
       </c>
       <c r="Z15" t="n">
-        <v>123.45</v>
+        <v>108.15</v>
       </c>
       <c r="AA15" t="n">
-        <v>79.76000000000001</v>
+        <v>-34.75</v>
       </c>
       <c r="AB15" t="n">
-        <v>98.09</v>
+        <v>81.76000000000001</v>
       </c>
       <c r="AC15" t="n">
-        <v>140.95</v>
+        <v>131.45</v>
       </c>
       <c r="AD15" t="n">
-        <v>124.09</v>
-      </c>
-      <c r="AF15" t="n">
-        <v>148.62</v>
+        <v>85.81</v>
       </c>
       <c r="AG15" t="n">
-        <v>55.25</v>
+        <v>92.54000000000001</v>
       </c>
       <c r="AH15" t="n">
-        <v>79.86</v>
+        <v>112.37</v>
       </c>
       <c r="AI15" t="n">
-        <v>96.18000000000001</v>
+        <v>50.16</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>100.46</v>
       </c>
       <c r="AK15" t="n">
-        <v>55.44</v>
-      </c>
-      <c r="AL15" t="n">
-        <v>142.13</v>
+        <v>48.7</v>
       </c>
       <c r="AM15" t="n">
-        <v>151.28</v>
-      </c>
-      <c r="AN15" t="n">
-        <v>96.98999999999999</v>
+        <v>34.59</v>
       </c>
       <c r="AP15" t="n">
-        <v>73.86</v>
+        <v>50.31</v>
       </c>
       <c r="AQ15" t="n">
-        <v>68.14</v>
-      </c>
-      <c r="AR15" t="n">
-        <v>83.37</v>
+        <v>80.31</v>
       </c>
       <c r="AS15" t="n">
-        <v>80.54000000000001</v>
-      </c>
-      <c r="AU15" t="n">
-        <v>108.8</v>
-      </c>
-      <c r="AV15" t="n">
-        <v>113.85</v>
+        <v>98.95999999999999</v>
+      </c>
+      <c r="AT15" t="n">
+        <v>85.40000000000001</v>
       </c>
       <c r="AW15" t="n">
-        <v>149.06</v>
+        <v>-32.84</v>
       </c>
       <c r="AX15" t="n">
-        <v>56.8</v>
+        <v>58.89</v>
       </c>
       <c r="AY15" t="n">
-        <v>83.45</v>
+        <v>40.19</v>
       </c>
       <c r="AZ15" t="n">
-        <v>136.81</v>
+        <v>-16.76</v>
       </c>
       <c r="BA15" t="n">
-        <v>67.67</v>
+        <v>83.47</v>
       </c>
       <c r="BB15" t="n">
-        <v>51.52</v>
+        <v>133.49</v>
       </c>
       <c r="BC15" t="n">
-        <v>107.33</v>
+        <v>133.81</v>
       </c>
       <c r="BD15" t="n">
-        <v>98.95999999999999</v>
-      </c>
-      <c r="BE15" t="n">
-        <v>55.11</v>
+        <v>144.95</v>
+      </c>
+      <c r="BF15" t="n">
+        <v>93.84</v>
+      </c>
+      <c r="BG15" t="n">
+        <v>58.52</v>
+      </c>
+      <c r="BH15" t="n">
+        <v>102.35</v>
+      </c>
+      <c r="BI15" t="n">
+        <v>84.44</v>
+      </c>
+      <c r="BJ15" t="n">
+        <v>41.71</v>
+      </c>
+      <c r="BL15" t="n">
+        <v>97.89</v>
+      </c>
+      <c r="BM15" t="n">
+        <v>94.43000000000001</v>
+      </c>
+      <c r="BN15" t="n">
+        <v>88.3</v>
+      </c>
+      <c r="BO15" t="n">
+        <v>82.53</v>
+      </c>
+      <c r="BP15" t="n">
+        <v>82.06</v>
+      </c>
+      <c r="BQ15" t="n">
+        <v>92.04000000000001</v>
+      </c>
+      <c r="BR15" t="n">
+        <v>-32.58</v>
+      </c>
+      <c r="BS15" t="n">
+        <v>111.91</v>
+      </c>
+      <c r="BT15" t="n">
+        <v>101.22</v>
+      </c>
+      <c r="BU15" t="n">
+        <v>132.37</v>
       </c>
     </row>
     <row r="16">
@@ -3379,124 +4059,148 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>96.41</v>
+        <v>162.38</v>
       </c>
       <c r="Q16" t="n">
-        <v>90.95</v>
+        <v>139.87</v>
+      </c>
+      <c r="S16" t="n">
+        <v>144.15</v>
       </c>
       <c r="T16" t="n">
-        <v>38.49</v>
+        <v>145.22</v>
       </c>
       <c r="U16" t="n">
-        <v>58.81</v>
+        <v>132.04</v>
       </c>
       <c r="V16" t="n">
-        <v>62.61</v>
+        <v>144.92</v>
       </c>
       <c r="W16" t="n">
-        <v>94.81</v>
+        <v>139.32</v>
       </c>
       <c r="X16" t="n">
-        <v>96.14</v>
+        <v>99.7</v>
       </c>
       <c r="Y16" t="n">
-        <v>77.28</v>
+        <v>150.08</v>
       </c>
       <c r="Z16" t="n">
-        <v>89.3</v>
+        <v>74.64</v>
       </c>
       <c r="AA16" t="n">
-        <v>87.68000000000001</v>
+        <v>207.58</v>
       </c>
       <c r="AB16" t="n">
-        <v>65.2</v>
+        <v>101.17</v>
       </c>
       <c r="AC16" t="n">
-        <v>44.67</v>
+        <v>178.72</v>
       </c>
       <c r="AD16" t="n">
-        <v>-23.24</v>
+        <v>134.16</v>
       </c>
       <c r="AE16" t="n">
-        <v>6.76</v>
+        <v>79.94</v>
       </c>
       <c r="AF16" t="n">
-        <v>-22.42</v>
+        <v>95.87</v>
       </c>
       <c r="AG16" t="n">
-        <v>106.2</v>
+        <v>70.23</v>
       </c>
       <c r="AH16" t="n">
-        <v>50.62</v>
+        <v>101.27</v>
       </c>
       <c r="AI16" t="n">
-        <v>109.31</v>
+        <v>178.55</v>
       </c>
       <c r="AJ16" t="n">
-        <v>47.82</v>
+        <v>97.01000000000001</v>
       </c>
       <c r="AK16" t="n">
-        <v>-26.64</v>
-      </c>
-      <c r="AL16" t="n">
-        <v>109.34</v>
+        <v>94.73999999999999</v>
       </c>
       <c r="AM16" t="n">
-        <v>117.8</v>
+        <v>76.22</v>
       </c>
       <c r="AN16" t="n">
-        <v>74.33</v>
+        <v>122.9</v>
       </c>
       <c r="AO16" t="n">
-        <v>43.23</v>
+        <v>127.31</v>
       </c>
       <c r="AP16" t="n">
-        <v>131.22</v>
-      </c>
-      <c r="AQ16" t="n">
-        <v>91.19</v>
+        <v>79.94</v>
       </c>
       <c r="AR16" t="n">
-        <v>81.23999999999999</v>
-      </c>
-      <c r="AS16" t="n">
-        <v>53.17</v>
+        <v>96.37</v>
       </c>
       <c r="AT16" t="n">
-        <v>74.78</v>
+        <v>85.29000000000001</v>
       </c>
       <c r="AU16" t="n">
-        <v>69.68000000000001</v>
-      </c>
-      <c r="AV16" t="n">
-        <v>100.41</v>
+        <v>119.29</v>
       </c>
       <c r="AW16" t="n">
-        <v>87.51000000000001</v>
+        <v>10.7</v>
       </c>
       <c r="AX16" t="n">
-        <v>53.43</v>
+        <v>70.42</v>
       </c>
       <c r="AY16" t="n">
-        <v>-21.23</v>
+        <v>91.41</v>
       </c>
       <c r="AZ16" t="n">
-        <v>36.42</v>
-      </c>
-      <c r="BA16" t="n">
-        <v>82.92</v>
+        <v>-23.9</v>
       </c>
       <c r="BB16" t="n">
-        <v>42.16</v>
-      </c>
-      <c r="BC16" t="n">
-        <v>39.32</v>
+        <v>117.38</v>
       </c>
       <c r="BD16" t="n">
-        <v>-12.52</v>
+        <v>139.86</v>
       </c>
       <c r="BE16" t="n">
-        <v>81.19</v>
+        <v>145.12</v>
+      </c>
+      <c r="BF16" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="BG16" t="n">
+        <v>141.55</v>
+      </c>
+      <c r="BI16" t="n">
+        <v>80.51000000000001</v>
+      </c>
+      <c r="BJ16" t="n">
+        <v>67.93000000000001</v>
+      </c>
+      <c r="BK16" t="n">
+        <v>145.68</v>
+      </c>
+      <c r="BL16" t="n">
+        <v>161.99</v>
+      </c>
+      <c r="BM16" t="n">
+        <v>-26.91</v>
+      </c>
+      <c r="BN16" t="n">
+        <v>83.7</v>
+      </c>
+      <c r="BO16" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="BP16" t="n">
+        <v>158.79</v>
+      </c>
+      <c r="BS16" t="n">
+        <v>131.58</v>
+      </c>
+      <c r="BT16" t="n">
+        <v>151.19</v>
+      </c>
+      <c r="BU16" t="n">
+        <v>81.91</v>
       </c>
     </row>
     <row r="17">
@@ -3576,118 +4280,151 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>23.39</v>
+        <v>46.27</v>
       </c>
       <c r="Q17" t="n">
-        <v>36.4</v>
+        <v>87.98999999999999</v>
+      </c>
+      <c r="R17" t="n">
+        <v>35.94</v>
       </c>
       <c r="S17" t="n">
-        <v>14.78</v>
+        <v>88.5</v>
       </c>
       <c r="T17" t="n">
-        <v>17.4</v>
+        <v>87.12</v>
       </c>
       <c r="U17" t="n">
-        <v>14.26</v>
+        <v>88.68000000000001</v>
       </c>
       <c r="V17" t="n">
-        <v>14.19</v>
+        <v>91.53</v>
       </c>
       <c r="W17" t="n">
-        <v>33.11</v>
+        <v>104.79</v>
       </c>
       <c r="X17" t="n">
-        <v>24.51</v>
+        <v>72.48999999999999</v>
       </c>
       <c r="Y17" t="n">
-        <v>27.93</v>
+        <v>-28.53</v>
       </c>
       <c r="Z17" t="n">
-        <v>21.12</v>
+        <v>80.42</v>
       </c>
       <c r="AA17" t="n">
-        <v>27.6</v>
+        <v>42.86</v>
       </c>
       <c r="AB17" t="n">
-        <v>24.18</v>
+        <v>71.48999999999999</v>
       </c>
       <c r="AC17" t="n">
-        <v>16.4</v>
+        <v>78.02</v>
       </c>
       <c r="AD17" t="n">
-        <v>30.54</v>
+        <v>75.66</v>
       </c>
       <c r="AE17" t="n">
-        <v>4.68</v>
+        <v>86.3</v>
       </c>
       <c r="AF17" t="n">
-        <v>17.59</v>
-      </c>
-      <c r="AG17" t="n">
-        <v>29.39</v>
-      </c>
-      <c r="AH17" t="n">
-        <v>33.47</v>
+        <v>96.94</v>
       </c>
       <c r="AI17" t="n">
-        <v>17.47</v>
-      </c>
-      <c r="AJ17" t="n">
-        <v>17.75</v>
+        <v>83.29000000000001</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>50.77</v>
       </c>
       <c r="AL17" t="n">
-        <v>13.96</v>
+        <v>110.73</v>
+      </c>
+      <c r="AM17" t="n">
+        <v>101.17</v>
       </c>
       <c r="AN17" t="n">
-        <v>32.33</v>
+        <v>45.37</v>
       </c>
       <c r="AO17" t="n">
-        <v>22.74</v>
+        <v>110.57</v>
       </c>
       <c r="AP17" t="n">
-        <v>17.23</v>
+        <v>85.08</v>
       </c>
       <c r="AQ17" t="n">
-        <v>23.15</v>
+        <v>41.14</v>
       </c>
       <c r="AR17" t="n">
-        <v>31.09</v>
-      </c>
-      <c r="AS17" t="n">
-        <v>27.88</v>
+        <v>83.56999999999999</v>
       </c>
       <c r="AT17" t="n">
-        <v>29.78</v>
+        <v>85.76000000000001</v>
       </c>
       <c r="AU17" t="n">
-        <v>36.88</v>
+        <v>54.83</v>
       </c>
       <c r="AV17" t="n">
-        <v>4</v>
+        <v>107.94</v>
       </c>
       <c r="AW17" t="n">
-        <v>22.95</v>
+        <v>67.63</v>
+      </c>
+      <c r="AX17" t="n">
+        <v>62.25</v>
       </c>
       <c r="AY17" t="n">
-        <v>39.91</v>
+        <v>81.37</v>
       </c>
       <c r="AZ17" t="n">
-        <v>36.39</v>
+        <v>62.7</v>
       </c>
       <c r="BA17" t="n">
-        <v>36.6</v>
+        <v>75.25</v>
       </c>
       <c r="BB17" t="n">
-        <v>16.65</v>
+        <v>34.49</v>
       </c>
       <c r="BC17" t="n">
-        <v>16.56</v>
-      </c>
-      <c r="BD17" t="n">
-        <v>23.96</v>
+        <v>38.17</v>
       </c>
       <c r="BE17" t="n">
-        <v>22.64</v>
+        <v>83.19</v>
+      </c>
+      <c r="BF17" t="n">
+        <v>30.21</v>
+      </c>
+      <c r="BH17" t="n">
+        <v>118.07</v>
+      </c>
+      <c r="BI17" t="n">
+        <v>36.29</v>
+      </c>
+      <c r="BK17" t="n">
+        <v>82.18000000000001</v>
+      </c>
+      <c r="BL17" t="n">
+        <v>77.27</v>
+      </c>
+      <c r="BM17" t="n">
+        <v>92</v>
+      </c>
+      <c r="BN17" t="n">
+        <v>49.31</v>
+      </c>
+      <c r="BQ17" t="n">
+        <v>74.65000000000001</v>
+      </c>
+      <c r="BR17" t="n">
+        <v>-26.89</v>
+      </c>
+      <c r="BS17" t="n">
+        <v>51.15</v>
+      </c>
+      <c r="BT17" t="n">
+        <v>97.34999999999999</v>
+      </c>
+      <c r="BU17" t="n">
+        <v>99.61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Make dashboard self-contained and surface load errors
'Nothing happens on load' was possible because index.html depended on
vendor/xlsx.full.min.js — copying just the HTML file left the Excel
engine missing and every failure was silent. Fixes:

- Embed SheetJS 0.18.5 inside index.html: one file, no vendor/ needed
- Status banner: read/parse progress, loaded-summary, and clear errors
  (unreadable file, empty sheet, no data rows, no period columns)
- Guard when the Excel engine is missing; surface window errors
- Coerce text values: '1,234.50', '(2.26)' accounting negatives,
  and TM1 '-' blank markers now aggregate correctly
- Sample generator emits text-formatted cells to cover this path

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018B5qKH9JxzLywUkLopxf6J
</commit_message>
<xml_diff>
--- a/tm1-dashboard/sample/GPS_Driller_sample.xlsx
+++ b/tm1-dashboard/sample/GPS_Driller_sample.xlsx
@@ -862,152 +862,168 @@
       <c r="Q2" t="n">
         <v>86.05</v>
       </c>
-      <c r="R2" t="n">
-        <v>122.79</v>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="S2" t="n">
-        <v>97.5</v>
+        <v>-36.84</v>
+      </c>
+      <c r="T2" t="n">
+        <v>96.58</v>
       </c>
       <c r="U2" t="n">
-        <v>82.13</v>
-      </c>
-      <c r="V2" t="n">
-        <v>85.31</v>
+        <v>81.56999999999999</v>
+      </c>
+      <c r="W2" t="n">
+        <v>70.51000000000001</v>
       </c>
       <c r="X2" t="n">
-        <v>114.57</v>
+        <v>54.78</v>
       </c>
       <c r="Y2" t="n">
-        <v>117.15</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>135.73</v>
+        <v>38.89</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>48.29</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>38.33</v>
       </c>
       <c r="AC2" t="n">
-        <v>74.20999999999999</v>
+        <v>41.48</v>
       </c>
       <c r="AD2" t="n">
-        <v>44.74</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="AE2" t="n">
-        <v>38.33</v>
+        <v>91.69</v>
       </c>
       <c r="AF2" t="n">
-        <v>-12.44</v>
+        <v>56.01</v>
       </c>
       <c r="AG2" t="n">
-        <v>75.79000000000001</v>
+        <v>48.33</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>39.42</v>
       </c>
       <c r="AI2" t="n">
-        <v>89.40000000000001</v>
+        <v>-19.17</v>
       </c>
       <c r="AJ2" t="n">
-        <v>65.62</v>
+        <v>94.5</v>
       </c>
       <c r="AK2" t="n">
-        <v>92.26000000000001</v>
+        <v>142.34</v>
       </c>
       <c r="AL2" t="n">
-        <v>99.66</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="AM2" t="n">
-        <v>117.62</v>
-      </c>
-      <c r="AN2" t="n">
-        <v>39.42</v>
-      </c>
-      <c r="AO2" t="n">
-        <v>63.91</v>
-      </c>
-      <c r="AQ2" t="n">
-        <v>76.43000000000001</v>
+        <v>99.13</v>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>111.34</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP2" t="n">
+        <v>78.03</v>
       </c>
       <c r="AR2" t="n">
-        <v>97.34</v>
-      </c>
-      <c r="AS2" t="n">
-        <v>30.21</v>
+        <v>112.26</v>
       </c>
       <c r="AT2" t="n">
-        <v>115.71</v>
+        <v>77.70999999999999</v>
       </c>
       <c r="AU2" t="n">
-        <v>75.62</v>
+        <v>70.06999999999999</v>
       </c>
       <c r="AV2" t="n">
-        <v>114.85</v>
+        <v>68.18000000000001</v>
       </c>
       <c r="AW2" t="n">
-        <v>-19.96</v>
-      </c>
-      <c r="AY2" t="n">
-        <v>77.81999999999999</v>
+        <v>104.84</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>133.23</v>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>32.25</t>
+        </is>
       </c>
       <c r="AZ2" t="n">
-        <v>103.37</v>
+        <v>-20.05</v>
       </c>
       <c r="BA2" t="n">
-        <v>89.01000000000001</v>
+        <v>-27.03</v>
       </c>
       <c r="BB2" t="n">
-        <v>122.32</v>
-      </c>
-      <c r="BC2" t="n">
-        <v>81.7</v>
+        <v>58</v>
       </c>
       <c r="BD2" t="n">
-        <v>100.97</v>
+        <v>79.97</v>
       </c>
       <c r="BE2" t="n">
-        <v>97.47</v>
+        <v>64.2</v>
       </c>
       <c r="BF2" t="n">
-        <v>61.29</v>
+        <v>35.41</v>
       </c>
       <c r="BG2" t="n">
-        <v>78.47</v>
+        <v>67.66</v>
       </c>
       <c r="BH2" t="n">
-        <v>66.27</v>
+        <v>92.73999999999999</v>
       </c>
       <c r="BI2" t="n">
-        <v>68.52</v>
+        <v>92.05</v>
       </c>
       <c r="BJ2" t="n">
-        <v>-30.86</v>
+        <v>86.41</v>
       </c>
       <c r="BK2" t="n">
-        <v>78.62</v>
+        <v>137.71</v>
       </c>
       <c r="BL2" t="n">
-        <v>75.18000000000001</v>
+        <v>111.4</v>
       </c>
       <c r="BM2" t="n">
-        <v>87.42</v>
+        <v>64.44</v>
       </c>
       <c r="BN2" t="n">
-        <v>120.69</v>
+        <v>51.18</v>
       </c>
       <c r="BO2" t="n">
-        <v>98.12</v>
+        <v>92.78</v>
       </c>
       <c r="BP2" t="n">
-        <v>73.26000000000001</v>
+        <v>91.95</v>
       </c>
       <c r="BQ2" t="n">
-        <v>134.07</v>
-      </c>
-      <c r="BR2" t="n">
-        <v>85.70999999999999</v>
+        <v>62.66</v>
+      </c>
+      <c r="BR2" t="inlineStr">
+        <is>
+          <t>27.35</t>
+        </is>
       </c>
       <c r="BS2" t="n">
-        <v>101.18</v>
+        <v>97.65000000000001</v>
       </c>
       <c r="BT2" t="n">
-        <v>92.73999999999999</v>
+        <v>88.17</v>
       </c>
       <c r="BU2" t="n">
-        <v>92.05</v>
+        <v>-19.51</v>
       </c>
     </row>
     <row r="3">
@@ -1086,158 +1102,184 @@
           <t>PR05011002 - Current Accounts - Interest Bearing</t>
         </is>
       </c>
+      <c r="P3" t="n">
+        <v>128</v>
+      </c>
       <c r="Q3" t="n">
-        <v>33.37</v>
+        <v>73.73</v>
+      </c>
+      <c r="R3" t="n">
+        <v>86.78</v>
       </c>
       <c r="S3" t="n">
-        <v>53.17</v>
+        <v>-66.8</v>
       </c>
       <c r="T3" t="n">
-        <v>47.07</v>
+        <v>132.89</v>
       </c>
       <c r="U3" t="n">
-        <v>48.69</v>
+        <v>98.95</v>
       </c>
       <c r="V3" t="n">
-        <v>32.08</v>
+        <v>181.81</v>
       </c>
       <c r="W3" t="n">
-        <v>34.79</v>
+        <v>177.86</v>
       </c>
       <c r="X3" t="n">
-        <v>16.17</v>
+        <v>143.98</v>
       </c>
       <c r="Y3" t="n">
-        <v>3.24</v>
+        <v>107.15</v>
       </c>
       <c r="Z3" t="n">
-        <v>30.38</v>
+        <v>118.5</v>
       </c>
       <c r="AA3" t="n">
-        <v>37.22</v>
+        <v>-30.67</v>
       </c>
       <c r="AB3" t="n">
-        <v>40.5</v>
+        <v>196.33</v>
       </c>
       <c r="AC3" t="n">
-        <v>-7.5</v>
+        <v>83.53</v>
       </c>
       <c r="AD3" t="n">
-        <v>44.72</v>
+        <v>-53.53</v>
       </c>
       <c r="AE3" t="n">
-        <v>6.34</v>
+        <v>113.48</v>
       </c>
       <c r="AF3" t="n">
-        <v>-9.82</v>
+        <v>133.06</v>
       </c>
       <c r="AG3" t="n">
-        <v>40.79</v>
+        <v>131.38</v>
       </c>
       <c r="AH3" t="n">
-        <v>32.81</v>
-      </c>
-      <c r="AI3" t="n">
-        <v>18.9</v>
-      </c>
-      <c r="AJ3" t="n">
-        <v>29.11</v>
+        <v>114.1</v>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>166.08</t>
+        </is>
       </c>
       <c r="AK3" t="n">
-        <v>24.29</v>
+        <v>97.29000000000001</v>
       </c>
       <c r="AL3" t="n">
-        <v>30.28</v>
+        <v>-28.15</v>
       </c>
       <c r="AM3" t="n">
-        <v>26.68</v>
+        <v>161.13</v>
       </c>
       <c r="AN3" t="n">
-        <v>34.53</v>
+        <v>88.79000000000001</v>
       </c>
       <c r="AO3" t="n">
-        <v>29.27</v>
+        <v>141.8</v>
       </c>
       <c r="AP3" t="n">
-        <v>46.6</v>
+        <v>39.52</v>
       </c>
       <c r="AQ3" t="n">
-        <v>45.59</v>
+        <v>70.34999999999999</v>
       </c>
       <c r="AR3" t="n">
-        <v>19.16</v>
+        <v>150.3</v>
       </c>
       <c r="AS3" t="n">
-        <v>23.85</v>
+        <v>185.13</v>
       </c>
       <c r="AT3" t="n">
-        <v>17.76</v>
+        <v>128.8</v>
       </c>
       <c r="AU3" t="n">
-        <v>39.97</v>
+        <v>122.92</v>
+      </c>
+      <c r="AV3" t="n">
+        <v>99.05</v>
       </c>
       <c r="AW3" t="n">
-        <v>-19.7</v>
+        <v>-38</v>
       </c>
       <c r="AX3" t="n">
-        <v>29.98</v>
+        <v>89.75</v>
       </c>
       <c r="AY3" t="n">
-        <v>46.32</v>
+        <v>91.95</v>
       </c>
       <c r="AZ3" t="n">
-        <v>15.47</v>
+        <v>85.83</v>
       </c>
       <c r="BA3" t="n">
-        <v>6.39</v>
+        <v>149.94</v>
+      </c>
+      <c r="BB3" t="n">
+        <v>110.72</v>
       </c>
       <c r="BC3" t="n">
-        <v>10.09</v>
-      </c>
-      <c r="BD3" t="n">
-        <v>35.61</v>
+        <v>77.54000000000001</v>
+      </c>
+      <c r="BE3" t="n">
+        <v>154.16</v>
       </c>
       <c r="BF3" t="n">
-        <v>28.19</v>
+        <v>-29.84</v>
       </c>
       <c r="BG3" t="n">
-        <v>28.88</v>
+        <v>83.7</v>
       </c>
       <c r="BH3" t="n">
-        <v>23.31</v>
+        <v>107.23</v>
       </c>
       <c r="BI3" t="n">
-        <v>32.98</v>
+        <v>152.17</v>
       </c>
       <c r="BJ3" t="n">
-        <v>-7.94</v>
+        <v>78.88</v>
       </c>
       <c r="BK3" t="n">
-        <v>24.94</v>
+        <v>-11.42</v>
       </c>
       <c r="BL3" t="n">
-        <v>24.05</v>
+        <v>65.39</v>
+      </c>
+      <c r="BM3" t="n">
+        <v>89.22</v>
+      </c>
+      <c r="BN3" t="n">
+        <v>126.74</v>
       </c>
       <c r="BO3" t="n">
-        <v>41.3</v>
+        <v>133.57</v>
       </c>
       <c r="BP3" t="n">
-        <v>22.76</v>
+        <v>-36.81</v>
       </c>
       <c r="BQ3" t="n">
-        <v>22.19</v>
+        <v>145.56</v>
       </c>
       <c r="BR3" t="n">
-        <v>51.55</v>
-      </c>
-      <c r="BS3" t="n">
-        <v>30.34</v>
+        <v>99.64</v>
+      </c>
+      <c r="BS3" t="inlineStr">
+        <is>
+          <t>98.49</t>
+        </is>
       </c>
       <c r="BT3" t="n">
-        <v>35.27</v>
-      </c>
-      <c r="BU3" t="n">
-        <v>44.14</v>
+        <v>120.78</v>
+      </c>
+      <c r="BU3" t="inlineStr">
+        <is>
+          <t>98.81</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -1317,154 +1359,175 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>195.37</v>
+        <v>13.26</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>39.38</v>
       </c>
       <c r="R4" t="n">
-        <v>70.43000000000001</v>
+        <v>30.98</v>
       </c>
       <c r="S4" t="n">
-        <v>199.75</v>
+        <v>19.95</v>
       </c>
       <c r="T4" t="n">
-        <v>121.83</v>
+        <v>33.95</v>
       </c>
       <c r="U4" t="n">
-        <v>98.17</v>
+        <v>50.44</v>
       </c>
       <c r="V4" t="n">
-        <v>83.31999999999999</v>
+        <v>32.25</v>
       </c>
       <c r="W4" t="n">
-        <v>-37.77</v>
-      </c>
-      <c r="X4" t="n">
-        <v>78.53</v>
+        <v>43.9</v>
       </c>
       <c r="Y4" t="n">
-        <v>189.58</v>
+        <v>21.88</v>
       </c>
       <c r="Z4" t="n">
-        <v>167.78</v>
+        <v>30.43</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>-10.44</v>
       </c>
       <c r="AB4" t="n">
-        <v>111.25</v>
+        <v>22.19</v>
       </c>
       <c r="AC4" t="n">
-        <v>115.36</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>136.83</v>
+        <v>33.43</v>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>18.85</t>
+        </is>
       </c>
       <c r="AE4" t="n">
-        <v>76.89</v>
-      </c>
-      <c r="AF4" t="n">
-        <v>114.36</v>
+        <v>28.49</v>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>22.84</t>
+        </is>
+      </c>
+      <c r="AG4" t="n">
+        <v>31.12</v>
       </c>
       <c r="AH4" t="n">
-        <v>53.73</v>
+        <v>-9.77</v>
       </c>
       <c r="AI4" t="n">
-        <v>101.61</v>
-      </c>
-      <c r="AK4" t="n">
-        <v>100.06</v>
+        <v>24.4</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>51.32</v>
       </c>
       <c r="AL4" t="n">
-        <v>148.46</v>
+        <v>44.59</v>
       </c>
       <c r="AM4" t="n">
-        <v>82.33</v>
+        <v>33.65</v>
       </c>
       <c r="AN4" t="n">
-        <v>139.93</v>
+        <v>40.38</v>
       </c>
       <c r="AO4" t="n">
-        <v>78.19</v>
+        <v>34.52</v>
       </c>
       <c r="AP4" t="n">
-        <v>37.73</v>
-      </c>
-      <c r="AR4" t="n">
-        <v>68.37</v>
+        <v>41.61</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>47.66</v>
       </c>
       <c r="AS4" t="n">
-        <v>140.32</v>
-      </c>
-      <c r="AT4" t="n">
-        <v>30.21</v>
+        <v>20.57</v>
       </c>
       <c r="AU4" t="n">
-        <v>132.07</v>
+        <v>7.02</v>
       </c>
       <c r="AV4" t="n">
-        <v>92.38</v>
+        <v>43.06</v>
       </c>
       <c r="AW4" t="n">
-        <v>89.76000000000001</v>
+        <v>20.77</v>
       </c>
       <c r="AX4" t="n">
-        <v>120.13</v>
-      </c>
-      <c r="AY4" t="n">
-        <v>125.93</v>
+        <v>22.9</v>
+      </c>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AZ4" t="n">
+        <v>33.25</v>
       </c>
       <c r="BA4" t="n">
-        <v>98.76000000000001</v>
+        <v>16.04</v>
       </c>
       <c r="BB4" t="n">
-        <v>97.62</v>
+        <v>41.22</v>
       </c>
       <c r="BC4" t="n">
-        <v>185.66</v>
+        <v>32.55</v>
+      </c>
+      <c r="BD4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="BE4" t="n">
-        <v>119.65</v>
+        <v>24.41</v>
       </c>
       <c r="BF4" t="n">
-        <v>104.17</v>
+        <v>31.6</v>
       </c>
       <c r="BG4" t="n">
-        <v>115.78</v>
+        <v>35.62</v>
       </c>
       <c r="BH4" t="n">
-        <v>56.9</v>
-      </c>
-      <c r="BI4" t="n">
-        <v>11.31</v>
+        <v>-9.24</v>
+      </c>
+      <c r="BI4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="BJ4" t="n">
-        <v>107.93</v>
+        <v>24.63</v>
       </c>
       <c r="BK4" t="n">
-        <v>69.51000000000001</v>
+        <v>25.33</v>
       </c>
       <c r="BL4" t="n">
-        <v>85.87</v>
+        <v>22.8</v>
       </c>
       <c r="BM4" t="n">
-        <v>122.3</v>
+        <v>19.37</v>
       </c>
       <c r="BN4" t="n">
-        <v>-28.28</v>
+        <v>36.08</v>
       </c>
       <c r="BO4" t="n">
-        <v>93.76000000000001</v>
+        <v>39.25</v>
       </c>
       <c r="BP4" t="n">
-        <v>95.56999999999999</v>
+        <v>38.96</v>
       </c>
       <c r="BQ4" t="n">
-        <v>111.67</v>
+        <v>28.52</v>
+      </c>
+      <c r="BR4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="BS4" t="n">
-        <v>76.23</v>
-      </c>
-      <c r="BT4" t="n">
-        <v>106.01</v>
+        <v>1.78</v>
       </c>
       <c r="BU4" t="n">
-        <v>90.11</v>
+        <v>28.81</v>
       </c>
     </row>
     <row r="5">
@@ -1543,158 +1606,188 @@
           <t>PR05040100 - Savings Accounts - Other</t>
         </is>
       </c>
-      <c r="Q5" t="n">
-        <v>17.06</v>
+      <c r="P5" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>12.29</t>
+        </is>
       </c>
       <c r="R5" t="n">
-        <v>65.77</v>
+        <v>20.93</v>
       </c>
       <c r="S5" t="n">
-        <v>43.62</v>
+        <v>-8.44</v>
       </c>
       <c r="T5" t="n">
-        <v>-15.67</v>
-      </c>
-      <c r="U5" t="n">
-        <v>66.66</v>
+        <v>23.84</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="V5" t="n">
-        <v>58.49</v>
+        <v>10.03</v>
       </c>
       <c r="W5" t="n">
-        <v>-19.57</v>
+        <v>12.04</v>
       </c>
       <c r="X5" t="n">
-        <v>45.07</v>
+        <v>16.28</v>
       </c>
       <c r="Y5" t="n">
-        <v>47.17</v>
+        <v>28.47</v>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>(6.56)</t>
+        </is>
       </c>
       <c r="AA5" t="n">
-        <v>52.36</v>
+        <v>23.04</v>
       </c>
       <c r="AB5" t="n">
-        <v>63.48</v>
+        <v>16.68</v>
       </c>
       <c r="AC5" t="n">
-        <v>-14.59</v>
+        <v>9.26</v>
       </c>
       <c r="AD5" t="n">
-        <v>55.8</v>
+        <v>26.1</v>
       </c>
       <c r="AE5" t="n">
-        <v>31.28</v>
+        <v>16.61</v>
       </c>
       <c r="AF5" t="n">
-        <v>24.67</v>
+        <v>15.5</v>
       </c>
       <c r="AG5" t="n">
-        <v>58.47</v>
-      </c>
-      <c r="AH5" t="n">
-        <v>50</v>
+        <v>30.15</v>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>11.55</t>
+        </is>
       </c>
       <c r="AI5" t="n">
-        <v>39.65</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>21.08</v>
-      </c>
-      <c r="AL5" t="n">
-        <v>-17.01</v>
+        <v>19.5</v>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AK5" t="n">
+        <v>24.12</v>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>11.85</t>
+        </is>
       </c>
       <c r="AM5" t="n">
-        <v>46.95</v>
+        <v>9.77</v>
       </c>
       <c r="AN5" t="n">
-        <v>-8.16</v>
-      </c>
-      <c r="AO5" t="n">
-        <v>65.09</v>
+        <v>21.35</v>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP5" t="n">
+        <v>14.44</v>
       </c>
       <c r="AQ5" t="n">
-        <v>62.36</v>
+        <v>28.34</v>
       </c>
       <c r="AR5" t="n">
-        <v>30.07</v>
+        <v>12.37</v>
       </c>
       <c r="AS5" t="n">
-        <v>33.96</v>
+        <v>17.19</v>
       </c>
       <c r="AT5" t="n">
-        <v>55.88</v>
+        <v>14.84</v>
       </c>
       <c r="AU5" t="n">
-        <v>82.95999999999999</v>
+        <v>12.37</v>
       </c>
       <c r="AV5" t="n">
-        <v>75.47</v>
+        <v>22</v>
       </c>
       <c r="AW5" t="n">
-        <v>44.24</v>
+        <v>27.78</v>
       </c>
       <c r="AX5" t="n">
-        <v>4.71</v>
-      </c>
-      <c r="AY5" t="n">
-        <v>23.33</v>
+        <v>19.79</v>
+      </c>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AZ5" t="n">
-        <v>59.63</v>
+        <v>23.53</v>
+      </c>
+      <c r="BA5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="BB5" t="n">
-        <v>49.48</v>
+        <v>8.67</v>
       </c>
       <c r="BC5" t="n">
-        <v>-20.34</v>
+        <v>19.63</v>
       </c>
       <c r="BD5" t="n">
-        <v>53.64</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="BE5" t="n">
-        <v>59.46</v>
+        <v>29.83</v>
       </c>
       <c r="BF5" t="n">
-        <v>48.34</v>
+        <v>26.97</v>
+      </c>
+      <c r="BG5" t="n">
+        <v>16.26</v>
       </c>
       <c r="BH5" t="n">
-        <v>51.15</v>
+        <v>24.58</v>
       </c>
       <c r="BI5" t="n">
-        <v>39.78</v>
+        <v>26.35</v>
       </c>
       <c r="BJ5" t="n">
-        <v>25.85</v>
-      </c>
-      <c r="BK5" t="n">
-        <v>43.53</v>
+        <v>16.64</v>
       </c>
       <c r="BL5" t="n">
-        <v>35.12</v>
+        <v>11.1</v>
       </c>
       <c r="BM5" t="n">
-        <v>48.35</v>
-      </c>
-      <c r="BN5" t="n">
-        <v>33.46</v>
+        <v>12.98</v>
       </c>
       <c r="BO5" t="n">
-        <v>51.78</v>
+        <v>8.67</v>
       </c>
       <c r="BP5" t="n">
-        <v>56.8</v>
+        <v>11.75</v>
       </c>
       <c r="BQ5" t="n">
-        <v>21.48</v>
+        <v>22.58</v>
       </c>
       <c r="BR5" t="n">
-        <v>51.46</v>
+        <v>25.62</v>
+      </c>
+      <c r="BS5" t="n">
+        <v>18.33</v>
       </c>
       <c r="BT5" t="n">
-        <v>-15.08</v>
-      </c>
-      <c r="BU5" t="n">
-        <v>59.37</v>
+        <v>15.1</v>
       </c>
     </row>
     <row r="6">
@@ -1774,157 +1867,168 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>110.14</v>
+        <v>19.42</v>
       </c>
       <c r="Q6" t="n">
-        <v>96.91</v>
+        <v>10.99</v>
       </c>
       <c r="R6" t="n">
-        <v>73.70999999999999</v>
+        <v>13.69</v>
       </c>
       <c r="T6" t="n">
-        <v>125.48</v>
+        <v>11.69</v>
       </c>
       <c r="U6" t="n">
-        <v>104</v>
+        <v>17.07</v>
       </c>
       <c r="W6" t="n">
-        <v>126.43</v>
+        <v>10.43</v>
       </c>
       <c r="X6" t="n">
-        <v>137.6</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>116.26</v>
+        <v>10.58</v>
       </c>
       <c r="Z6" t="n">
-        <v>72.66</v>
+        <v>18.38</v>
       </c>
       <c r="AA6" t="n">
-        <v>110.71</v>
+        <v>8.93</v>
       </c>
       <c r="AB6" t="n">
-        <v>76.33</v>
+        <v>12.86</v>
       </c>
       <c r="AC6" t="n">
-        <v>78.31999999999999</v>
+        <v>21.57</v>
       </c>
       <c r="AD6" t="n">
-        <v>104.27</v>
+        <v>16.63</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>18.73</v>
       </c>
       <c r="AG6" t="n">
-        <v>96.79000000000001</v>
+        <v>14.73</v>
       </c>
       <c r="AH6" t="n">
-        <v>124.5</v>
+        <v>8.77</v>
       </c>
       <c r="AI6" t="n">
-        <v>180.79</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="AJ6" t="n">
-        <v>130.55</v>
+        <v>10.52</v>
       </c>
       <c r="AK6" t="n">
-        <v>61.28</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="AL6" t="n">
-        <v>63.32</v>
+        <v>13.95</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>15.01</v>
       </c>
       <c r="AN6" t="n">
-        <v>45.37</v>
+        <v>15.2</v>
       </c>
       <c r="AO6" t="n">
-        <v>86.38</v>
+        <v>8.26</v>
       </c>
       <c r="AP6" t="n">
-        <v>102.8</v>
+        <v>21.6</v>
       </c>
       <c r="AQ6" t="n">
-        <v>69.23999999999999</v>
+        <v>11</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>18.43</v>
       </c>
       <c r="AS6" t="n">
-        <v>116.9</v>
+        <v>13.36</v>
       </c>
       <c r="AT6" t="n">
-        <v>205</v>
+        <v>-4.63</v>
       </c>
       <c r="AU6" t="n">
-        <v>173.9</v>
-      </c>
-      <c r="AV6" t="n">
-        <v>-30.54</v>
+        <v>14.94</v>
       </c>
       <c r="AW6" t="n">
-        <v>88.37</v>
+        <v>16.09</v>
       </c>
       <c r="AX6" t="n">
-        <v>139.45</v>
-      </c>
-      <c r="AY6" t="n">
-        <v>104</v>
+        <v>10.81</v>
+      </c>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AZ6" t="n">
+        <v>16.13</v>
       </c>
       <c r="BA6" t="n">
-        <v>86.55</v>
+        <v>16.6</v>
       </c>
       <c r="BB6" t="n">
-        <v>169.89</v>
+        <v>11.1</v>
       </c>
       <c r="BC6" t="n">
-        <v>187.72</v>
+        <v>-4.18</v>
       </c>
       <c r="BD6" t="n">
-        <v>91.7</v>
+        <v>21.3</v>
       </c>
       <c r="BE6" t="n">
-        <v>158</v>
+        <v>10.16</v>
       </c>
       <c r="BF6" t="n">
-        <v>109.28</v>
+        <v>13.72</v>
       </c>
       <c r="BG6" t="n">
-        <v>94.47</v>
-      </c>
-      <c r="BH6" t="n">
-        <v>130.73</v>
+        <v>15.01</v>
       </c>
       <c r="BI6" t="n">
-        <v>131.92</v>
+        <v>12.96</v>
       </c>
       <c r="BJ6" t="n">
-        <v>166.57</v>
-      </c>
-      <c r="BK6" t="n">
-        <v>172.38</v>
+        <v>15.2</v>
+      </c>
+      <c r="BK6" t="inlineStr">
+        <is>
+          <t>11.66</t>
+        </is>
       </c>
       <c r="BL6" t="n">
-        <v>107.62</v>
-      </c>
-      <c r="BM6" t="n">
-        <v>223.49</v>
+        <v>15.11</v>
+      </c>
+      <c r="BM6" t="inlineStr">
+        <is>
+          <t>(4.77)</t>
+        </is>
       </c>
       <c r="BN6" t="n">
-        <v>187.65</v>
+        <v>18.76</v>
       </c>
       <c r="BO6" t="n">
-        <v>51.99</v>
+        <v>19.88</v>
       </c>
       <c r="BP6" t="n">
-        <v>117.71</v>
-      </c>
-      <c r="BQ6" t="n">
-        <v>119.09</v>
+        <v>15.26</v>
+      </c>
+      <c r="BQ6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="BR6" t="n">
-        <v>168.86</v>
+        <v>14.13</v>
       </c>
       <c r="BS6" t="n">
-        <v>138.68</v>
-      </c>
-      <c r="BT6" t="n">
-        <v>92.2</v>
+        <v>12.42</v>
       </c>
       <c r="BU6" t="n">
-        <v>131.37</v>
+        <v>7.28</v>
       </c>
     </row>
     <row r="7">
@@ -2003,161 +2107,174 @@
           <t>PR05040105 - Commercial Money Market</t>
         </is>
       </c>
-      <c r="P7" t="n">
-        <v>53.81</v>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="Q7" t="n">
-        <v>49.83</v>
+        <v>-5.28</v>
       </c>
       <c r="R7" t="n">
-        <v>66.89</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="S7" t="n">
-        <v>87.25</v>
+        <v>12.2</v>
       </c>
       <c r="T7" t="n">
-        <v>108.86</v>
+        <v>17.56</v>
+      </c>
+      <c r="U7" t="n">
+        <v>8</v>
       </c>
       <c r="V7" t="n">
-        <v>59.63</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="W7" t="n">
-        <v>27.97</v>
+        <v>14.86</v>
       </c>
       <c r="X7" t="n">
-        <v>65.53</v>
+        <v>21.56</v>
       </c>
       <c r="Y7" t="n">
-        <v>72.7</v>
+        <v>17.09</v>
       </c>
       <c r="Z7" t="n">
-        <v>43.65</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="AA7" t="n">
-        <v>83.86</v>
+        <v>11.86</v>
       </c>
       <c r="AB7" t="n">
-        <v>88.65000000000001</v>
+        <v>19.7</v>
       </c>
       <c r="AC7" t="n">
-        <v>96.06</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>102.11</v>
+        <v>12.19</v>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AE7" t="n">
-        <v>32.67</v>
+        <v>8.08</v>
       </c>
       <c r="AF7" t="n">
-        <v>-22.66</v>
+        <v>19.35</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>12.77</v>
       </c>
       <c r="AH7" t="n">
-        <v>21.1</v>
+        <v>12.6</v>
       </c>
       <c r="AI7" t="n">
-        <v>71.95</v>
+        <v>13.17</v>
       </c>
       <c r="AJ7" t="n">
-        <v>45.43</v>
-      </c>
-      <c r="AK7" t="n">
-        <v>-16.08</v>
+        <v>13.89</v>
       </c>
       <c r="AL7" t="n">
-        <v>21</v>
+        <v>14.52</v>
       </c>
       <c r="AM7" t="n">
-        <v>91.55</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>97.23999999999999</v>
+        <v>18.25</v>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AP7" t="n">
-        <v>58.74</v>
+        <v>8.25</v>
       </c>
       <c r="AQ7" t="n">
-        <v>59.63</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="AR7" t="n">
-        <v>72.38</v>
-      </c>
-      <c r="AS7" t="n">
-        <v>75.98</v>
+        <v>17.22</v>
+      </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>16.72</t>
+        </is>
       </c>
       <c r="AT7" t="n">
-        <v>50.68</v>
+        <v>12.98</v>
       </c>
       <c r="AU7" t="n">
-        <v>80.86</v>
-      </c>
-      <c r="AV7" t="n">
-        <v>82.03</v>
+        <v>13.11</v>
       </c>
       <c r="AW7" t="n">
-        <v>58.53</v>
+        <v>15.52</v>
       </c>
       <c r="AX7" t="n">
-        <v>1.54</v>
+        <v>17.56</v>
       </c>
       <c r="AY7" t="n">
-        <v>36.45</v>
+        <v>14.34</v>
       </c>
       <c r="AZ7" t="n">
-        <v>37.15</v>
+        <v>13.69</v>
+      </c>
+      <c r="BA7" t="n">
+        <v>14.18</v>
       </c>
       <c r="BB7" t="n">
-        <v>56.96</v>
-      </c>
-      <c r="BC7" t="n">
-        <v>62.25</v>
+        <v>14.09</v>
+      </c>
+      <c r="BC7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="BD7" t="n">
-        <v>116.77</v>
+        <v>13.71</v>
       </c>
       <c r="BE7" t="n">
-        <v>54.72</v>
+        <v>19.72</v>
       </c>
       <c r="BF7" t="n">
-        <v>36.06</v>
+        <v>11.14</v>
       </c>
       <c r="BG7" t="n">
-        <v>59.27</v>
+        <v>13.3</v>
       </c>
       <c r="BH7" t="n">
-        <v>55.15</v>
+        <v>13.68</v>
+      </c>
+      <c r="BI7" t="n">
+        <v>16.09</v>
       </c>
       <c r="BJ7" t="n">
-        <v>72.25</v>
+        <v>5.57</v>
       </c>
       <c r="BK7" t="n">
-        <v>56.73</v>
+        <v>13.74</v>
       </c>
       <c r="BL7" t="n">
-        <v>113.41</v>
+        <v>17.8</v>
       </c>
       <c r="BM7" t="n">
-        <v>47.77</v>
-      </c>
-      <c r="BN7" t="n">
-        <v>72</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="BO7" t="n">
-        <v>49.43</v>
-      </c>
-      <c r="BP7" t="n">
-        <v>98.48999999999999</v>
+        <v>-3.46</v>
       </c>
       <c r="BQ7" t="n">
-        <v>41.14</v>
+        <v>18.25</v>
       </c>
       <c r="BR7" t="n">
-        <v>73.56999999999999</v>
+        <v>7.63</v>
       </c>
       <c r="BS7" t="n">
-        <v>68.39</v>
+        <v>14.84</v>
       </c>
       <c r="BT7" t="n">
-        <v>31.83</v>
+        <v>-3.24</v>
+      </c>
+      <c r="BU7" t="n">
+        <v>13.86</v>
       </c>
     </row>
     <row r="8">
@@ -2236,140 +2353,171 @@
           <t>PR05040200 - Time Deposits Other</t>
         </is>
       </c>
+      <c r="P8" t="n">
+        <v>63.36</v>
+      </c>
       <c r="Q8" t="n">
-        <v>21.38</v>
+        <v>86.69</v>
       </c>
       <c r="R8" t="n">
-        <v>32.61</v>
-      </c>
-      <c r="S8" t="n">
-        <v>35.86</v>
-      </c>
-      <c r="T8" t="n">
-        <v>49.12</v>
+        <v>47.33</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="U8" t="n">
-        <v>52.66</v>
+        <v>88.33</v>
       </c>
       <c r="V8" t="n">
-        <v>39.97</v>
+        <v>100.32</v>
       </c>
       <c r="W8" t="n">
-        <v>41.13</v>
+        <v>38.14</v>
       </c>
       <c r="X8" t="n">
-        <v>31.58</v>
+        <v>39.94</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>81.65000000000001</v>
       </c>
       <c r="Z8" t="n">
-        <v>25.43</v>
+        <v>80.23</v>
       </c>
       <c r="AA8" t="n">
-        <v>42.4</v>
+        <v>31.24</v>
       </c>
       <c r="AB8" t="n">
-        <v>34.08</v>
+        <v>69.52</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>76.89</v>
       </c>
       <c r="AD8" t="n">
-        <v>2.28</v>
-      </c>
-      <c r="AE8" t="n">
-        <v>23.39</v>
+        <v>93.5</v>
       </c>
       <c r="AF8" t="n">
-        <v>38.99</v>
+        <v>85.5</v>
       </c>
       <c r="AG8" t="n">
-        <v>21.86</v>
+        <v>84.81999999999999</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>98.47</v>
       </c>
       <c r="AI8" t="n">
-        <v>32.12</v>
+        <v>64.89</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>86.86</v>
       </c>
       <c r="AK8" t="n">
-        <v>37.68</v>
+        <v>21.93</v>
       </c>
       <c r="AL8" t="n">
-        <v>38.7</v>
+        <v>71.13</v>
       </c>
       <c r="AM8" t="n">
-        <v>-7.38</v>
+        <v>6.45</v>
       </c>
       <c r="AN8" t="n">
-        <v>35.51</v>
+        <v>53.16</v>
       </c>
       <c r="AO8" t="n">
-        <v>36.54</v>
-      </c>
-      <c r="AR8" t="n">
-        <v>32.64</v>
-      </c>
-      <c r="AT8" t="n">
-        <v>41.73</v>
+        <v>53.36</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>59.57</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>77.25</v>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>81.93</t>
+        </is>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>69.38</t>
+        </is>
       </c>
       <c r="AU8" t="n">
-        <v>12.74</v>
+        <v>133.93</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>74.79000000000001</v>
       </c>
       <c r="AW8" t="n">
-        <v>34.77</v>
-      </c>
-      <c r="AY8" t="n">
-        <v>40.98</v>
+        <v>76.81999999999999</v>
       </c>
       <c r="AZ8" t="n">
-        <v>-6.55</v>
-      </c>
-      <c r="BA8" t="n">
-        <v>18.04</v>
-      </c>
-      <c r="BB8" t="n">
-        <v>-12.52</v>
+        <v>77.18000000000001</v>
+      </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>39.07</t>
+        </is>
+      </c>
+      <c r="BC8" t="n">
+        <v>69.66</v>
       </c>
       <c r="BD8" t="n">
-        <v>40.09</v>
+        <v>-11.87</v>
       </c>
       <c r="BE8" t="n">
-        <v>35.48</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="BF8" t="n">
-        <v>19.84</v>
+        <v>81.34999999999999</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>87.58</v>
       </c>
       <c r="BH8" t="n">
-        <v>29.55</v>
+        <v>74.14</v>
       </c>
       <c r="BI8" t="n">
-        <v>34.01</v>
+        <v>-23.93</v>
       </c>
       <c r="BJ8" t="n">
-        <v>14.19</v>
+        <v>61.02</v>
       </c>
       <c r="BK8" t="n">
-        <v>20.8</v>
+        <v>-18.35</v>
       </c>
       <c r="BL8" t="n">
-        <v>35.22</v>
+        <v>43.28</v>
       </c>
       <c r="BM8" t="n">
-        <v>-13.92</v>
+        <v>52.53</v>
       </c>
       <c r="BN8" t="n">
-        <v>52.58</v>
+        <v>33.66</v>
       </c>
       <c r="BP8" t="n">
-        <v>37.27</v>
+        <v>112.59</v>
       </c>
       <c r="BQ8" t="n">
-        <v>18.72</v>
+        <v>76.39</v>
       </c>
       <c r="BR8" t="n">
-        <v>21.88</v>
+        <v>39.09</v>
       </c>
       <c r="BS8" t="n">
-        <v>45.03</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="BT8" t="n">
-        <v>23.5</v>
+        <v>80.23</v>
       </c>
       <c r="BU8" t="n">
-        <v>25.76</v>
+        <v>49.62</v>
       </c>
     </row>
     <row r="9">
@@ -2448,158 +2596,171 @@
           <t>PR05040220 - Time Deposits 3 - 6 Months</t>
         </is>
       </c>
+      <c r="P9" t="n">
+        <v>137.75</v>
+      </c>
       <c r="Q9" t="n">
-        <v>18.48</v>
+        <v>119.1</v>
       </c>
       <c r="R9" t="n">
-        <v>44.3</v>
-      </c>
-      <c r="S9" t="n">
-        <v>36.98</v>
+        <v>68.5</v>
+      </c>
+      <c r="T9" t="n">
+        <v>75.59999999999999</v>
       </c>
       <c r="U9" t="n">
-        <v>17.28</v>
+        <v>-53.74</v>
       </c>
       <c r="V9" t="n">
-        <v>37.89</v>
-      </c>
-      <c r="W9" t="n">
-        <v>-13.8</v>
-      </c>
-      <c r="X9" t="n">
-        <v>20.82</v>
+        <v>86.79000000000001</v>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>126.14</t>
+        </is>
       </c>
       <c r="Y9" t="n">
-        <v>-7.91</v>
+        <v>133.47</v>
       </c>
       <c r="Z9" t="n">
-        <v>33.23</v>
+        <v>56.65</v>
       </c>
       <c r="AA9" t="n">
-        <v>41.76</v>
+        <v>65.69</v>
       </c>
       <c r="AB9" t="n">
-        <v>-7.99</v>
+        <v>81.93000000000001</v>
       </c>
       <c r="AC9" t="n">
-        <v>28.92</v>
+        <v>76.33</v>
       </c>
       <c r="AD9" t="n">
-        <v>28.59</v>
+        <v>94.73999999999999</v>
       </c>
       <c r="AE9" t="n">
-        <v>46.51</v>
+        <v>134.02</v>
       </c>
       <c r="AF9" t="n">
-        <v>39.41</v>
+        <v>27.66</v>
       </c>
       <c r="AG9" t="n">
-        <v>38.28</v>
+        <v>118.72</v>
       </c>
       <c r="AH9" t="n">
-        <v>41.16</v>
+        <v>136.14</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>113.99</v>
       </c>
       <c r="AJ9" t="n">
-        <v>33.83</v>
+        <v>79.86</v>
       </c>
       <c r="AK9" t="n">
-        <v>-9.130000000000001</v>
+        <v>-28.85</v>
       </c>
       <c r="AL9" t="n">
-        <v>40.39</v>
+        <v>111.38</v>
       </c>
       <c r="AM9" t="n">
-        <v>27.15</v>
+        <v>56.5</v>
       </c>
       <c r="AN9" t="n">
-        <v>-5.59</v>
+        <v>-31.42</v>
       </c>
       <c r="AO9" t="n">
-        <v>32.81</v>
+        <v>34.29</v>
       </c>
       <c r="AP9" t="n">
-        <v>31.34</v>
+        <v>139.75</v>
       </c>
       <c r="AQ9" t="n">
-        <v>27.97</v>
+        <v>56.07</v>
       </c>
       <c r="AS9" t="n">
-        <v>19.94</v>
+        <v>108.8</v>
       </c>
       <c r="AT9" t="n">
-        <v>42.72</v>
+        <v>113.85</v>
       </c>
       <c r="AU9" t="n">
-        <v>9.73</v>
+        <v>96.95</v>
       </c>
       <c r="AV9" t="n">
-        <v>20.09</v>
+        <v>145.4</v>
       </c>
       <c r="AW9" t="n">
-        <v>29.17</v>
+        <v>115.5</v>
       </c>
       <c r="AX9" t="n">
-        <v>25.5</v>
+        <v>90.06999999999999</v>
       </c>
       <c r="AY9" t="n">
-        <v>30.44</v>
+        <v>107.34</v>
       </c>
       <c r="AZ9" t="n">
-        <v>39.1</v>
+        <v>98.97</v>
       </c>
       <c r="BA9" t="n">
-        <v>12.82</v>
+        <v>49.38</v>
       </c>
       <c r="BB9" t="n">
-        <v>31.8</v>
+        <v>97.72</v>
       </c>
       <c r="BC9" t="n">
-        <v>15.09</v>
+        <v>107.85</v>
       </c>
       <c r="BD9" t="n">
-        <v>31.52</v>
+        <v>102.42</v>
       </c>
       <c r="BE9" t="n">
-        <v>19.05</v>
+        <v>90.44</v>
       </c>
       <c r="BF9" t="n">
-        <v>40.75</v>
+        <v>29.96</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>94.31999999999999</v>
       </c>
       <c r="BH9" t="n">
-        <v>19.39</v>
+        <v>122.64</v>
       </c>
       <c r="BI9" t="n">
-        <v>42.82</v>
+        <v>113.4</v>
       </c>
       <c r="BJ9" t="n">
-        <v>-10.57</v>
+        <v>122.67</v>
       </c>
       <c r="BK9" t="n">
-        <v>49.87</v>
+        <v>94.48</v>
       </c>
       <c r="BL9" t="n">
-        <v>40.77</v>
-      </c>
-      <c r="BM9" t="n">
-        <v>12.8</v>
+        <v>104</v>
       </c>
       <c r="BN9" t="n">
-        <v>24.4</v>
+        <v>133.75</v>
       </c>
       <c r="BO9" t="n">
-        <v>25.47</v>
+        <v>63.75</v>
+      </c>
+      <c r="BP9" t="n">
+        <v>99.95</v>
+      </c>
+      <c r="BQ9" t="n">
+        <v>64.8</v>
       </c>
       <c r="BR9" t="n">
-        <v>41.82</v>
-      </c>
-      <c r="BS9" t="n">
-        <v>24.16</v>
+        <v>99.62</v>
+      </c>
+      <c r="BS9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="BT9" t="n">
-        <v>30.6</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="BU9" t="n">
-        <v>36.43</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10">
@@ -2678,161 +2839,175 @@
           <t>PR05040240 - Time Deposits 12 - 24 Months</t>
         </is>
       </c>
-      <c r="P10" t="n">
-        <v>66.78</v>
-      </c>
       <c r="Q10" t="n">
-        <v>47.97</v>
+        <v>48.78</v>
       </c>
       <c r="R10" t="n">
-        <v>46.64</v>
+        <v>41.83</v>
       </c>
       <c r="S10" t="n">
-        <v>30.06</v>
+        <v>46.2</v>
       </c>
       <c r="T10" t="n">
-        <v>19.03</v>
+        <v>41.3</v>
       </c>
       <c r="U10" t="n">
-        <v>24.02</v>
+        <v>97.68000000000001</v>
       </c>
       <c r="V10" t="n">
-        <v>90.63</v>
+        <v>91.23999999999999</v>
       </c>
       <c r="W10" t="n">
-        <v>45.54</v>
+        <v>-17.66</v>
       </c>
       <c r="X10" t="n">
-        <v>68.48</v>
+        <v>70.28</v>
       </c>
       <c r="Y10" t="n">
-        <v>50.06</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>24.39</v>
-      </c>
-      <c r="AA10" t="n">
-        <v>44.55</v>
+        <v>25.46</v>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>69.21</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>52.11</t>
+        </is>
       </c>
       <c r="AB10" t="n">
-        <v>60.73</v>
+        <v>81.95999999999999</v>
       </c>
       <c r="AC10" t="n">
-        <v>56.74</v>
+        <v>89.79000000000001</v>
       </c>
       <c r="AE10" t="n">
-        <v>57.56</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="AF10" t="n">
-        <v>68.04000000000001</v>
+        <v>81.22</v>
       </c>
       <c r="AG10" t="n">
-        <v>55.88</v>
+        <v>39.58</v>
       </c>
       <c r="AH10" t="n">
-        <v>67.3</v>
+        <v>92.34</v>
       </c>
       <c r="AI10" t="n">
-        <v>24.74</v>
+        <v>47.92</v>
       </c>
       <c r="AJ10" t="n">
-        <v>46.02</v>
+        <v>56.94</v>
       </c>
       <c r="AK10" t="n">
-        <v>40.01</v>
+        <v>32.86</v>
       </c>
       <c r="AL10" t="n">
-        <v>36.7</v>
+        <v>103.97</v>
       </c>
       <c r="AM10" t="n">
-        <v>48.69</v>
+        <v>85.17</v>
       </c>
       <c r="AN10" t="n">
-        <v>101.66</v>
+        <v>13.04</v>
       </c>
       <c r="AO10" t="n">
-        <v>34.88</v>
+        <v>61.5</v>
       </c>
       <c r="AP10" t="n">
-        <v>84.8</v>
+        <v>87.47</v>
       </c>
       <c r="AQ10" t="n">
-        <v>44.95</v>
+        <v>48.57</v>
       </c>
       <c r="AR10" t="n">
-        <v>68.29000000000001</v>
+        <v>-16.21</v>
       </c>
       <c r="AS10" t="n">
-        <v>35.55</v>
+        <v>-27.84</v>
       </c>
       <c r="AT10" t="n">
-        <v>53.2</v>
+        <v>84.69</v>
       </c>
       <c r="AU10" t="n">
-        <v>37.53</v>
+        <v>48.06</v>
       </c>
       <c r="AV10" t="n">
-        <v>55.49</v>
+        <v>64.56999999999999</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>54.83</v>
       </c>
       <c r="AY10" t="n">
-        <v>71.64</v>
+        <v>84.51000000000001</v>
       </c>
       <c r="AZ10" t="n">
-        <v>48.93</v>
-      </c>
-      <c r="BA10" t="n">
-        <v>55.09</v>
+        <v>62.12</v>
       </c>
       <c r="BB10" t="n">
-        <v>61.72</v>
+        <v>111.3</v>
       </c>
       <c r="BC10" t="n">
-        <v>63.4</v>
+        <v>101.5</v>
       </c>
       <c r="BD10" t="n">
-        <v>-15.07</v>
+        <v>48.48</v>
       </c>
       <c r="BE10" t="n">
-        <v>52.6</v>
+        <v>65.37</v>
       </c>
       <c r="BF10" t="n">
-        <v>48.83</v>
+        <v>69.69</v>
       </c>
       <c r="BG10" t="n">
-        <v>29.94</v>
+        <v>35.1</v>
+      </c>
+      <c r="BH10" t="n">
+        <v>90.34</v>
       </c>
       <c r="BI10" t="n">
-        <v>57.49</v>
+        <v>79.38</v>
       </c>
       <c r="BJ10" t="n">
-        <v>32.65</v>
+        <v>63.79</v>
       </c>
       <c r="BL10" t="n">
-        <v>52.52</v>
-      </c>
-      <c r="BM10" t="n">
-        <v>62.13</v>
+        <v>8.23</v>
+      </c>
+      <c r="BM10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="BN10" t="n">
-        <v>48.06</v>
+        <v>41.09</v>
+      </c>
+      <c r="BO10" t="n">
+        <v>76.98</v>
       </c>
       <c r="BP10" t="n">
-        <v>45.4</v>
+        <v>50.94</v>
       </c>
       <c r="BQ10" t="n">
-        <v>34.93</v>
+        <v>52.36</v>
       </c>
       <c r="BR10" t="n">
-        <v>45.96</v>
+        <v>35.79</v>
       </c>
       <c r="BS10" t="n">
-        <v>83.93000000000001</v>
-      </c>
-      <c r="BT10" t="n">
-        <v>55.28</v>
+        <v>67.45999999999999</v>
+      </c>
+      <c r="BT10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="BU10" t="n">
-        <v>-15.15</v>
+        <v>59.98</v>
       </c>
     </row>
     <row r="11">
@@ -2912,148 +3087,163 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>46.55</v>
+        <v>58.79</v>
       </c>
       <c r="Q11" t="n">
-        <v>32.11</v>
-      </c>
-      <c r="R11" t="n">
-        <v>-22.76</v>
+        <v>56.25</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="S11" t="n">
-        <v>-14.61</v>
+        <v>66.47</v>
       </c>
       <c r="T11" t="n">
-        <v>-21.9</v>
+        <v>60.07</v>
       </c>
       <c r="U11" t="n">
-        <v>-3.22</v>
+        <v>70.18000000000001</v>
       </c>
       <c r="V11" t="n">
-        <v>60.91</v>
+        <v>61.6</v>
       </c>
       <c r="W11" t="n">
-        <v>42.05</v>
+        <v>64.56</v>
       </c>
       <c r="X11" t="n">
-        <v>100.14</v>
+        <v>91.89</v>
       </c>
       <c r="Y11" t="n">
-        <v>97.86</v>
+        <v>72.81</v>
       </c>
       <c r="Z11" t="n">
-        <v>42.75</v>
+        <v>32.46</v>
       </c>
       <c r="AA11" t="n">
-        <v>13.89</v>
+        <v>100.31</v>
       </c>
       <c r="AB11" t="n">
-        <v>68.63</v>
-      </c>
-      <c r="AD11" t="n">
-        <v>80.87</v>
+        <v>59.38</v>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>80.17</t>
+        </is>
+      </c>
+      <c r="AE11" t="n">
+        <v>54.18</v>
       </c>
       <c r="AF11" t="n">
-        <v>41.02</v>
+        <v>41.52</v>
       </c>
       <c r="AG11" t="n">
-        <v>35.33</v>
+        <v>66.16</v>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>56.48</t>
+        </is>
       </c>
       <c r="AI11" t="n">
-        <v>84.05</v>
-      </c>
-      <c r="AJ11" t="n">
-        <v>57.59</v>
+        <v>72.98999999999999</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>71.66</v>
       </c>
       <c r="AL11" t="n">
-        <v>133.38</v>
+        <v>73.29000000000001</v>
       </c>
       <c r="AM11" t="n">
-        <v>42.63</v>
+        <v>61.85</v>
       </c>
       <c r="AN11" t="n">
-        <v>14.83</v>
+        <v>58.19</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>49.49</v>
       </c>
       <c r="AQ11" t="n">
-        <v>52.23</v>
+        <v>106.12</v>
       </c>
       <c r="AR11" t="n">
-        <v>85.15000000000001</v>
+        <v>32.04</v>
       </c>
       <c r="AS11" t="n">
-        <v>39.86</v>
+        <v>72.63</v>
       </c>
       <c r="AT11" t="n">
-        <v>96.79000000000001</v>
+        <v>47.66</v>
       </c>
       <c r="AU11" t="n">
-        <v>67.81999999999999</v>
+        <v>56.29</v>
       </c>
       <c r="AV11" t="n">
-        <v>79.44</v>
+        <v>103.41</v>
       </c>
       <c r="AW11" t="n">
-        <v>66.43000000000001</v>
+        <v>68.7</v>
       </c>
       <c r="AX11" t="n">
-        <v>86.17</v>
+        <v>84.01000000000001</v>
       </c>
       <c r="AY11" t="n">
-        <v>55.67</v>
+        <v>63.86</v>
       </c>
       <c r="AZ11" t="n">
-        <v>68.45999999999999</v>
+        <v>103.35</v>
       </c>
       <c r="BA11" t="n">
-        <v>98.38</v>
-      </c>
-      <c r="BB11" t="n">
-        <v>86.61</v>
+        <v>20.37</v>
+      </c>
+      <c r="BC11" t="n">
+        <v>74.18000000000001</v>
       </c>
       <c r="BD11" t="n">
-        <v>103.73</v>
+        <v>50.4</v>
       </c>
       <c r="BE11" t="n">
-        <v>38.56</v>
+        <v>70.31999999999999</v>
       </c>
       <c r="BF11" t="n">
-        <v>55.74</v>
+        <v>46.03</v>
       </c>
       <c r="BG11" t="n">
-        <v>67.13</v>
+        <v>63.27</v>
+      </c>
+      <c r="BH11" t="n">
+        <v>96.17</v>
       </c>
       <c r="BI11" t="n">
-        <v>38.7</v>
+        <v>23.4</v>
       </c>
       <c r="BJ11" t="n">
-        <v>99.2</v>
+        <v>96.69</v>
       </c>
       <c r="BK11" t="n">
-        <v>105.59</v>
+        <v>55.5</v>
       </c>
       <c r="BL11" t="n">
-        <v>67.7</v>
+        <v>47.58</v>
+      </c>
+      <c r="BM11" t="n">
+        <v>38.12</v>
       </c>
       <c r="BN11" t="n">
-        <v>51.55</v>
+        <v>72.02</v>
       </c>
       <c r="BO11" t="n">
-        <v>47.56</v>
-      </c>
-      <c r="BP11" t="n">
-        <v>58.19</v>
-      </c>
-      <c r="BQ11" t="n">
-        <v>56.22</v>
+        <v>54.06</v>
+      </c>
+      <c r="BR11" t="n">
+        <v>101.25</v>
       </c>
       <c r="BS11" t="n">
-        <v>75.94</v>
-      </c>
-      <c r="BT11" t="n">
-        <v>79.45999999999999</v>
+        <v>56.05</v>
       </c>
       <c r="BU11" t="n">
-        <v>104.04</v>
+        <v>44.91</v>
       </c>
     </row>
     <row r="12">
@@ -3133,172 +3323,183 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>45.64</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>46.47</v>
+        <v>-24.48</v>
       </c>
       <c r="R12" t="n">
-        <v>71.29000000000001</v>
+        <v>-15.46</v>
       </c>
       <c r="S12" t="n">
-        <v>71.2</v>
-      </c>
-      <c r="T12" t="n">
-        <v>41.43</v>
+        <v>118.25</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V12" t="n">
+        <v>69.81999999999999</v>
       </c>
       <c r="W12" t="n">
-        <v>42.92</v>
+        <v>84.78</v>
       </c>
       <c r="X12" t="n">
-        <v>59.65</v>
+        <v>75.70999999999999</v>
       </c>
       <c r="Y12" t="n">
-        <v>62.28</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>61.84</v>
+        <v>59.64</v>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AA12" t="n">
-        <v>-22.47</v>
+        <v>-16.13</v>
       </c>
       <c r="AB12" t="n">
-        <v>88.19</v>
-      </c>
-      <c r="AC12" t="n">
-        <v>59.5</v>
+        <v>58.23</v>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>66.52</t>
+        </is>
       </c>
       <c r="AD12" t="n">
-        <v>63.34</v>
+        <v>53.18</v>
       </c>
       <c r="AE12" t="n">
-        <v>95.93000000000001</v>
+        <v>68.55</v>
       </c>
       <c r="AF12" t="n">
-        <v>97.27</v>
+        <v>-18.89</v>
       </c>
       <c r="AG12" t="n">
-        <v>78.19</v>
+        <v>87.94</v>
       </c>
       <c r="AH12" t="n">
-        <v>90.36</v>
+        <v>-16.14</v>
       </c>
       <c r="AI12" t="n">
-        <v>88.70999999999999</v>
+        <v>71.23999999999999</v>
       </c>
       <c r="AJ12" t="n">
-        <v>65.97</v>
+        <v>42.43</v>
       </c>
       <c r="AK12" t="n">
-        <v>45.19</v>
+        <v>-0.96</v>
       </c>
       <c r="AL12" t="n">
-        <v>-23.52</v>
+        <v>60.28</v>
       </c>
       <c r="AM12" t="n">
-        <v>6.84</v>
+        <v>-9.44</v>
       </c>
       <c r="AN12" t="n">
-        <v>-22.68</v>
+        <v>82.65000000000001</v>
       </c>
       <c r="AO12" t="n">
-        <v>107.45</v>
+        <v>31.47</v>
       </c>
       <c r="AP12" t="n">
-        <v>51.21</v>
-      </c>
-      <c r="AQ12" t="n">
-        <v>110.6</v>
+        <v>73.84999999999999</v>
+      </c>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AR12" t="n">
-        <v>48.38</v>
-      </c>
-      <c r="AS12" t="n">
-        <v>-26.95</v>
-      </c>
-      <c r="AT12" t="n">
-        <v>110.63</v>
+        <v>53.4</v>
+      </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AU12" t="n">
-        <v>119.19</v>
+        <v>31.38</v>
       </c>
       <c r="AV12" t="n">
-        <v>75.20999999999999</v>
-      </c>
-      <c r="AW12" t="n">
-        <v>43.74</v>
+        <v>69.44</v>
       </c>
       <c r="AX12" t="n">
-        <v>132.76</v>
+        <v>81.94</v>
       </c>
       <c r="AY12" t="n">
-        <v>92.26000000000001</v>
+        <v>47.34</v>
       </c>
       <c r="AZ12" t="n">
-        <v>82.2</v>
+        <v>72.2</v>
       </c>
       <c r="BA12" t="n">
-        <v>53.8</v>
+        <v>70.61</v>
       </c>
       <c r="BB12" t="n">
-        <v>75.66</v>
+        <v>-23.62</v>
       </c>
       <c r="BC12" t="n">
-        <v>70.5</v>
+        <v>52.13</v>
       </c>
       <c r="BD12" t="n">
-        <v>101.59</v>
-      </c>
-      <c r="BE12" t="n">
-        <v>88.54000000000001</v>
+        <v>61.41</v>
+      </c>
+      <c r="BE12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="BF12" t="n">
-        <v>54.05</v>
+        <v>78.64</v>
       </c>
       <c r="BG12" t="n">
-        <v>-21.48</v>
+        <v>54.55</v>
       </c>
       <c r="BH12" t="n">
-        <v>36.85</v>
+        <v>71.89</v>
       </c>
       <c r="BI12" t="n">
-        <v>83.90000000000001</v>
+        <v>58.72</v>
       </c>
       <c r="BJ12" t="n">
-        <v>42.66</v>
+        <v>52.16</v>
       </c>
       <c r="BK12" t="n">
-        <v>39.78</v>
+        <v>92.13</v>
       </c>
       <c r="BL12" t="n">
-        <v>-12.67</v>
+        <v>81.18000000000001</v>
       </c>
       <c r="BM12" t="n">
-        <v>82.15000000000001</v>
+        <v>78.48</v>
       </c>
       <c r="BN12" t="n">
-        <v>81.43000000000001</v>
+        <v>54.68</v>
       </c>
       <c r="BO12" t="n">
-        <v>87.64</v>
+        <v>38.57</v>
       </c>
       <c r="BP12" t="n">
-        <v>-5.2</v>
+        <v>50.01</v>
       </c>
       <c r="BQ12" t="n">
-        <v>84.44</v>
+        <v>-14.65</v>
       </c>
       <c r="BR12" t="n">
-        <v>101.38</v>
+        <v>40.11</v>
       </c>
       <c r="BS12" t="n">
-        <v>99.31999999999999</v>
+        <v>75.28</v>
       </c>
       <c r="BT12" t="n">
-        <v>64.92</v>
+        <v>31.15</v>
       </c>
       <c r="BU12" t="n">
-        <v>64.95999999999999</v>
+        <v>53.62</v>
       </c>
     </row>
     <row r="13">
@@ -3378,154 +3579,174 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>18.34</v>
+        <v>8.52</v>
       </c>
       <c r="Q13" t="n">
-        <v>30.51</v>
+        <v>-2.07</v>
       </c>
       <c r="R13" t="n">
-        <v>42.56</v>
+        <v>5.47</v>
       </c>
       <c r="S13" t="n">
-        <v>52.36</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="T13" t="n">
-        <v>24.94</v>
+        <v>9.65</v>
       </c>
       <c r="U13" t="n">
-        <v>54.74</v>
+        <v>10.75</v>
       </c>
       <c r="V13" t="n">
-        <v>30.67</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="W13" t="n">
-        <v>30.94</v>
+        <v>13.7</v>
       </c>
       <c r="X13" t="n">
-        <v>22.86</v>
+        <v>8.09</v>
       </c>
       <c r="Y13" t="n">
-        <v>7</v>
+        <v>16.22</v>
       </c>
       <c r="Z13" t="n">
-        <v>26.84</v>
+        <v>10.18</v>
       </c>
       <c r="AA13" t="n">
-        <v>34.17</v>
+        <v>12.28</v>
       </c>
       <c r="AB13" t="n">
-        <v>-15.21</v>
+        <v>-2.31</v>
       </c>
       <c r="AC13" t="n">
-        <v>32.26</v>
-      </c>
-      <c r="AE13" t="n">
-        <v>28.09</v>
+        <v>7.19</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>11.71</v>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AF13" t="n">
-        <v>55.34</v>
+        <v>15.77</v>
       </c>
       <c r="AG13" t="n">
-        <v>23.84</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="AH13" t="n">
-        <v>17.84</v>
+        <v>17.11</v>
       </c>
       <c r="AI13" t="n">
-        <v>13.12</v>
+        <v>12.86</v>
       </c>
       <c r="AJ13" t="n">
-        <v>57.14</v>
+        <v>6.05</v>
       </c>
       <c r="AK13" t="n">
-        <v>23.35</v>
+        <v>12.32</v>
       </c>
       <c r="AL13" t="n">
-        <v>45.09</v>
+        <v>12.13</v>
       </c>
       <c r="AM13" t="n">
-        <v>33.14</v>
+        <v>12.07</v>
       </c>
       <c r="AN13" t="n">
-        <v>34.49</v>
-      </c>
-      <c r="AP13" t="n">
-        <v>32.24</v>
+        <v>14.71</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>-2.57</v>
       </c>
       <c r="AQ13" t="n">
-        <v>20.23</v>
+        <v>13.65</v>
       </c>
       <c r="AR13" t="n">
-        <v>29.69</v>
-      </c>
-      <c r="AS13" t="n">
-        <v>38.63</v>
+        <v>4.73</v>
+      </c>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>10.26</t>
+        </is>
       </c>
       <c r="AT13" t="n">
-        <v>37.87</v>
+        <v>9.35</v>
       </c>
       <c r="AU13" t="n">
-        <v>37.18</v>
+        <v>12.83</v>
       </c>
       <c r="AV13" t="n">
-        <v>18.72</v>
-      </c>
-      <c r="AW13" t="n">
-        <v>39.88</v>
+        <v>11.41</v>
+      </c>
+      <c r="AW13" t="inlineStr">
+        <is>
+          <t>11.23</t>
+        </is>
       </c>
       <c r="AX13" t="n">
-        <v>20.91</v>
+        <v>-0.15</v>
       </c>
       <c r="AY13" t="n">
-        <v>29.42</v>
+        <v>7.02</v>
       </c>
       <c r="AZ13" t="n">
-        <v>41.24</v>
+        <v>6.32</v>
       </c>
       <c r="BA13" t="n">
-        <v>-8.210000000000001</v>
+        <v>15.39</v>
       </c>
       <c r="BB13" t="n">
-        <v>51.06</v>
+        <v>6.81</v>
+      </c>
+      <c r="BC13" t="n">
+        <v>14.58</v>
       </c>
       <c r="BE13" t="n">
-        <v>21.92</v>
+        <v>9.24</v>
       </c>
       <c r="BF13" t="n">
-        <v>41.07</v>
+        <v>14.41</v>
+      </c>
+      <c r="BG13" t="n">
+        <v>9.41</v>
       </c>
       <c r="BH13" t="n">
-        <v>28.85</v>
+        <v>8.67</v>
       </c>
       <c r="BI13" t="n">
-        <v>48.83</v>
+        <v>11.88</v>
       </c>
       <c r="BJ13" t="n">
-        <v>23.82</v>
+        <v>8.1</v>
       </c>
       <c r="BK13" t="n">
-        <v>25.89</v>
+        <v>9.67</v>
       </c>
       <c r="BL13" t="n">
-        <v>35.09</v>
+        <v>13.72</v>
       </c>
       <c r="BM13" t="n">
-        <v>41.98</v>
-      </c>
-      <c r="BN13" t="n">
-        <v>32</v>
+        <v>13.22</v>
+      </c>
+      <c r="BO13" t="n">
+        <v>8.77</v>
       </c>
       <c r="BP13" t="n">
-        <v>28.84</v>
+        <v>-2.51</v>
       </c>
       <c r="BQ13" t="n">
-        <v>39.48</v>
+        <v>7.24</v>
+      </c>
+      <c r="BR13" t="n">
+        <v>11.61</v>
       </c>
       <c r="BS13" t="n">
-        <v>41.77</v>
-      </c>
-      <c r="BU13" t="n">
-        <v>37.97</v>
+        <v>7.27</v>
+      </c>
+      <c r="BU13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -3604,164 +3825,176 @@
           <t>PR05040400 - Term Deposits Liabilities - Other</t>
         </is>
       </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>141.87</t>
+        </is>
+      </c>
       <c r="Q14" t="n">
-        <v>36.89</v>
+        <v>141.42</v>
       </c>
       <c r="R14" t="n">
-        <v>28.1</v>
+        <v>83.63</v>
       </c>
       <c r="S14" t="n">
-        <v>-24.02</v>
+        <v>79.29000000000001</v>
       </c>
       <c r="T14" t="n">
-        <v>116.96</v>
-      </c>
-      <c r="V14" t="n">
-        <v>-24.81</v>
-      </c>
-      <c r="W14" t="n">
-        <v>61.61</v>
+        <v>112.08</v>
+      </c>
+      <c r="U14" t="n">
+        <v>124</v>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>111.18</t>
+        </is>
       </c>
       <c r="X14" t="n">
-        <v>23.46</v>
+        <v>112.81</v>
       </c>
       <c r="Y14" t="n">
-        <v>27.47</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>84.89</v>
+        <v>103.76</v>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AA14" t="n">
-        <v>29.1</v>
+        <v>104.57</v>
       </c>
       <c r="AB14" t="n">
-        <v>50.37</v>
+        <v>95.5</v>
       </c>
       <c r="AC14" t="n">
-        <v>-16.66</v>
+        <v>-23.2</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>87.06999999999999</v>
       </c>
       <c r="AE14" t="n">
-        <v>43.38</v>
-      </c>
-      <c r="AF14" t="n">
-        <v>20.79</v>
+        <v>49.01</v>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AG14" t="n">
-        <v>50.06</v>
+        <v>67.42</v>
       </c>
       <c r="AH14" t="n">
-        <v>55.99</v>
+        <v>77.66</v>
       </c>
       <c r="AI14" t="n">
-        <v>47.8</v>
+        <v>58.3</v>
       </c>
       <c r="AJ14" t="n">
-        <v>71.15000000000001</v>
+        <v>68.37</v>
+      </c>
+      <c r="AK14" t="inlineStr">
+        <is>
+          <t>39.97</t>
+        </is>
       </c>
       <c r="AL14" t="n">
-        <v>58.87</v>
+        <v>91.84</v>
+      </c>
+      <c r="AM14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AN14" t="n">
-        <v>45.51</v>
+        <v>61.23</v>
       </c>
       <c r="AO14" t="n">
-        <v>-19.8</v>
+        <v>72.43000000000001</v>
       </c>
       <c r="AP14" t="n">
-        <v>48.49</v>
+        <v>61.67</v>
       </c>
       <c r="AQ14" t="n">
-        <v>93.45</v>
+        <v>-39.88</v>
       </c>
       <c r="AR14" t="n">
-        <v>50.2</v>
+        <v>106.54</v>
       </c>
       <c r="AS14" t="n">
-        <v>72.94</v>
+        <v>98.06</v>
       </c>
       <c r="AT14" t="n">
-        <v>103.03</v>
+        <v>131.03</v>
       </c>
       <c r="AU14" t="n">
-        <v>75.86</v>
+        <v>115.59</v>
       </c>
       <c r="AV14" t="n">
-        <v>3.63</v>
+        <v>62.86</v>
       </c>
       <c r="AW14" t="n">
-        <v>59.02</v>
+        <v>-26.29</v>
       </c>
       <c r="AX14" t="n">
-        <v>47.63</v>
+        <v>101.7</v>
       </c>
       <c r="AY14" t="n">
-        <v>63.28</v>
+        <v>85.69</v>
       </c>
       <c r="AZ14" t="n">
-        <v>47.64</v>
+        <v>94.16</v>
       </c>
       <c r="BA14" t="n">
-        <v>87.52</v>
+        <v>78.38</v>
       </c>
       <c r="BB14" t="n">
-        <v>47.42</v>
+        <v>91.47</v>
       </c>
       <c r="BC14" t="n">
-        <v>53.73</v>
-      </c>
-      <c r="BD14" t="n">
-        <v>62.62</v>
+        <v>75.36</v>
       </c>
       <c r="BE14" t="n">
-        <v>50.26</v>
-      </c>
-      <c r="BF14" t="n">
-        <v>24.85</v>
+        <v>93.48</v>
       </c>
       <c r="BG14" t="n">
-        <v>32.85</v>
+        <v>107.13</v>
       </c>
       <c r="BH14" t="n">
-        <v>17.24</v>
+        <v>77.92</v>
       </c>
       <c r="BI14" t="n">
-        <v>-18.83</v>
-      </c>
-      <c r="BJ14" t="n">
-        <v>67.31</v>
+        <v>114.03</v>
       </c>
       <c r="BK14" t="n">
-        <v>55.16</v>
+        <v>96.44</v>
       </c>
       <c r="BL14" t="n">
-        <v>70.14</v>
+        <v>132.75</v>
       </c>
       <c r="BM14" t="n">
-        <v>100.44</v>
+        <v>93.11</v>
       </c>
       <c r="BN14" t="n">
-        <v>47.59</v>
+        <v>60.48</v>
       </c>
       <c r="BO14" t="n">
-        <v>69.66</v>
+        <v>23.39</v>
       </c>
       <c r="BP14" t="n">
-        <v>19.71</v>
+        <v>94.23</v>
       </c>
       <c r="BQ14" t="n">
-        <v>64.87</v>
-      </c>
-      <c r="BR14" t="n">
-        <v>59.56</v>
+        <v>82.19</v>
       </c>
       <c r="BS14" t="n">
-        <v>68.66</v>
+        <v>158.11</v>
       </c>
       <c r="BT14" t="n">
-        <v>67.90000000000001</v>
+        <v>51.71</v>
       </c>
       <c r="BU14" t="n">
-        <v>72.27</v>
+        <v>105.16</v>
       </c>
     </row>
     <row r="15">
@@ -3840,146 +4073,173 @@
           <t>PR05070001 - Other Deposits Interest Bearing</t>
         </is>
       </c>
-      <c r="P15" t="n">
-        <v>77.88</v>
-      </c>
       <c r="Q15" t="n">
-        <v>132.39</v>
+        <v>34.33</v>
       </c>
       <c r="R15" t="n">
-        <v>85.05</v>
+        <v>-13.15</v>
       </c>
       <c r="S15" t="n">
-        <v>63.85</v>
+        <v>32.41</v>
       </c>
       <c r="T15" t="n">
-        <v>-22.24</v>
+        <v>-8.34</v>
       </c>
       <c r="U15" t="n">
-        <v>72.68000000000001</v>
+        <v>55.03</v>
       </c>
       <c r="V15" t="n">
-        <v>82.89</v>
-      </c>
-      <c r="W15" t="n">
-        <v>51.42</v>
+        <v>47.64</v>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="Y15" t="n">
-        <v>53.04</v>
+        <v>35.14</v>
       </c>
       <c r="Z15" t="n">
-        <v>108.15</v>
+        <v>29.04</v>
       </c>
       <c r="AA15" t="n">
-        <v>-34.75</v>
+        <v>38.85</v>
       </c>
       <c r="AB15" t="n">
-        <v>81.76000000000001</v>
+        <v>-4.82</v>
       </c>
       <c r="AC15" t="n">
-        <v>131.45</v>
+        <v>27.37</v>
       </c>
       <c r="AD15" t="n">
-        <v>85.81</v>
-      </c>
-      <c r="AG15" t="n">
-        <v>92.54000000000001</v>
+        <v>29.76</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>29.92</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>41.7</v>
       </c>
       <c r="AH15" t="n">
-        <v>112.37</v>
+        <v>30.8</v>
       </c>
       <c r="AI15" t="n">
-        <v>50.16</v>
+        <v>37.68</v>
       </c>
       <c r="AJ15" t="n">
-        <v>100.46</v>
+        <v>44.79</v>
       </c>
       <c r="AK15" t="n">
-        <v>48.7</v>
+        <v>35.48</v>
+      </c>
+      <c r="AL15" t="n">
+        <v>55.01</v>
       </c>
       <c r="AM15" t="n">
-        <v>34.59</v>
+        <v>34.83</v>
+      </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>25.38</t>
+        </is>
       </c>
       <c r="AP15" t="n">
-        <v>50.31</v>
+        <v>28.74</v>
       </c>
       <c r="AQ15" t="n">
-        <v>80.31</v>
+        <v>-11.45</v>
+      </c>
+      <c r="AR15" t="n">
+        <v>24.03</v>
       </c>
       <c r="AS15" t="n">
-        <v>98.95999999999999</v>
+        <v>50.5</v>
       </c>
       <c r="AT15" t="n">
-        <v>85.40000000000001</v>
-      </c>
-      <c r="AW15" t="n">
-        <v>-32.84</v>
+        <v>36.43</v>
+      </c>
+      <c r="AV15" t="n">
+        <v>33.45</v>
       </c>
       <c r="AX15" t="n">
-        <v>58.89</v>
+        <v>42.9</v>
       </c>
       <c r="AY15" t="n">
-        <v>40.19</v>
+        <v>17.01</v>
       </c>
       <c r="AZ15" t="n">
-        <v>-16.76</v>
+        <v>30.54</v>
       </c>
       <c r="BA15" t="n">
-        <v>83.47</v>
+        <v>7.66</v>
       </c>
       <c r="BB15" t="n">
-        <v>133.49</v>
+        <v>35.66</v>
       </c>
       <c r="BC15" t="n">
-        <v>133.81</v>
+        <v>33.91</v>
       </c>
       <c r="BD15" t="n">
-        <v>144.95</v>
-      </c>
-      <c r="BF15" t="n">
-        <v>93.84</v>
+        <v>29.22</v>
+      </c>
+      <c r="BE15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BF15" t="inlineStr">
+        <is>
+          <t>30.97</t>
+        </is>
       </c>
       <c r="BG15" t="n">
-        <v>58.52</v>
+        <v>54.46</v>
       </c>
       <c r="BH15" t="n">
-        <v>102.35</v>
+        <v>19.6</v>
       </c>
       <c r="BI15" t="n">
-        <v>84.44</v>
+        <v>50.76</v>
       </c>
       <c r="BJ15" t="n">
-        <v>41.71</v>
+        <v>50.95</v>
+      </c>
+      <c r="BK15" t="n">
+        <v>36.37</v>
       </c>
       <c r="BL15" t="n">
-        <v>97.89</v>
+        <v>23.21</v>
       </c>
       <c r="BM15" t="n">
-        <v>94.43000000000001</v>
-      </c>
-      <c r="BN15" t="n">
-        <v>88.3</v>
+        <v>33.68</v>
       </c>
       <c r="BO15" t="n">
-        <v>82.53</v>
-      </c>
-      <c r="BP15" t="n">
-        <v>82.06</v>
+        <v>35.03</v>
+      </c>
+      <c r="BP15" t="inlineStr">
+        <is>
+          <t>39.05</t>
+        </is>
       </c>
       <c r="BQ15" t="n">
-        <v>92.04000000000001</v>
+        <v>50.58</v>
       </c>
       <c r="BR15" t="n">
-        <v>-32.58</v>
+        <v>23.23</v>
       </c>
       <c r="BS15" t="n">
-        <v>111.91</v>
+        <v>41.12</v>
       </c>
       <c r="BT15" t="n">
-        <v>101.22</v>
+        <v>39.03</v>
       </c>
       <c r="BU15" t="n">
-        <v>132.37</v>
+        <v>47.21</v>
       </c>
     </row>
     <row r="16">
@@ -4059,148 +4319,172 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>162.38</v>
+        <v>173.71</v>
       </c>
       <c r="Q16" t="n">
-        <v>139.87</v>
+        <v>88.93000000000001</v>
+      </c>
+      <c r="R16" t="n">
+        <v>79.34</v>
       </c>
       <c r="S16" t="n">
-        <v>144.15</v>
+        <v>139.97</v>
       </c>
       <c r="T16" t="n">
-        <v>145.22</v>
+        <v>104.68</v>
       </c>
       <c r="U16" t="n">
-        <v>132.04</v>
+        <v>94.78</v>
       </c>
       <c r="V16" t="n">
-        <v>144.92</v>
+        <v>70.87</v>
       </c>
       <c r="W16" t="n">
-        <v>139.32</v>
-      </c>
-      <c r="X16" t="n">
-        <v>99.7</v>
-      </c>
-      <c r="Y16" t="n">
-        <v>150.08</v>
+        <v>123.03</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>71.74</t>
+        </is>
       </c>
       <c r="Z16" t="n">
-        <v>74.64</v>
+        <v>85.88</v>
       </c>
       <c r="AA16" t="n">
-        <v>207.58</v>
+        <v>7.88</v>
       </c>
       <c r="AB16" t="n">
-        <v>101.17</v>
-      </c>
-      <c r="AC16" t="n">
-        <v>178.72</v>
+        <v>127.36</v>
       </c>
       <c r="AD16" t="n">
-        <v>134.16</v>
+        <v>58.93</v>
       </c>
       <c r="AE16" t="n">
-        <v>79.94</v>
+        <v>113.74</v>
       </c>
       <c r="AF16" t="n">
-        <v>95.87</v>
+        <v>104.68</v>
       </c>
       <c r="AG16" t="n">
-        <v>70.23</v>
+        <v>-19.95</v>
       </c>
       <c r="AH16" t="n">
-        <v>101.27</v>
-      </c>
-      <c r="AI16" t="n">
-        <v>178.55</v>
+        <v>70.37</v>
+      </c>
+      <c r="AI16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AJ16" t="n">
-        <v>97.01000000000001</v>
+        <v>114.53</v>
       </c>
       <c r="AK16" t="n">
-        <v>94.73999999999999</v>
+        <v>143.54</v>
       </c>
       <c r="AM16" t="n">
-        <v>76.22</v>
+        <v>105.83</v>
       </c>
       <c r="AN16" t="n">
-        <v>122.9</v>
+        <v>79.2</v>
       </c>
       <c r="AO16" t="n">
-        <v>127.31</v>
+        <v>115.7</v>
       </c>
       <c r="AP16" t="n">
-        <v>79.94</v>
+        <v>98.8</v>
+      </c>
+      <c r="AQ16" t="n">
+        <v>87.75</v>
       </c>
       <c r="AR16" t="n">
-        <v>96.37</v>
+        <v>83.11</v>
+      </c>
+      <c r="AS16" t="n">
+        <v>72.14</v>
       </c>
       <c r="AT16" t="n">
-        <v>85.29000000000001</v>
+        <v>100.72</v>
       </c>
       <c r="AU16" t="n">
-        <v>119.29</v>
+        <v>9.68</v>
+      </c>
+      <c r="AV16" t="n">
+        <v>72.63</v>
       </c>
       <c r="AW16" t="n">
-        <v>10.7</v>
-      </c>
-      <c r="AX16" t="n">
-        <v>70.42</v>
+        <v>120.93</v>
       </c>
       <c r="AY16" t="n">
-        <v>91.41</v>
+        <v>67.34999999999999</v>
       </c>
       <c r="AZ16" t="n">
-        <v>-23.9</v>
+        <v>111.18</v>
+      </c>
+      <c r="BA16" t="n">
+        <v>47.72</v>
       </c>
       <c r="BB16" t="n">
-        <v>117.38</v>
+        <v>101.74</v>
+      </c>
+      <c r="BC16" t="n">
+        <v>79.3</v>
       </c>
       <c r="BD16" t="n">
-        <v>139.86</v>
+        <v>91.86</v>
       </c>
       <c r="BE16" t="n">
-        <v>145.12</v>
+        <v>168.91</v>
       </c>
       <c r="BF16" t="n">
-        <v>58.7</v>
+        <v>29.87</v>
       </c>
       <c r="BG16" t="n">
-        <v>141.55</v>
+        <v>113.17</v>
+      </c>
+      <c r="BH16" t="n">
+        <v>47.55</v>
       </c>
       <c r="BI16" t="n">
-        <v>80.51000000000001</v>
+        <v>65.94</v>
       </c>
       <c r="BJ16" t="n">
-        <v>67.93000000000001</v>
+        <v>76.38</v>
       </c>
       <c r="BK16" t="n">
-        <v>145.68</v>
+        <v>-37.22</v>
       </c>
       <c r="BL16" t="n">
-        <v>161.99</v>
+        <v>-16.68</v>
       </c>
       <c r="BM16" t="n">
-        <v>-26.91</v>
+        <v>63.07</v>
       </c>
       <c r="BN16" t="n">
-        <v>83.7</v>
+        <v>100.9</v>
       </c>
       <c r="BO16" t="n">
-        <v>68.3</v>
-      </c>
-      <c r="BP16" t="n">
-        <v>158.79</v>
+        <v>91.43000000000001</v>
+      </c>
+      <c r="BP16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BQ16" t="n">
+        <v>155.56</v>
+      </c>
+      <c r="BR16" t="n">
+        <v>163.09</v>
       </c>
       <c r="BS16" t="n">
-        <v>131.58</v>
+        <v>110.47</v>
       </c>
       <c r="BT16" t="n">
-        <v>151.19</v>
+        <v>155.98</v>
       </c>
       <c r="BU16" t="n">
-        <v>81.91</v>
+        <v>80.61</v>
       </c>
     </row>
     <row r="17">
@@ -4279,152 +4563,178 @@
           <t>PR05070003 - Global Money</t>
         </is>
       </c>
-      <c r="P17" t="n">
-        <v>46.27</v>
-      </c>
       <c r="Q17" t="n">
-        <v>87.98999999999999</v>
+        <v>147.07</v>
       </c>
       <c r="R17" t="n">
-        <v>35.94</v>
+        <v>26.14</v>
       </c>
       <c r="S17" t="n">
-        <v>88.5</v>
+        <v>128.57</v>
       </c>
       <c r="T17" t="n">
-        <v>87.12</v>
+        <v>141.32</v>
       </c>
       <c r="U17" t="n">
-        <v>88.68000000000001</v>
+        <v>112.97</v>
       </c>
       <c r="V17" t="n">
-        <v>91.53</v>
+        <v>154.8</v>
       </c>
       <c r="W17" t="n">
-        <v>104.79</v>
+        <v>68.12</v>
       </c>
       <c r="X17" t="n">
-        <v>72.48999999999999</v>
+        <v>139.55</v>
       </c>
       <c r="Y17" t="n">
-        <v>-28.53</v>
+        <v>-19.26</v>
       </c>
       <c r="Z17" t="n">
-        <v>80.42</v>
-      </c>
-      <c r="AA17" t="n">
-        <v>42.86</v>
+        <v>187.79</v>
       </c>
       <c r="AB17" t="n">
-        <v>71.48999999999999</v>
+        <v>110.69</v>
       </c>
       <c r="AC17" t="n">
-        <v>78.02</v>
+        <v>81.78</v>
       </c>
       <c r="AD17" t="n">
-        <v>75.66</v>
+        <v>75.65000000000001</v>
       </c>
       <c r="AE17" t="n">
-        <v>86.3</v>
+        <v>92.34999999999999</v>
       </c>
       <c r="AF17" t="n">
-        <v>96.94</v>
+        <v>116.51</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>-30.24</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>123.07</v>
       </c>
       <c r="AI17" t="n">
-        <v>83.29000000000001</v>
+        <v>130.53</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>86.54000000000001</v>
       </c>
       <c r="AK17" t="n">
-        <v>50.77</v>
+        <v>76.20999999999999</v>
       </c>
       <c r="AL17" t="n">
-        <v>110.73</v>
+        <v>58.63</v>
       </c>
       <c r="AM17" t="n">
-        <v>101.17</v>
+        <v>162.98</v>
       </c>
       <c r="AN17" t="n">
-        <v>45.37</v>
+        <v>118.95</v>
       </c>
       <c r="AO17" t="n">
-        <v>110.57</v>
+        <v>152.28</v>
       </c>
       <c r="AP17" t="n">
-        <v>85.08</v>
-      </c>
-      <c r="AQ17" t="n">
-        <v>41.14</v>
+        <v>75.40000000000001</v>
+      </c>
+      <c r="AQ17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AR17" t="n">
-        <v>83.56999999999999</v>
+        <v>102.45</v>
+      </c>
+      <c r="AS17" t="n">
+        <v>173.54</v>
       </c>
       <c r="AT17" t="n">
-        <v>85.76000000000001</v>
+        <v>104.97</v>
       </c>
       <c r="AU17" t="n">
-        <v>54.83</v>
+        <v>74.33</v>
       </c>
       <c r="AV17" t="n">
-        <v>107.94</v>
+        <v>138.96</v>
       </c>
       <c r="AW17" t="n">
-        <v>67.63</v>
+        <v>69.53</v>
       </c>
       <c r="AX17" t="n">
-        <v>62.25</v>
+        <v>102.42</v>
       </c>
       <c r="AY17" t="n">
-        <v>81.37</v>
+        <v>117.94</v>
       </c>
       <c r="AZ17" t="n">
-        <v>62.7</v>
+        <v>74.87</v>
       </c>
       <c r="BA17" t="n">
-        <v>75.25</v>
+        <v>114.66</v>
       </c>
       <c r="BB17" t="n">
-        <v>34.49</v>
+        <v>135.8</v>
       </c>
       <c r="BC17" t="n">
-        <v>38.17</v>
+        <v>107</v>
+      </c>
+      <c r="BD17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="BE17" t="n">
-        <v>83.19</v>
-      </c>
-      <c r="BF17" t="n">
-        <v>30.21</v>
+        <v>80.89</v>
+      </c>
+      <c r="BG17" t="inlineStr">
+        <is>
+          <t>78.04</t>
+        </is>
       </c>
       <c r="BH17" t="n">
-        <v>118.07</v>
+        <v>118.19</v>
       </c>
       <c r="BI17" t="n">
-        <v>36.29</v>
+        <v>85.2</v>
+      </c>
+      <c r="BJ17" t="n">
+        <v>69.29000000000001</v>
       </c>
       <c r="BK17" t="n">
-        <v>82.18000000000001</v>
+        <v>139.2</v>
       </c>
       <c r="BL17" t="n">
-        <v>77.27</v>
+        <v>65.38</v>
       </c>
       <c r="BM17" t="n">
-        <v>92</v>
+        <v>172.3</v>
       </c>
       <c r="BN17" t="n">
-        <v>49.31</v>
-      </c>
-      <c r="BQ17" t="n">
-        <v>74.65000000000001</v>
+        <v>139</v>
+      </c>
+      <c r="BO17" t="n">
+        <v>87.56</v>
+      </c>
+      <c r="BP17" t="n">
+        <v>-21.03</v>
+      </c>
+      <c r="BQ17" t="inlineStr">
+        <is>
+          <t>146.17</t>
+        </is>
       </c>
       <c r="BR17" t="n">
-        <v>-26.89</v>
+        <v>-23.31</v>
       </c>
       <c r="BS17" t="n">
-        <v>51.15</v>
+        <v>60.1</v>
       </c>
       <c r="BT17" t="n">
-        <v>97.34999999999999</v>
+        <v>138.86</v>
       </c>
       <c r="BU17" t="n">
-        <v>99.61</v>
+        <v>153.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Exclude 'calculated' subtotal rows from aggregation
Rows whose dimension cells contain calculate/calculated are derived
consolidations of other rows; summing them alongside the leaves
double-counts. They are now flagged on load and excluded from the tree
and all totals by default:
- load banner + footnote report the excluded count
- sidebar checkbox re-includes them (with a double-count warning)
- sample generator emits two such rows; verified totals are unchanged
  by their presence and jump only when re-included

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018B5qKH9JxzLywUkLopxf6J
</commit_message>
<xml_diff>
--- a/tm1-dashboard/sample/GPS_Driller_sample.xlsx
+++ b/tm1-dashboard/sample/GPS_Driller_sample.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BU17"/>
+  <dimension ref="A1:BU19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4735,6 +4735,508 @@
       </c>
       <c r="BU17" t="n">
         <v>153.1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>P&amp;L-Calculate-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>P&amp;L-Calculate-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Calculated</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Calculated</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>MP10101000000 - NII - Net Interest Income</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>RTN16559</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>CG3000000</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Calculate - NII Total</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
+        <v>1408.45</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>705.75</v>
+      </c>
+      <c r="R18" t="n">
+        <v>1745.98</v>
+      </c>
+      <c r="S18" t="n">
+        <v>657.37</v>
+      </c>
+      <c r="T18" t="n">
+        <v>1578.15</v>
+      </c>
+      <c r="U18" t="n">
+        <v>676.6</v>
+      </c>
+      <c r="V18" t="n">
+        <v>671.02</v>
+      </c>
+      <c r="W18" t="n">
+        <v>659.4</v>
+      </c>
+      <c r="X18" t="n">
+        <v>797.97</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>799.62</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>894.49</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>1284.72</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>802.51</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>1555.16</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>943.03</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>559.11</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>1244.53</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>811.54</v>
+      </c>
+      <c r="AH18" t="n">
+        <v>1899.69</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>995.91</v>
+      </c>
+      <c r="AJ18" t="n">
+        <v>504.11</v>
+      </c>
+      <c r="AK18" t="n">
+        <v>1507.45</v>
+      </c>
+      <c r="AL18" t="n">
+        <v>1860.32</v>
+      </c>
+      <c r="AM18" t="n">
+        <v>1752.85</v>
+      </c>
+      <c r="AN18" t="n">
+        <v>1503.53</v>
+      </c>
+      <c r="AO18" t="n">
+        <v>723.72</v>
+      </c>
+      <c r="AP18" t="n">
+        <v>635.12</v>
+      </c>
+      <c r="AQ18" t="n">
+        <v>1267.56</v>
+      </c>
+      <c r="AR18" t="n">
+        <v>1585.35</v>
+      </c>
+      <c r="AS18" t="n">
+        <v>651.9400000000001</v>
+      </c>
+      <c r="AT18" t="n">
+        <v>883.84</v>
+      </c>
+      <c r="AU18" t="n">
+        <v>846.74</v>
+      </c>
+      <c r="AV18" t="n">
+        <v>1983</v>
+      </c>
+      <c r="AW18" t="n">
+        <v>944.03</v>
+      </c>
+      <c r="AX18" t="n">
+        <v>1196.42</v>
+      </c>
+      <c r="AY18" t="n">
+        <v>649.71</v>
+      </c>
+      <c r="AZ18" t="n">
+        <v>762.05</v>
+      </c>
+      <c r="BA18" t="n">
+        <v>559.17</v>
+      </c>
+      <c r="BB18" t="n">
+        <v>935.85</v>
+      </c>
+      <c r="BC18" t="n">
+        <v>1702.39</v>
+      </c>
+      <c r="BD18" t="n">
+        <v>969.0599999999999</v>
+      </c>
+      <c r="BE18" t="n">
+        <v>1607.81</v>
+      </c>
+      <c r="BF18" t="n">
+        <v>642.5</v>
+      </c>
+      <c r="BG18" t="n">
+        <v>1637.31</v>
+      </c>
+      <c r="BH18" t="n">
+        <v>568.83</v>
+      </c>
+      <c r="BI18" t="n">
+        <v>1778</v>
+      </c>
+      <c r="BJ18" t="n">
+        <v>1495.03</v>
+      </c>
+      <c r="BK18" t="n">
+        <v>755.77</v>
+      </c>
+      <c r="BL18" t="n">
+        <v>1036.29</v>
+      </c>
+      <c r="BM18" t="n">
+        <v>1156.57</v>
+      </c>
+      <c r="BN18" t="n">
+        <v>1432.71</v>
+      </c>
+      <c r="BO18" t="n">
+        <v>1817.71</v>
+      </c>
+      <c r="BP18" t="n">
+        <v>639.4299999999999</v>
+      </c>
+      <c r="BQ18" t="n">
+        <v>1722.45</v>
+      </c>
+      <c r="BR18" t="n">
+        <v>774.3</v>
+      </c>
+      <c r="BS18" t="n">
+        <v>1101.17</v>
+      </c>
+      <c r="BT18" t="n">
+        <v>1943.46</v>
+      </c>
+      <c r="BU18" t="n">
+        <v>907.75</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>P&amp;L-Calculate-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>P&amp;L-Calculate-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Calculated</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Calculated</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Non-NII</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Non-NII</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>MP10101000000 - NII - Net Interest Income</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>RTN16559</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>CG3000000</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Calculate - Non-NII Total</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>1078.57</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>1776.01</v>
+      </c>
+      <c r="R19" t="n">
+        <v>1699.85</v>
+      </c>
+      <c r="S19" t="n">
+        <v>1473.27</v>
+      </c>
+      <c r="T19" t="n">
+        <v>1695.36</v>
+      </c>
+      <c r="U19" t="n">
+        <v>669.58</v>
+      </c>
+      <c r="V19" t="n">
+        <v>1544.25</v>
+      </c>
+      <c r="W19" t="n">
+        <v>587.97</v>
+      </c>
+      <c r="X19" t="n">
+        <v>1913.7</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>739.09</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>1124.04</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>1386.13</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>1703.4</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>1517.59</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>771.89</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>1069.63</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>1037.9</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>543.22</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>1526.7</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>1757.8</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>1960.17</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>695.98</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>1880.6</v>
+      </c>
+      <c r="AM19" t="n">
+        <v>669.41</v>
+      </c>
+      <c r="AN19" t="n">
+        <v>1116.93</v>
+      </c>
+      <c r="AO19" t="n">
+        <v>568.96</v>
+      </c>
+      <c r="AP19" t="n">
+        <v>892.42</v>
+      </c>
+      <c r="AQ19" t="n">
+        <v>971.36</v>
+      </c>
+      <c r="AR19" t="n">
+        <v>1556.85</v>
+      </c>
+      <c r="AS19" t="n">
+        <v>1516.89</v>
+      </c>
+      <c r="AT19" t="n">
+        <v>1651.29</v>
+      </c>
+      <c r="AU19" t="n">
+        <v>1364.97</v>
+      </c>
+      <c r="AV19" t="n">
+        <v>1347.52</v>
+      </c>
+      <c r="AW19" t="n">
+        <v>1966.84</v>
+      </c>
+      <c r="AX19" t="n">
+        <v>1504.77</v>
+      </c>
+      <c r="AY19" t="n">
+        <v>1007.45</v>
+      </c>
+      <c r="AZ19" t="n">
+        <v>1284.65</v>
+      </c>
+      <c r="BA19" t="n">
+        <v>1550.87</v>
+      </c>
+      <c r="BB19" t="n">
+        <v>642.86</v>
+      </c>
+      <c r="BC19" t="n">
+        <v>1492.57</v>
+      </c>
+      <c r="BD19" t="n">
+        <v>872.87</v>
+      </c>
+      <c r="BE19" t="n">
+        <v>1018.62</v>
+      </c>
+      <c r="BF19" t="n">
+        <v>1514.44</v>
+      </c>
+      <c r="BG19" t="n">
+        <v>1077.31</v>
+      </c>
+      <c r="BH19" t="n">
+        <v>1758.55</v>
+      </c>
+      <c r="BI19" t="n">
+        <v>1337.52</v>
+      </c>
+      <c r="BJ19" t="n">
+        <v>1981.69</v>
+      </c>
+      <c r="BK19" t="n">
+        <v>581.85</v>
+      </c>
+      <c r="BL19" t="n">
+        <v>1465.1</v>
+      </c>
+      <c r="BM19" t="n">
+        <v>735.39</v>
+      </c>
+      <c r="BN19" t="n">
+        <v>1773.27</v>
+      </c>
+      <c r="BO19" t="n">
+        <v>1777.81</v>
+      </c>
+      <c r="BP19" t="n">
+        <v>1804.12</v>
+      </c>
+      <c r="BQ19" t="n">
+        <v>612.3</v>
+      </c>
+      <c r="BR19" t="n">
+        <v>1237.47</v>
+      </c>
+      <c r="BS19" t="n">
+        <v>861.34</v>
+      </c>
+      <c r="BT19" t="n">
+        <v>1955.22</v>
+      </c>
+      <c r="BU19" t="n">
+        <v>575.53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Partition dashboard into Ac Type panes: P&L, Avg Bal, RWA, metrics
Grand totals previously summed every row regardless of Ac Type, mixing
P&L flows with average balances and RWA. Now:
- rows are partitioned by the Ac Type dimension; a pane bar above the
  KPIs shows each category's own total (first selected period) and count
- the active pane filters the tree, grand total, KPI cards and crosstab;
  P&L ranks first and is the default
- grand-total row, KPI subtitles and footnote name the active pane
- Ac Type is dropped from the default row hierarchy when partitioned
- pane choice persists across reloads; sample gains Avg Bal/RWA/Metrics
  rows and P&L totals are unchanged by their presence

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018B5qKH9JxzLywUkLopxf6J
</commit_message>
<xml_diff>
--- a/tm1-dashboard/sample/GPS_Driller_sample.xlsx
+++ b/tm1-dashboard/sample/GPS_Driller_sample.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BU19"/>
+  <dimension ref="A1:BU27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5237,6 +5237,1968 @@
       </c>
       <c r="BU19" t="n">
         <v>575.53</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Avg Bal-IBCA-Current Accounts-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Avg Bal-GPS_NII_IBCA-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Avg Bal</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>IBCA-Current Accounts</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>GPS_NII_IBCA</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>MB20101000000 - Avg Bal</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>RTN16559</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>CG3000000</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>PR05010000 - Current Accounts - Other</t>
+        </is>
+      </c>
+      <c r="P20" t="n">
+        <v>46743.27</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>43277.63</v>
+      </c>
+      <c r="R20" t="n">
+        <v>78092.35000000001</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>76,715.30</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U20" t="n">
+        <v>46880</v>
+      </c>
+      <c r="V20" t="n">
+        <v>47823.57</v>
+      </c>
+      <c r="X20" t="n">
+        <v>34179.5</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>67596.64999999999</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>63388.91</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>78889.56</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>81192.00999999999</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>85764.44</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>24703.65</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>69764.28999999999</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>63187.25</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>37241.63</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>72772.03</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>39539.66</v>
+      </c>
+      <c r="AL20" t="n">
+        <v>38377.81</v>
+      </c>
+      <c r="AM20" t="n">
+        <v>78489.28999999999</v>
+      </c>
+      <c r="AN20" t="n">
+        <v>52015.1</v>
+      </c>
+      <c r="AO20" t="n">
+        <v>113463.21</v>
+      </c>
+      <c r="AP20" t="n">
+        <v>50121.56</v>
+      </c>
+      <c r="AQ20" t="n">
+        <v>91124.34</v>
+      </c>
+      <c r="AR20" t="n">
+        <v>55125.09</v>
+      </c>
+      <c r="AS20" t="n">
+        <v>78703.53999999999</v>
+      </c>
+      <c r="AT20" t="n">
+        <v>55431.68</v>
+      </c>
+      <c r="AU20" t="n">
+        <v>69342.71000000001</v>
+      </c>
+      <c r="AV20" t="n">
+        <v>69361.45</v>
+      </c>
+      <c r="AW20" t="n">
+        <v>-13658.85</v>
+      </c>
+      <c r="AX20" t="n">
+        <v>70828.77</v>
+      </c>
+      <c r="AY20" t="n">
+        <v>93258.12</v>
+      </c>
+      <c r="AZ20" t="n">
+        <v>60121.52</v>
+      </c>
+      <c r="BA20" t="n">
+        <v>54619.49</v>
+      </c>
+      <c r="BB20" t="n">
+        <v>45663.89</v>
+      </c>
+      <c r="BC20" t="n">
+        <v>54191.12</v>
+      </c>
+      <c r="BD20" t="n">
+        <v>115191.08</v>
+      </c>
+      <c r="BF20" t="n">
+        <v>44603.57</v>
+      </c>
+      <c r="BG20" t="n">
+        <v>82273.95</v>
+      </c>
+      <c r="BH20" t="n">
+        <v>19473.87</v>
+      </c>
+      <c r="BI20" t="n">
+        <v>77090.05</v>
+      </c>
+      <c r="BJ20" t="n">
+        <v>56099.77</v>
+      </c>
+      <c r="BK20" t="n">
+        <v>35874.27</v>
+      </c>
+      <c r="BL20" t="n">
+        <v>71630.22</v>
+      </c>
+      <c r="BM20" t="n">
+        <v>-21162.95</v>
+      </c>
+      <c r="BN20" t="n">
+        <v>75245.13</v>
+      </c>
+      <c r="BO20" t="n">
+        <v>36906.62</v>
+      </c>
+      <c r="BP20" t="n">
+        <v>-26582.67</v>
+      </c>
+      <c r="BQ20" t="n">
+        <v>51025.28</v>
+      </c>
+      <c r="BR20" t="n">
+        <v>57873.02</v>
+      </c>
+      <c r="BS20" t="n">
+        <v>-9564.51</v>
+      </c>
+      <c r="BU20" t="n">
+        <v>46503.73</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Avg Bal-IBCA-Savings-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Avg Bal-GPS_NII_IBCA-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Avg Bal</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>IBCA-Savings</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>GPS_NII_IBCA</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>MB20101000000 - Avg Bal</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>RTN16559</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>CG3000000</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>PR05040100 - Savings Accounts - Other</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>16186.72</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>17554.38</v>
+      </c>
+      <c r="R21" t="n">
+        <v>37899.05</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>78,935.79</t>
+        </is>
+      </c>
+      <c r="T21" t="n">
+        <v>51685.46</v>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>62,696.73</t>
+        </is>
+      </c>
+      <c r="W21" t="n">
+        <v>49652.81</v>
+      </c>
+      <c r="X21" t="n">
+        <v>13828.68</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>22408.82</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>15278.15</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>25754.14</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>37646.75</v>
+      </c>
+      <c r="AE21" t="n">
+        <v>22980.85</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>40102.19</v>
+      </c>
+      <c r="AG21" t="n">
+        <v>66761.31</v>
+      </c>
+      <c r="AH21" t="n">
+        <v>62129.87</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>25810.29</v>
+      </c>
+      <c r="AJ21" t="n">
+        <v>48164.6</v>
+      </c>
+      <c r="AK21" t="n">
+        <v>29603.57</v>
+      </c>
+      <c r="AL21" t="n">
+        <v>13677.13</v>
+      </c>
+      <c r="AM21" t="n">
+        <v>46130.75</v>
+      </c>
+      <c r="AN21" t="n">
+        <v>46105.95</v>
+      </c>
+      <c r="AO21" t="n">
+        <v>35964.27</v>
+      </c>
+      <c r="AP21" t="n">
+        <v>58504.24</v>
+      </c>
+      <c r="AQ21" t="n">
+        <v>56806.6</v>
+      </c>
+      <c r="AR21" t="n">
+        <v>70656.27</v>
+      </c>
+      <c r="AS21" t="n">
+        <v>43513.83</v>
+      </c>
+      <c r="AT21" t="n">
+        <v>50691.27</v>
+      </c>
+      <c r="AU21" t="n">
+        <v>62710.15</v>
+      </c>
+      <c r="AV21" t="n">
+        <v>57874.84</v>
+      </c>
+      <c r="AW21" t="n">
+        <v>31257.18</v>
+      </c>
+      <c r="AY21" t="n">
+        <v>38996.28</v>
+      </c>
+      <c r="AZ21" t="n">
+        <v>49537.44</v>
+      </c>
+      <c r="BA21" t="n">
+        <v>37861.05</v>
+      </c>
+      <c r="BB21" t="n">
+        <v>54674.61</v>
+      </c>
+      <c r="BC21" t="n">
+        <v>64216.81</v>
+      </c>
+      <c r="BD21" t="n">
+        <v>-15159.14</v>
+      </c>
+      <c r="BF21" t="n">
+        <v>47882.22</v>
+      </c>
+      <c r="BG21" t="n">
+        <v>26303.94</v>
+      </c>
+      <c r="BH21" t="n">
+        <v>38717.58</v>
+      </c>
+      <c r="BI21" t="n">
+        <v>43625.95</v>
+      </c>
+      <c r="BJ21" t="n">
+        <v>32010.44</v>
+      </c>
+      <c r="BK21" t="n">
+        <v>52559.26</v>
+      </c>
+      <c r="BL21" t="n">
+        <v>24624.18</v>
+      </c>
+      <c r="BM21" t="n">
+        <v>70175.64999999999</v>
+      </c>
+      <c r="BN21" t="n">
+        <v>39825.22</v>
+      </c>
+      <c r="BO21" t="n">
+        <v>55334.89</v>
+      </c>
+      <c r="BP21" t="inlineStr">
+        <is>
+          <t>47,848.85</t>
+        </is>
+      </c>
+      <c r="BQ21" t="n">
+        <v>33974.75</v>
+      </c>
+      <c r="BR21" t="n">
+        <v>66954.10000000001</v>
+      </c>
+      <c r="BS21" t="n">
+        <v>36455.6</v>
+      </c>
+      <c r="BT21" t="n">
+        <v>32649.68</v>
+      </c>
+      <c r="BU21" t="n">
+        <v>25915.83</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Avg Bal-NIBCA-Current Accounts-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Avg Bal-GPS_NII_NIBCA-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Avg Bal</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>NIBCA-Current Accounts</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>GPS_NII_NIBCA</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>MB20101000000 - Avg Bal</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>RTN16559</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>CG3000000</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>PR05020000 - Money Market Call Deposits</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>46857.19</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>43345.62</v>
+      </c>
+      <c r="R22" t="n">
+        <v>37022</v>
+      </c>
+      <c r="S22" t="n">
+        <v>36284.33</v>
+      </c>
+      <c r="T22" t="n">
+        <v>14463.03</v>
+      </c>
+      <c r="W22" t="n">
+        <v>-11351.98</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>42549.68</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>28124.63</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>29207.9</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>34315.88</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>25245.06</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>28464.56</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>46782.53</v>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG22" t="n">
+        <v>37905.36</v>
+      </c>
+      <c r="AH22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI22" t="inlineStr">
+        <is>
+          <t>20,394.00</t>
+        </is>
+      </c>
+      <c r="AJ22" t="n">
+        <v>24750.83</v>
+      </c>
+      <c r="AK22" t="n">
+        <v>29890.18</v>
+      </c>
+      <c r="AL22" t="inlineStr">
+        <is>
+          <t>22,450.96</t>
+        </is>
+      </c>
+      <c r="AM22" t="n">
+        <v>19714.42</v>
+      </c>
+      <c r="AN22" t="n">
+        <v>19718.04</v>
+      </c>
+      <c r="AO22" t="n">
+        <v>39506.17</v>
+      </c>
+      <c r="AP22" t="n">
+        <v>32279.22</v>
+      </c>
+      <c r="AQ22" t="n">
+        <v>50660.27</v>
+      </c>
+      <c r="AR22" t="n">
+        <v>-7608.28</v>
+      </c>
+      <c r="AS22" t="n">
+        <v>27525.54</v>
+      </c>
+      <c r="AT22" t="n">
+        <v>25343.79</v>
+      </c>
+      <c r="AU22" t="n">
+        <v>23455.98</v>
+      </c>
+      <c r="AV22" t="n">
+        <v>14287.7</v>
+      </c>
+      <c r="AW22" t="n">
+        <v>39529.9</v>
+      </c>
+      <c r="AX22" t="n">
+        <v>25271.67</v>
+      </c>
+      <c r="AY22" t="n">
+        <v>13534.14</v>
+      </c>
+      <c r="AZ22" t="n">
+        <v>32352.57</v>
+      </c>
+      <c r="BA22" t="n">
+        <v>40358.99</v>
+      </c>
+      <c r="BB22" t="n">
+        <v>34586.52</v>
+      </c>
+      <c r="BC22" t="n">
+        <v>-9045.76</v>
+      </c>
+      <c r="BD22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BF22" t="n">
+        <v>44418.07</v>
+      </c>
+      <c r="BG22" t="n">
+        <v>28586.63</v>
+      </c>
+      <c r="BH22" t="n">
+        <v>23463.84</v>
+      </c>
+      <c r="BI22" t="n">
+        <v>-9791.040000000001</v>
+      </c>
+      <c r="BJ22" t="n">
+        <v>-9220.6</v>
+      </c>
+      <c r="BL22" t="n">
+        <v>36356.7</v>
+      </c>
+      <c r="BM22" t="n">
+        <v>18972.58</v>
+      </c>
+      <c r="BO22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BP22" t="n">
+        <v>38537.87</v>
+      </c>
+      <c r="BQ22" t="n">
+        <v>38224.22</v>
+      </c>
+      <c r="BR22" t="n">
+        <v>28068.54</v>
+      </c>
+      <c r="BS22" t="n">
+        <v>33193.16</v>
+      </c>
+      <c r="BT22" t="n">
+        <v>32524.28</v>
+      </c>
+      <c r="BU22" t="n">
+        <v>15593.63</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Avg Bal-IBCA-TD-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Avg Bal-GPS_NII_IBCA-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Avg Bal</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>IBCA-TD</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>GPS_NII_IBCA</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>MB20101000000 - Avg Bal</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>RTN16559</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>CG3000000</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>PR05040200 - Time Deposits Other</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>18893.07</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>-4115.62</v>
+      </c>
+      <c r="S23" t="n">
+        <v>27842.17</v>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>16,239.94</t>
+        </is>
+      </c>
+      <c r="U23" t="n">
+        <v>44991</v>
+      </c>
+      <c r="V23" t="n">
+        <v>26502.81</v>
+      </c>
+      <c r="W23" t="n">
+        <v>21861.56</v>
+      </c>
+      <c r="X23" t="n">
+        <v>17166.25</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>7472.15</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>25023.25</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>37148.93</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>-7792.99</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>14116.82</v>
+      </c>
+      <c r="AD23" t="n">
+        <v>31901.58</v>
+      </c>
+      <c r="AE23" t="n">
+        <v>17535.68</v>
+      </c>
+      <c r="AG23" t="n">
+        <v>14184.99</v>
+      </c>
+      <c r="AH23" t="n">
+        <v>26482.39</v>
+      </c>
+      <c r="AI23" t="n">
+        <v>-3612.49</v>
+      </c>
+      <c r="AJ23" t="n">
+        <v>28321.01</v>
+      </c>
+      <c r="AK23" t="n">
+        <v>18859.39</v>
+      </c>
+      <c r="AL23" t="n">
+        <v>23065.9</v>
+      </c>
+      <c r="AM23" t="n">
+        <v>13062.52</v>
+      </c>
+      <c r="AN23" t="n">
+        <v>37348.04</v>
+      </c>
+      <c r="AO23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP23" t="n">
+        <v>25829.23</v>
+      </c>
+      <c r="AQ23" t="n">
+        <v>34272.76</v>
+      </c>
+      <c r="AR23" t="n">
+        <v>-3801.9</v>
+      </c>
+      <c r="AS23" t="n">
+        <v>25072.78</v>
+      </c>
+      <c r="AT23" t="n">
+        <v>16968.01</v>
+      </c>
+      <c r="AU23" t="n">
+        <v>21353.08</v>
+      </c>
+      <c r="AV23" t="n">
+        <v>20800.23</v>
+      </c>
+      <c r="AW23" t="n">
+        <v>-9640.959999999999</v>
+      </c>
+      <c r="AX23" t="n">
+        <v>30672.53</v>
+      </c>
+      <c r="AY23" t="n">
+        <v>23661.37</v>
+      </c>
+      <c r="AZ23" t="n">
+        <v>10752.9</v>
+      </c>
+      <c r="BA23" t="n">
+        <v>26121.83</v>
+      </c>
+      <c r="BB23" t="n">
+        <v>27816.22</v>
+      </c>
+      <c r="BC23" t="n">
+        <v>-5273.32</v>
+      </c>
+      <c r="BD23" t="n">
+        <v>22037.46</v>
+      </c>
+      <c r="BE23" t="n">
+        <v>31630.23</v>
+      </c>
+      <c r="BF23" t="n">
+        <v>5595.06</v>
+      </c>
+      <c r="BH23" t="n">
+        <v>13205.73</v>
+      </c>
+      <c r="BI23" t="n">
+        <v>29632.86</v>
+      </c>
+      <c r="BJ23" t="inlineStr">
+        <is>
+          <t>27,549.39</t>
+        </is>
+      </c>
+      <c r="BK23" t="n">
+        <v>25343.25</v>
+      </c>
+      <c r="BL23" t="n">
+        <v>21367.91</v>
+      </c>
+      <c r="BM23" t="n">
+        <v>22383.36</v>
+      </c>
+      <c r="BO23" t="n">
+        <v>36997.85</v>
+      </c>
+      <c r="BP23" t="n">
+        <v>35778.76</v>
+      </c>
+      <c r="BQ23" t="n">
+        <v>23291.53</v>
+      </c>
+      <c r="BR23" t="n">
+        <v>16545.96</v>
+      </c>
+      <c r="BS23" t="n">
+        <v>15877.78</v>
+      </c>
+      <c r="BT23" t="n">
+        <v>28184.59</v>
+      </c>
+      <c r="BU23" t="n">
+        <v>-4830.97</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>RWA-IBCA-Current Accounts-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>RWA-GPS_NII_IBCA-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>RWA</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>IBCA-Current Accounts</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>GPS_NII_IBCA</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>MB20101000000 - RWA</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>RTN16559</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>CG3000000</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>PR05010000 - Current Accounts - Other</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>-1874.09</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>10,618.79</t>
+        </is>
+      </c>
+      <c r="R24" t="n">
+        <v>-2237.7</v>
+      </c>
+      <c r="S24" t="n">
+        <v>9957.110000000001</v>
+      </c>
+      <c r="T24" t="n">
+        <v>7775.01</v>
+      </c>
+      <c r="U24" t="n">
+        <v>5226.4</v>
+      </c>
+      <c r="V24" t="n">
+        <v>9505.51</v>
+      </c>
+      <c r="W24" t="n">
+        <v>4021.46</v>
+      </c>
+      <c r="X24" t="n">
+        <v>7018.65</v>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>11,862.86</t>
+        </is>
+      </c>
+      <c r="AA24" t="n">
+        <v>8509.51</v>
+      </c>
+      <c r="AB24" t="n">
+        <v>9196.709999999999</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>6679.09</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>10027.15</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>8907.370000000001</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>7715.51</v>
+      </c>
+      <c r="AG24" t="n">
+        <v>8674.200000000001</v>
+      </c>
+      <c r="AH24" t="n">
+        <v>6741.08</v>
+      </c>
+      <c r="AJ24" t="n">
+        <v>8446.959999999999</v>
+      </c>
+      <c r="AK24" t="n">
+        <v>4631.6</v>
+      </c>
+      <c r="AL24" t="n">
+        <v>14361.78</v>
+      </c>
+      <c r="AM24" t="n">
+        <v>9726.9</v>
+      </c>
+      <c r="AN24" t="n">
+        <v>8275.540000000001</v>
+      </c>
+      <c r="AO24" t="n">
+        <v>9342.76</v>
+      </c>
+      <c r="AP24" t="n">
+        <v>8818.879999999999</v>
+      </c>
+      <c r="AQ24" t="n">
+        <v>8045.99</v>
+      </c>
+      <c r="AR24" t="n">
+        <v>11264.2</v>
+      </c>
+      <c r="AS24" t="n">
+        <v>-3033.62</v>
+      </c>
+      <c r="AT24" t="n">
+        <v>8374.07</v>
+      </c>
+      <c r="AU24" t="n">
+        <v>6596.9</v>
+      </c>
+      <c r="AV24" t="n">
+        <v>9501.48</v>
+      </c>
+      <c r="AW24" t="n">
+        <v>12008.97</v>
+      </c>
+      <c r="AX24" t="n">
+        <v>7406.61</v>
+      </c>
+      <c r="AY24" t="n">
+        <v>6283.13</v>
+      </c>
+      <c r="AZ24" t="n">
+        <v>7003.64</v>
+      </c>
+      <c r="BA24" t="inlineStr">
+        <is>
+          <t>7,644.68</t>
+        </is>
+      </c>
+      <c r="BB24" t="n">
+        <v>-2009.92</v>
+      </c>
+      <c r="BC24" t="n">
+        <v>9235.809999999999</v>
+      </c>
+      <c r="BD24" t="n">
+        <v>5310.24</v>
+      </c>
+      <c r="BE24" t="n">
+        <v>7328.15</v>
+      </c>
+      <c r="BF24" t="n">
+        <v>-3185.84</v>
+      </c>
+      <c r="BG24" t="n">
+        <v>10179.9</v>
+      </c>
+      <c r="BH24" t="n">
+        <v>10963.81</v>
+      </c>
+      <c r="BI24" t="n">
+        <v>10118.07</v>
+      </c>
+      <c r="BJ24" t="n">
+        <v>7155.64</v>
+      </c>
+      <c r="BK24" t="n">
+        <v>7336.9</v>
+      </c>
+      <c r="BL24" t="n">
+        <v>11320.98</v>
+      </c>
+      <c r="BM24" t="n">
+        <v>9331.799999999999</v>
+      </c>
+      <c r="BN24" t="n">
+        <v>9035.08</v>
+      </c>
+      <c r="BO24" t="n">
+        <v>8270.299999999999</v>
+      </c>
+      <c r="BP24" t="n">
+        <v>9270.620000000001</v>
+      </c>
+      <c r="BQ24" t="n">
+        <v>11177.7</v>
+      </c>
+      <c r="BR24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BS24" t="n">
+        <v>6053.23</v>
+      </c>
+      <c r="BT24" t="n">
+        <v>10415.53</v>
+      </c>
+      <c r="BU24" t="n">
+        <v>13489.36</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>RWA-IBCA-TD-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>RWA-GPS_NII_IBCA-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>RWA</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>IBCA-TD</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>GPS_NII_IBCA</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>MB20101000000 - RWA</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>RTN16559</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>CG3000000</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>PR05040200 - Time Deposits Other</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>10271.66</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>5165.3</v>
+      </c>
+      <c r="R25" t="n">
+        <v>3150.14</v>
+      </c>
+      <c r="S25" t="n">
+        <v>4885.19</v>
+      </c>
+      <c r="T25" t="n">
+        <v>9467.74</v>
+      </c>
+      <c r="U25" t="n">
+        <v>6482.23</v>
+      </c>
+      <c r="V25" t="n">
+        <v>-1481.58</v>
+      </c>
+      <c r="W25" t="n">
+        <v>4639.08</v>
+      </c>
+      <c r="X25" t="n">
+        <v>-2158</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>3448.54</v>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA25" t="n">
+        <v>6714.04</v>
+      </c>
+      <c r="AB25" t="n">
+        <v>5287.17</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>3960.65</v>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>(1,417.15)</t>
+        </is>
+      </c>
+      <c r="AE25" t="n">
+        <v>2723.33</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>7383.59</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>-717.42</v>
+      </c>
+      <c r="AH25" t="n">
+        <v>4828.73</v>
+      </c>
+      <c r="AI25" t="inlineStr">
+        <is>
+          <t>5,477.75</t>
+        </is>
+      </c>
+      <c r="AJ25" t="n">
+        <v>3513.69</v>
+      </c>
+      <c r="AK25" t="n">
+        <v>6184.9</v>
+      </c>
+      <c r="AL25" t="n">
+        <v>-2093.56</v>
+      </c>
+      <c r="AM25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AN25" t="n">
+        <v>6129.28</v>
+      </c>
+      <c r="AO25" t="n">
+        <v>3114.39</v>
+      </c>
+      <c r="AP25" t="n">
+        <v>4263.06</v>
+      </c>
+      <c r="AR25" t="n">
+        <v>3231.12</v>
+      </c>
+      <c r="AS25" t="n">
+        <v>8559</v>
+      </c>
+      <c r="AT25" t="n">
+        <v>6475.07</v>
+      </c>
+      <c r="AU25" t="n">
+        <v>5226.1</v>
+      </c>
+      <c r="AW25" t="n">
+        <v>5526.44</v>
+      </c>
+      <c r="AX25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AZ25" t="n">
+        <v>6609.38</v>
+      </c>
+      <c r="BA25" t="n">
+        <v>7682.37</v>
+      </c>
+      <c r="BC25" t="n">
+        <v>5232.03</v>
+      </c>
+      <c r="BD25" t="n">
+        <v>4890.7</v>
+      </c>
+      <c r="BE25" t="n">
+        <v>-2102.18</v>
+      </c>
+      <c r="BF25" t="n">
+        <v>6029.74</v>
+      </c>
+      <c r="BG25" t="n">
+        <v>-1586.57</v>
+      </c>
+      <c r="BI25" t="n">
+        <v>4543.26</v>
+      </c>
+      <c r="BK25" t="n">
+        <v>8390.709999999999</v>
+      </c>
+      <c r="BL25" t="n">
+        <v>5793.01</v>
+      </c>
+      <c r="BM25" t="n">
+        <v>4882.62</v>
+      </c>
+      <c r="BN25" t="n">
+        <v>5326.4</v>
+      </c>
+      <c r="BO25" t="n">
+        <v>4837.16</v>
+      </c>
+      <c r="BP25" t="n">
+        <v>3535.13</v>
+      </c>
+      <c r="BQ25" t="n">
+        <v>6966.09</v>
+      </c>
+      <c r="BR25" t="n">
+        <v>-2244.51</v>
+      </c>
+      <c r="BS25" t="n">
+        <v>2957.5</v>
+      </c>
+      <c r="BT25" t="n">
+        <v>6462.75</v>
+      </c>
+      <c r="BU25" t="n">
+        <v>5900.11</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Metrics-IBCA-Current Accounts-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Metrics-GPS_NII_IBCA-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Metrics</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>IBCA-Current Accounts</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>GPS_NII_IBCA</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>MB20101000000 - Metrics</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>RTN16559</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>CG3000000</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>PR05010000 - Current Accounts - Other</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="R26" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="S26" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="T26" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="U26" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="V26" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="W26" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="X26" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="AB26" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="AC26" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="AH26" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="AJ26" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="AK26" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="AL26" t="inlineStr">
+        <is>
+          <t>1.24</t>
+        </is>
+      </c>
+      <c r="AM26" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="AN26" t="inlineStr">
+        <is>
+          <t>1.21</t>
+        </is>
+      </c>
+      <c r="AO26" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="AP26" t="inlineStr">
+        <is>
+          <t>1.29</t>
+        </is>
+      </c>
+      <c r="AQ26" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="AR26" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="AS26" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="AT26" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="AU26" t="n">
+        <v>2.84</v>
+      </c>
+      <c r="AV26" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="AW26" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="AX26" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="AY26" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="AZ26" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="BA26" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="BB26" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="BC26" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="BD26" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="BE26" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="BF26" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="BG26" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="BI26" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="BJ26" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="BL26" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="BM26" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="BN26" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="BO26" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="BP26" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="BQ26" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="BR26" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="BS26" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="BT26" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="BU26" t="n">
+        <v>1.95</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Metrics-IBCA-Savings-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Metrics-GPS_NII_IBCA-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Metrics</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>IBCA-Savings</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>GPS_NII_IBCA</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>MB20101000000 - Metrics</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>RTN16559</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>CG3000000</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>PR05040100 - Savings Accounts - Other</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="R27" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="S27" t="n">
+        <v>1</v>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>0.77</t>
+        </is>
+      </c>
+      <c r="U27" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="V27" t="n">
+        <v>-0.21</v>
+      </c>
+      <c r="W27" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="AA27" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="AB27" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AD27" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>-0.38</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AG27" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="AH27" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="AI27" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="AJ27" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="AK27" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="AL27" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AM27" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AN27" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="AO27" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="AQ27" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="AR27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AS27" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="AT27" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="AU27" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="AV27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW27" t="inlineStr">
+        <is>
+          <t>1.26</t>
+        </is>
+      </c>
+      <c r="AX27" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="AY27" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="AZ27" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="BA27" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="BB27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BD27" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="BE27" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="BF27" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="BG27" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="BH27" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="BI27" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="BJ27" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="BK27" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="BL27" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="BM27" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="BN27" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="BO27" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="BP27" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="BQ27" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="BR27" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="BS27" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="BU27" t="n">
+        <v>0.64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Split FTE headcount and contractor out of the Metrics pane
FTE rows were being summed together inside Metrics. Rows classified into
a Metrics-family pane are now re-paned by their marker text: contractor
wording -> 'FTE Contractor', else headcount/FTE wording -> 'FTE
Headcount'; genuine ratio rows stay in Metrics. FTE panes rank after
Metrics in the bar. Sample gains four FTE rows; verified each pane totals
only its own rows and P&L is unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018B5qKH9JxzLywUkLopxf6J
</commit_message>
<xml_diff>
--- a/tm1-dashboard/sample/GPS_Driller_sample.xlsx
+++ b/tm1-dashboard/sample/GPS_Driller_sample.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BU27"/>
+  <dimension ref="A1:BU31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7199,6 +7199,990 @@
       </c>
       <c r="BU27" t="n">
         <v>0.64</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Metrics-FTE-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Metrics-GPS-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Metrics</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>GPS</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>MB20101000000 - Metrics</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>RTN16559</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>CG3000000</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>FTE - Headcount - Permanent Staff</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>98.2</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>138.26</v>
+      </c>
+      <c r="R28" t="n">
+        <v>128.54</v>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>188.94</t>
+        </is>
+      </c>
+      <c r="U28" t="n">
+        <v>60.94</v>
+      </c>
+      <c r="V28" t="n">
+        <v>95.54000000000001</v>
+      </c>
+      <c r="W28" t="n">
+        <v>106.96</v>
+      </c>
+      <c r="X28" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>167.66</v>
+      </c>
+      <c r="AA28" t="n">
+        <v>-25.17</v>
+      </c>
+      <c r="AB28" t="n">
+        <v>158.81</v>
+      </c>
+      <c r="AC28" t="n">
+        <v>126.05</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>185.09</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>93.20999999999999</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>124.26</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>-39.23</v>
+      </c>
+      <c r="AH28" t="n">
+        <v>132.11</v>
+      </c>
+      <c r="AI28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ28" t="n">
+        <v>79.98</v>
+      </c>
+      <c r="AK28" t="n">
+        <v>143.38</v>
+      </c>
+      <c r="AL28" t="n">
+        <v>82.56999999999999</v>
+      </c>
+      <c r="AM28" t="n">
+        <v>132.15</v>
+      </c>
+      <c r="AN28" t="n">
+        <v>75.28</v>
+      </c>
+      <c r="AO28" t="n">
+        <v>148.05</v>
+      </c>
+      <c r="AP28" t="n">
+        <v>111.51</v>
+      </c>
+      <c r="AQ28" t="n">
+        <v>98.34999999999999</v>
+      </c>
+      <c r="AS28" t="n">
+        <v>160.35</v>
+      </c>
+      <c r="AU28" t="n">
+        <v>145.06</v>
+      </c>
+      <c r="AW28" t="n">
+        <v>128.42</v>
+      </c>
+      <c r="AX28" t="n">
+        <v>73.51000000000001</v>
+      </c>
+      <c r="AY28" t="n">
+        <v>117.25</v>
+      </c>
+      <c r="AZ28" t="n">
+        <v>130.92</v>
+      </c>
+      <c r="BA28" t="n">
+        <v>126.66</v>
+      </c>
+      <c r="BB28" t="n">
+        <v>131.94</v>
+      </c>
+      <c r="BC28" t="n">
+        <v>140.17</v>
+      </c>
+      <c r="BD28" t="n">
+        <v>-27.83</v>
+      </c>
+      <c r="BE28" t="n">
+        <v>99.84</v>
+      </c>
+      <c r="BF28" t="n">
+        <v>106.89</v>
+      </c>
+      <c r="BG28" t="n">
+        <v>144.91</v>
+      </c>
+      <c r="BH28" t="n">
+        <v>90.66</v>
+      </c>
+      <c r="BI28" t="n">
+        <v>123.95</v>
+      </c>
+      <c r="BJ28" t="n">
+        <v>89.29000000000001</v>
+      </c>
+      <c r="BK28" t="n">
+        <v>120.72</v>
+      </c>
+      <c r="BL28" t="n">
+        <v>99.16</v>
+      </c>
+      <c r="BM28" t="n">
+        <v>72.18000000000001</v>
+      </c>
+      <c r="BN28" t="n">
+        <v>-49.51</v>
+      </c>
+      <c r="BO28" t="inlineStr">
+        <is>
+          <t>73.39</t>
+        </is>
+      </c>
+      <c r="BP28" t="n">
+        <v>23.34</v>
+      </c>
+      <c r="BQ28" t="n">
+        <v>192.27</v>
+      </c>
+      <c r="BR28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BS28" t="n">
+        <v>79.09999999999999</v>
+      </c>
+      <c r="BT28" t="n">
+        <v>114.49</v>
+      </c>
+      <c r="BU28" t="n">
+        <v>64.28</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Metrics-FTE-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Metrics-GPS-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Metrics</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>GPS</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>MB20101000000 - Metrics</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>RTN16559</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>CG3000000</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>FTE - Headcount - Fixed Term</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>28.58</v>
+      </c>
+      <c r="R29" t="n">
+        <v>34.56</v>
+      </c>
+      <c r="S29" t="n">
+        <v>30.68</v>
+      </c>
+      <c r="T29" t="n">
+        <v>45.08</v>
+      </c>
+      <c r="U29" t="n">
+        <v>44.16</v>
+      </c>
+      <c r="V29" t="n">
+        <v>27.31</v>
+      </c>
+      <c r="W29" t="n">
+        <v>22.44</v>
+      </c>
+      <c r="X29" t="n">
+        <v>44.78</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>19.73</v>
+      </c>
+      <c r="AB29" t="n">
+        <v>28.96</v>
+      </c>
+      <c r="AC29" t="n">
+        <v>41.27</v>
+      </c>
+      <c r="AD29" t="n">
+        <v>30.86</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>22.68</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>29.96</v>
+      </c>
+      <c r="AG29" t="n">
+        <v>41.41</v>
+      </c>
+      <c r="AH29" t="n">
+        <v>22.97</v>
+      </c>
+      <c r="AI29" t="n">
+        <v>8.35</v>
+      </c>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>33.56</t>
+        </is>
+      </c>
+      <c r="AK29" t="n">
+        <v>11.93</v>
+      </c>
+      <c r="AL29" t="n">
+        <v>39.09</v>
+      </c>
+      <c r="AM29" t="n">
+        <v>26.07</v>
+      </c>
+      <c r="AN29" t="n">
+        <v>34.17</v>
+      </c>
+      <c r="AO29" t="inlineStr">
+        <is>
+          <t>28.95</t>
+        </is>
+      </c>
+      <c r="AP29" t="n">
+        <v>35.87</v>
+      </c>
+      <c r="AQ29" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="AR29" t="n">
+        <v>34.39</v>
+      </c>
+      <c r="AS29" t="n">
+        <v>-10.59</v>
+      </c>
+      <c r="AT29" t="n">
+        <v>10.54</v>
+      </c>
+      <c r="AW29" t="n">
+        <v>-7.74</v>
+      </c>
+      <c r="AX29" t="n">
+        <v>24.23</v>
+      </c>
+      <c r="AY29" t="n">
+        <v>19.91</v>
+      </c>
+      <c r="BA29" t="inlineStr">
+        <is>
+          <t>23.27</t>
+        </is>
+      </c>
+      <c r="BB29" t="n">
+        <v>20.25</v>
+      </c>
+      <c r="BD29" t="n">
+        <v>33.14</v>
+      </c>
+      <c r="BE29" t="n">
+        <v>18.84</v>
+      </c>
+      <c r="BF29" t="n">
+        <v>33.49</v>
+      </c>
+      <c r="BG29" t="n">
+        <v>48.65</v>
+      </c>
+      <c r="BH29" t="n">
+        <v>24.93</v>
+      </c>
+      <c r="BI29" t="n">
+        <v>27.38</v>
+      </c>
+      <c r="BJ29" t="n">
+        <v>36.87</v>
+      </c>
+      <c r="BK29" t="inlineStr">
+        <is>
+          <t>38.43</t>
+        </is>
+      </c>
+      <c r="BL29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM29" t="n">
+        <v>-4.84</v>
+      </c>
+      <c r="BO29" t="n">
+        <v>18.18</v>
+      </c>
+      <c r="BP29" t="n">
+        <v>13.52</v>
+      </c>
+      <c r="BQ29" t="n">
+        <v>39.58</v>
+      </c>
+      <c r="BR29" t="n">
+        <v>-13</v>
+      </c>
+      <c r="BS29" t="n">
+        <v>24.53</v>
+      </c>
+      <c r="BT29" t="n">
+        <v>29.42</v>
+      </c>
+      <c r="BU29" t="n">
+        <v>30.82</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Metrics-FTE-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Metrics-GPS-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Metrics</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>GPS</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>MB20101000000 - Metrics</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>RTN16559</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>CG3000000</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>FTE - Contractor - Onshore</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>19.03</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>23.48</v>
+      </c>
+      <c r="R30" t="n">
+        <v>34.73</v>
+      </c>
+      <c r="T30" t="n">
+        <v>23.05</v>
+      </c>
+      <c r="U30" t="n">
+        <v>-9</v>
+      </c>
+      <c r="V30" t="n">
+        <v>11.13</v>
+      </c>
+      <c r="W30" t="n">
+        <v>38.85</v>
+      </c>
+      <c r="X30" t="n">
+        <v>37.38</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>26.41</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>17.35</v>
+      </c>
+      <c r="AA30" t="n">
+        <v>6.69</v>
+      </c>
+      <c r="AB30" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>-2.23</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>19.82</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>26.38</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>36.18</v>
+      </c>
+      <c r="AH30" t="n">
+        <v>45.31</v>
+      </c>
+      <c r="AI30" t="n">
+        <v>28.68</v>
+      </c>
+      <c r="AJ30" t="n">
+        <v>18.95</v>
+      </c>
+      <c r="AK30" t="inlineStr">
+        <is>
+          <t>20.83</t>
+        </is>
+      </c>
+      <c r="AL30" t="n">
+        <v>-6.69</v>
+      </c>
+      <c r="AM30" t="n">
+        <v>35.53</v>
+      </c>
+      <c r="AN30" t="n">
+        <v>27.26</v>
+      </c>
+      <c r="AO30" t="n">
+        <v>39.15</v>
+      </c>
+      <c r="AP30" t="n">
+        <v>26.11</v>
+      </c>
+      <c r="AQ30" t="n">
+        <v>20.39</v>
+      </c>
+      <c r="AS30" t="n">
+        <v>37.84</v>
+      </c>
+      <c r="AT30" t="n">
+        <v>27.09</v>
+      </c>
+      <c r="AU30" t="n">
+        <v>-5.06</v>
+      </c>
+      <c r="AV30" t="n">
+        <v>34.02</v>
+      </c>
+      <c r="AW30" t="n">
+        <v>26.88</v>
+      </c>
+      <c r="AX30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AY30" t="n">
+        <v>24.74</v>
+      </c>
+      <c r="AZ30" t="n">
+        <v>22.07</v>
+      </c>
+      <c r="BA30" t="n">
+        <v>21.39</v>
+      </c>
+      <c r="BB30" t="n">
+        <v>29.06</v>
+      </c>
+      <c r="BC30" t="n">
+        <v>32.55</v>
+      </c>
+      <c r="BD30" t="n">
+        <v>31.53</v>
+      </c>
+      <c r="BE30" t="n">
+        <v>20.85</v>
+      </c>
+      <c r="BG30" t="n">
+        <v>30.51</v>
+      </c>
+      <c r="BH30" t="n">
+        <v>21.71</v>
+      </c>
+      <c r="BI30" t="n">
+        <v>12.24</v>
+      </c>
+      <c r="BJ30" t="n">
+        <v>28</v>
+      </c>
+      <c r="BK30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BL30" t="n">
+        <v>23.83</v>
+      </c>
+      <c r="BM30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN30" t="n">
+        <v>21.66</v>
+      </c>
+      <c r="BO30" t="n">
+        <v>15.31</v>
+      </c>
+      <c r="BP30" t="n">
+        <v>30.45</v>
+      </c>
+      <c r="BQ30" t="n">
+        <v>-9.289999999999999</v>
+      </c>
+      <c r="BR30" t="n">
+        <v>36.91</v>
+      </c>
+      <c r="BS30" t="n">
+        <v>20.92</v>
+      </c>
+      <c r="BT30" t="n">
+        <v>30.19</v>
+      </c>
+      <c r="BU30" t="n">
+        <v>17.04</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Metrics-FTE-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Metrics-GPS-1000ALT2_1MGT-GB GPS</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Metrics</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>GB GPS</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>GPS</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>NII</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>1000ALT2_1MGT</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>MB20101000000 - Metrics</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>RTN16559</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>CG3000000</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>FTE - Contractor - Offshore</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
+        <v>-19.08</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>35.61</v>
+      </c>
+      <c r="R31" t="n">
+        <v>31.73</v>
+      </c>
+      <c r="S31" t="n">
+        <v>76.75</v>
+      </c>
+      <c r="U31" t="n">
+        <v>47.62</v>
+      </c>
+      <c r="W31" t="n">
+        <v>47.76</v>
+      </c>
+      <c r="X31" t="n">
+        <v>46.19</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>50.12</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>62.92</v>
+      </c>
+      <c r="AA31" t="n">
+        <v>40.62</v>
+      </c>
+      <c r="AB31" t="n">
+        <v>58.15</v>
+      </c>
+      <c r="AC31" t="n">
+        <v>37.79</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>46.21</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="AF31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AH31" t="n">
+        <v>31.41</v>
+      </c>
+      <c r="AJ31" t="n">
+        <v>35.03</v>
+      </c>
+      <c r="AK31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL31" t="n">
+        <v>44.19</v>
+      </c>
+      <c r="AM31" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="AN31" t="n">
+        <v>30.77</v>
+      </c>
+      <c r="AO31" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="AP31" t="n">
+        <v>-1.19</v>
+      </c>
+      <c r="AQ31" t="n">
+        <v>55.06</v>
+      </c>
+      <c r="AR31" t="n">
+        <v>51.91</v>
+      </c>
+      <c r="AS31" t="n">
+        <v>54.32</v>
+      </c>
+      <c r="AU31" t="n">
+        <v>40.23</v>
+      </c>
+      <c r="AV31" t="n">
+        <v>33.98</v>
+      </c>
+      <c r="AW31" t="n">
+        <v>45.86</v>
+      </c>
+      <c r="AY31" t="n">
+        <v>46.81</v>
+      </c>
+      <c r="AZ31" t="n">
+        <v>-11.05</v>
+      </c>
+      <c r="BA31" t="n">
+        <v>40.74</v>
+      </c>
+      <c r="BB31" t="n">
+        <v>51.36</v>
+      </c>
+      <c r="BC31" t="n">
+        <v>30.92</v>
+      </c>
+      <c r="BD31" t="n">
+        <v>61.16</v>
+      </c>
+      <c r="BE31" t="n">
+        <v>49.43</v>
+      </c>
+      <c r="BF31" t="n">
+        <v>52.26</v>
+      </c>
+      <c r="BG31" t="n">
+        <v>-15.44</v>
+      </c>
+      <c r="BH31" t="n">
+        <v>45.51</v>
+      </c>
+      <c r="BI31" t="n">
+        <v>46.29</v>
+      </c>
+      <c r="BJ31" t="n">
+        <v>55.49</v>
+      </c>
+      <c r="BK31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BL31" t="n">
+        <v>33.45</v>
+      </c>
+      <c r="BM31" t="n">
+        <v>35.29</v>
+      </c>
+      <c r="BN31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BO31" t="inlineStr">
+        <is>
+          <t>29.13</t>
+        </is>
+      </c>
+      <c r="BP31" t="n">
+        <v>28.74</v>
+      </c>
+      <c r="BQ31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BR31" t="n">
+        <v>51.54</v>
+      </c>
+      <c r="BS31" t="n">
+        <v>20.01</v>
+      </c>
+      <c r="BT31" t="n">
+        <v>22.73</v>
+      </c>
+      <c r="BU31" t="n">
+        <v>62.95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>